<commit_message>
Project BOM: $0 for made-at-work and unpriced lines (R210), To do sheet, first Digi-Key prices
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Needs Dan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$P$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$P$185</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Needs Dan'!$A$1:$D$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,7 +476,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,7 +507,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>of which printed-material est. USD</t>
+          <t>lines at $0 (made at work / not priced)</t>
         </is>
       </c>
     </row>
@@ -524,13 +524,13 @@
         <v>103</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>469.02</v>
+        <v>309.07</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>153.82</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -546,13 +546,13 @@
         <v>153</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>299.05</v>
+        <v>360.93</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -568,13 +568,13 @@
         <v>256</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>768.0700000000001</v>
+        <v>670</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>153.82</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -1093,16 +1093,16 @@
         <v>1</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>19.04</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>19.04</v>
+        <v>0</v>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1153,16 +1153,16 @@
         <v>1</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>10.74</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>10.74</v>
+        <v>0</v>
       </c>
       <c r="L9" s="3" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1972,14 +1972,22 @@
       <c r="I22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2512,14 +2520,22 @@
       <c r="I32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr"/>
@@ -2564,14 +2580,22 @@
       <c r="I33" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L33" s="3" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr"/>
-      <c r="N33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -2634,7 +2658,7 @@
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 1 per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -2685,10 +2709,10 @@
         <v>22</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>5.5</v>
+        <v>2.2</v>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
@@ -2698,7 +2722,7 @@
       <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 22+ per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
@@ -3797,16 +3821,16 @@
         <v>1</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>40.8</v>
+        <v>0</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>40.8</v>
+        <v>0</v>
       </c>
       <c r="L53" s="3" t="inlineStr"/>
       <c r="M53" s="3" t="inlineStr"/>
       <c r="N53" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -3857,16 +3881,16 @@
         <v>1</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>10.31</v>
+        <v>0</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>10.31</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
@@ -3917,16 +3941,16 @@
         <v>1</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>8.529999999999999</v>
+        <v>0</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>8.529999999999999</v>
+        <v>0</v>
       </c>
       <c r="L55" s="3" t="inlineStr"/>
       <c r="M55" s="3" t="inlineStr"/>
       <c r="N55" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O55" s="3" t="inlineStr">
@@ -4998,7 +5022,7 @@
       <c r="M72" s="2" t="inlineStr"/>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 1 per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
@@ -5049,10 +5073,10 @@
         <v>2</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="L73" s="5" t="inlineStr">
         <is>
@@ -5062,7 +5086,7 @@
       <c r="M73" s="3" t="inlineStr"/>
       <c r="N73" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 22+ per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O73" s="3" t="inlineStr">
@@ -6325,16 +6349,16 @@
         <v>1</v>
       </c>
       <c r="J93" s="3" t="n">
-        <v>36.16</v>
+        <v>0</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>36.16</v>
+        <v>0</v>
       </c>
       <c r="L93" s="3" t="inlineStr"/>
       <c r="M93" s="3" t="inlineStr"/>
       <c r="N93" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O93" s="3" t="inlineStr">
@@ -6385,16 +6409,16 @@
         <v>1</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr"/>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O94" s="2" t="inlineStr">
@@ -6445,16 +6469,16 @@
         <v>1</v>
       </c>
       <c r="J95" s="3" t="n">
-        <v>12.04</v>
+        <v>0</v>
       </c>
       <c r="K95" s="3" t="n">
-        <v>12.04</v>
+        <v>0</v>
       </c>
       <c r="L95" s="3" t="inlineStr"/>
       <c r="M95" s="3" t="inlineStr"/>
       <c r="N95" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O95" s="3" t="inlineStr">
@@ -6505,16 +6529,16 @@
         <v>1</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="inlineStr"/>
       <c r="M96" s="2" t="inlineStr"/>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr">
@@ -6564,12 +6588,8 @@
       <c r="I97" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J97" s="3" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="K97" s="3" t="n">
-        <v>2.53</v>
-      </c>
+      <c r="J97" s="3" t="inlineStr"/>
+      <c r="K97" s="3" t="inlineStr"/>
       <c r="L97" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-1-4-0-STK.html</t>
@@ -7576,14 +7596,22 @@
       <c r="I114" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J114" s="2" t="inlineStr"/>
-      <c r="K114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L114" s="2" t="inlineStr"/>
       <c r="M114" s="2" t="inlineStr"/>
-      <c r="N114" s="2" t="inlineStr"/>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P114" s="2" t="inlineStr"/>
@@ -7628,11 +7656,19 @@
       <c r="I115" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J115" s="3" t="inlineStr"/>
-      <c r="K115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L115" s="3" t="inlineStr"/>
       <c r="M115" s="3" t="inlineStr"/>
-      <c r="N115" s="3" t="inlineStr"/>
+      <c r="N115" s="3" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O115" s="3" t="inlineStr">
         <is>
           <t>printed on Dan's PA12 printer (R82: no buy link)</t>
@@ -8580,7 +8616,7 @@
       <c r="M15" s="3" t="inlineStr"/>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 1 per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -8631,10 +8667,10 @@
         <v>24</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>6</v>
+        <v>2.4</v>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
@@ -8644,7 +8680,7 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 22+ per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -12930,18 +12966,26 @@
       <c r="I95" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J95" s="3" t="inlineStr"/>
-      <c r="K95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K95" s="3" t="n">
+        <v>3.35</v>
+      </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT04-2P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT04-2P/6566582</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
-      <c r="N95" s="3" t="inlineStr"/>
+      <c r="N95" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O95" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P95" s="3" t="inlineStr"/>
@@ -12986,18 +13030,26 @@
       <c r="I96" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J96" s="2" t="inlineStr"/>
-      <c r="K96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="K96" s="2" t="n">
+        <v>0.96</v>
+      </c>
       <c r="L96" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT04-3P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT04-3P/6566583</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr"/>
-      <c r="N96" s="2" t="inlineStr"/>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr"/>
@@ -13042,18 +13094,26 @@
       <c r="I97" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J97" s="3" t="inlineStr"/>
-      <c r="K97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="K97" s="3" t="n">
+        <v>4.68</v>
+      </c>
       <c r="L97" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT04-6P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT04-6P/6566585</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
-      <c r="N97" s="3" t="inlineStr"/>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O97" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P97" s="3" t="inlineStr"/>
@@ -13098,15 +13158,23 @@
       <c r="I98" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J98" s="2" t="inlineStr"/>
-      <c r="K98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="K98" s="2" t="n">
+        <v>2.34</v>
+      </c>
       <c r="L98" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-DT04-6P-CE03.html</t>
         </is>
       </c>
       <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>family price (DT04-6P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -13154,18 +13222,26 @@
       <c r="I99" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J99" s="3" t="inlineStr"/>
-      <c r="K99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="K99" s="3" t="n">
+        <v>7.62</v>
+      </c>
       <c r="L99" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-08SA.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-08SA/6566565</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
-      <c r="N99" s="3" t="inlineStr"/>
+      <c r="N99" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O99" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P99" s="3" t="inlineStr"/>
@@ -13258,18 +13334,26 @@
       <c r="I101" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J101" s="3" t="inlineStr"/>
-      <c r="K101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K101" s="3" t="n">
+        <v>0.77</v>
+      </c>
       <c r="L101" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-2S/6566572</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr"/>
-      <c r="N101" s="3" t="inlineStr"/>
+      <c r="N101" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O101" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P101" s="3" t="inlineStr"/>
@@ -13314,15 +13398,23 @@
       <c r="I102" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J102" s="2" t="inlineStr"/>
-      <c r="K102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K102" s="2" t="n">
+        <v>6.16</v>
+      </c>
       <c r="L102" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-DT06-2S-CE05.html</t>
         </is>
       </c>
       <c r="M102" s="2" t="inlineStr"/>
-      <c r="N102" s="2" t="inlineStr"/>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>family price (DT06-2S, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -13418,18 +13510,26 @@
       <c r="I104" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J104" s="2" t="inlineStr"/>
-      <c r="K104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="K104" s="2" t="n">
+        <v>2.06</v>
+      </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-3S-CE05.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-3S-CE05/7219768</t>
         </is>
       </c>
       <c r="M104" s="2" t="inlineStr"/>
-      <c r="N104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P104" s="2" t="inlineStr"/>
@@ -13474,18 +13574,26 @@
       <c r="I105" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J105" s="3" t="inlineStr"/>
-      <c r="K105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="K105" s="3" t="n">
+        <v>5.04</v>
+      </c>
       <c r="L105" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-6S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-6S/6566575</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
-      <c r="N105" s="3" t="inlineStr"/>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O105" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P105" s="3" t="inlineStr"/>
@@ -13530,18 +13638,26 @@
       <c r="I106" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J106" s="2" t="inlineStr"/>
-      <c r="K106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="K106" s="2" t="n">
+        <v>2.68</v>
+      </c>
       <c r="L106" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-6S-CE05.html</t>
+          <t>https://www.digikey.com/en/products/detail/wee/DT06-6S-CE05/29360522</t>
         </is>
       </c>
       <c r="M106" s="2" t="inlineStr"/>
-      <c r="N106" s="2" t="inlineStr"/>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key listing opened 2026-10-19 (reseller "wee", not TE direct)</t>
         </is>
       </c>
       <c r="P106" s="2" t="inlineStr"/>
@@ -13586,18 +13702,26 @@
       <c r="I107" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J107" s="3" t="inlineStr"/>
-      <c r="K107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="K107" s="3" t="n">
+        <v>13.92</v>
+      </c>
       <c r="L107" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DTHD06-1-8S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DTHD06-1-8S/9554131</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
-      <c r="N107" s="3" t="inlineStr"/>
+      <c r="N107" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O107" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P107" s="3" t="inlineStr"/>
@@ -16170,14 +16294,26 @@
       <c r="I154" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J154" s="2" t="inlineStr"/>
-      <c r="K154" s="2" t="inlineStr"/>
-      <c r="L154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="K154" s="2" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="L154" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/amphenol-technical-products-international/RL9080-301-F1/16271602</t>
+        </is>
+      </c>
       <c r="M154" s="2" t="inlineStr"/>
-      <c r="N154" s="2" t="inlineStr"/>
+      <c r="N154" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O154" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P154" s="2" t="inlineStr"/>
@@ -16274,15 +16410,23 @@
       <c r="I156" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J156" s="2" t="inlineStr"/>
-      <c r="K156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L156" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-16-4-STK.html</t>
         </is>
       </c>
       <c r="M156" s="2" t="inlineStr"/>
-      <c r="N156" s="2" t="inlineStr"/>
+      <c r="N156" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16330,15 +16474,23 @@
       <c r="I157" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J157" s="3" t="inlineStr"/>
-      <c r="K157" s="3" t="inlineStr"/>
+      <c r="J157" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L157" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-16-6-STK.html</t>
         </is>
       </c>
       <c r="M157" s="3" t="inlineStr"/>
-      <c r="N157" s="3" t="inlineStr"/>
+      <c r="N157" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O157" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16386,15 +16538,23 @@
       <c r="I158" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J158" s="2" t="inlineStr"/>
-      <c r="K158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L158" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-16-9-STK.html</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr"/>
-      <c r="N158" s="2" t="inlineStr"/>
+      <c r="N158" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O158" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16442,15 +16602,23 @@
       <c r="I159" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J159" s="3" t="inlineStr"/>
-      <c r="K159" s="3" t="inlineStr"/>
+      <c r="J159" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L159" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-32-4-STK.html</t>
         </is>
       </c>
       <c r="M159" s="3" t="inlineStr"/>
-      <c r="N159" s="3" t="inlineStr"/>
+      <c r="N159" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O159" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16498,15 +16666,23 @@
       <c r="I160" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J160" s="2" t="inlineStr"/>
-      <c r="K160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L160" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-32-6-STK.html</t>
         </is>
       </c>
       <c r="M160" s="2" t="inlineStr"/>
-      <c r="N160" s="2" t="inlineStr"/>
+      <c r="N160" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16554,15 +16730,23 @@
       <c r="I161" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J161" s="3" t="inlineStr"/>
-      <c r="K161" s="3" t="inlineStr"/>
+      <c r="J161" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-32-9-STK.html</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
-      <c r="N161" s="3" t="inlineStr"/>
+      <c r="N161" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O161" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16610,15 +16794,23 @@
       <c r="I162" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J162" s="2" t="inlineStr"/>
-      <c r="K162" s="2" t="inlineStr"/>
+      <c r="J162" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K162" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L162" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-8-4-STK.html</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr"/>
-      <c r="N162" s="2" t="inlineStr"/>
+      <c r="N162" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16666,15 +16858,23 @@
       <c r="I163" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J163" s="3" t="inlineStr"/>
-      <c r="K163" s="3" t="inlineStr"/>
+      <c r="J163" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-8-6-STK.html</t>
         </is>
       </c>
       <c r="M163" s="3" t="inlineStr"/>
-      <c r="N163" s="3" t="inlineStr"/>
+      <c r="N163" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O163" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16774,15 +16974,23 @@
       <c r="I165" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="J165" s="3" t="inlineStr"/>
-      <c r="K165" s="3" t="inlineStr"/>
+      <c r="J165" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K165" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-TMS-SCE-1-2-2.0-9.html</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
-      <c r="N165" s="3" t="inlineStr"/>
+      <c r="N165" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O165" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16830,15 +17038,23 @@
       <c r="I166" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="J166" s="2" t="inlineStr"/>
-      <c r="K166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K166" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L166" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-TMS-SCE-3-16-2.0-9.html</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr"/>
-      <c r="N166" s="2" t="inlineStr"/>
+      <c r="N166" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O166" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16886,15 +17102,23 @@
       <c r="I167" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="J167" s="3" t="inlineStr"/>
-      <c r="K167" s="3" t="inlineStr"/>
+      <c r="J167" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K167" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L167" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-TMS-SCE-3-8-2.0-9.html</t>
         </is>
       </c>
       <c r="M167" s="3" t="inlineStr"/>
-      <c r="N167" s="3" t="inlineStr"/>
+      <c r="N167" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O167" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -17094,18 +17318,26 @@
       <c r="I171" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J171" s="3" t="inlineStr"/>
-      <c r="K171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K171" s="3" t="n">
+        <v>0.65</v>
+      </c>
       <c r="L171" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="M171" s="3" t="inlineStr"/>
-      <c r="N171" s="3" t="inlineStr"/>
+      <c r="N171" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O171" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P171" s="3" t="inlineStr"/>
@@ -17150,15 +17382,23 @@
       <c r="I172" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J172" s="2" t="inlineStr"/>
-      <c r="K172" s="2" t="inlineStr"/>
+      <c r="J172" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K172" s="2" t="n">
+        <v>1.43</v>
+      </c>
       <c r="L172" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr"/>
-      <c r="N172" s="2" t="inlineStr"/>
+      <c r="N172" s="2" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -17206,15 +17446,23 @@
       <c r="I173" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J173" s="3" t="inlineStr"/>
-      <c r="K173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K173" s="3" t="n">
+        <v>0.13</v>
+      </c>
       <c r="L173" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-W3P.html</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
-      <c r="N173" s="3" t="inlineStr"/>
+      <c r="N173" s="3" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O173" s="3" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -17262,15 +17510,23 @@
       <c r="I174" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J174" s="2" t="inlineStr"/>
-      <c r="K174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K174" s="2" t="n">
+        <v>0.26</v>
+      </c>
       <c r="L174" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr"/>
-      <c r="N174" s="2" t="inlineStr"/>
+      <c r="N174" s="2" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -17955,31 +18211,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L158" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L159" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L160" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L166" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L154" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L158" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L159" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L160" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L166" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -17992,7 +18249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18251,12 +18508,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-1/4-0-STK</t>
+          <t>280919-2</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -18273,12 +18530,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>50M060100P030</t>
+          <t>6-1419137-4</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -18295,17 +18552,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ISO 10642 M3 x 12 A2</t>
+          <t>RNF-100-1/4-0-STK</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18317,7 +18574,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>LP-16-C05SX-02-101</t>
+          <t>50M060100P030</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -18339,7 +18596,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>LP-16-C05SX-02-101</t>
+          <t>ISO 10642 M3 x 12 A2</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -18349,7 +18606,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18361,7 +18618,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Lemu 2990806014</t>
+          <t>LP-16-C05SX-02-101</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -18383,7 +18640,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>N0674-70 2-039</t>
+          <t>LP-16-C05SX-02-101</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -18400,12 +18657,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Wire harness</t>
+          <t>Mechanical assemblies</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>1.8k 1/4W</t>
+          <t>Lemu 2990806014</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -18415,19 +18672,19 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Wire harness</t>
+          <t>Mechanical assemblies</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>10k 1/4W</t>
+          <t>N0674-70 2-039</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -18437,7 +18694,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18449,12 +18706,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>0413-204-2005</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -18471,12 +18728,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>120R 1/4W</t>
+          <t>0413-214-1205</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -18493,12 +18750,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>12110293</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -18515,12 +18772,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>0462-201-2031</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -18537,7 +18794,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>1.8k 1/4W</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -18547,7 +18804,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18559,7 +18816,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>10k 1/4W</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -18569,7 +18826,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18581,12 +18838,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>1N5822</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -18603,17 +18860,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1k 1/4W</t>
+          <t>12084200</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>Waytek listing seen 2026-10-19 (100 pc min, 0 stock; Aptiv sheet not checked)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18625,7 +18882,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1/4W 1%</t>
+          <t>120R 1/4W</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -18635,7 +18892,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18904,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>3.9k 1/4W</t>
+          <t>12110293</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -18657,7 +18914,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18669,12 +18926,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>301A011-25-0</t>
+          <t>12191819</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -18691,12 +18948,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>301A022-25-0</t>
+          <t>15326426</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -18713,12 +18970,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>301A028-25-0</t>
+          <t>15419715</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -18735,12 +18992,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>342A012-25-0</t>
+          <t>1N5822</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -18757,17 +19014,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>342A024-25-0</t>
+          <t>1k 1/4W</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18779,17 +19036,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>342A034-25-0</t>
+          <t>2.2k 1/4W 1%</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18801,12 +19058,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>342A048-25-0</t>
+          <t>280919-2</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -18823,17 +19080,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>382A012-25-0</t>
+          <t>3.9k 1/4W</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18845,7 +19102,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>382A023-25-0</t>
+          <t>301A011-25-0</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -18867,7 +19124,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>382A034-25-0</t>
+          <t>301A022-25-0</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -18889,12 +19146,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>3R5</t>
+          <t>301A028-25-0</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -18911,12 +19168,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>462A023-25-0</t>
+          <t>320238</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -18933,17 +19190,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>470R 1/4W</t>
+          <t>320575</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18955,12 +19212,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>52-45780</t>
+          <t>342A012-25-0</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -18977,12 +19234,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>342A024-25-0</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -18999,12 +19256,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>880014175</t>
+          <t>342A034-25-0</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -19021,17 +19278,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>90980-10341</t>
+          <t>342A048-25-0</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19043,17 +19300,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>90980-11062</t>
+          <t>382A012-25-0</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19065,17 +19322,17 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>90980-11143</t>
+          <t>382A023-25-0</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19087,17 +19344,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>90980-11250</t>
+          <t>382A034-25-0</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19109,7 +19366,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>90980-11885</t>
+          <t>3R5</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -19119,7 +19376,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19131,17 +19388,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>ANL/MEGA 300A + holder</t>
+          <t>462A023-25-0</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19153,7 +19410,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>BC-1/0-BLK</t>
+          <t>470R 1/4W</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -19163,7 +19420,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19175,7 +19432,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>BC-1/0-RED</t>
+          <t>52-45780</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -19185,7 +19442,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19197,17 +19454,17 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>BC-2-RED</t>
+          <t>6-1419137-4</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19219,7 +19476,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>BC-4-BLK</t>
+          <t>8100-0461</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -19229,7 +19486,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19241,7 +19498,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>BDK 2.8</t>
+          <t>880014175</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -19263,17 +19520,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1-0-SP</t>
+          <t>90980-10341</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19285,17 +19542,17 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1-1/2-0-SP</t>
+          <t>90980-11062</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19307,17 +19564,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1/2-0-SP</t>
+          <t>90980-11143</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19329,17 +19586,17 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1/4-0-SP</t>
+          <t>90980-11250</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19351,17 +19608,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>DR-25-2-0-SP</t>
+          <t>90980-11885</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19373,17 +19630,17 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>DR-25-3/16-0-SP</t>
+          <t>ANL/MEGA 300A + holder</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19395,17 +19652,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DR-25-3/4-0-SP</t>
+          <t>BC-1/0-BLK</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19417,17 +19674,17 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>DR-25-3/8-0-SP</t>
+          <t>BC-1/0-RED</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19439,7 +19696,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>GENERIC CRIMP SPLICE 14-10</t>
+          <t>BC-2-RED</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -19449,7 +19706,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19461,7 +19718,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>GENERIC FLYING LEAD</t>
+          <t>BC-4-BLK</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -19471,7 +19728,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19483,7 +19740,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>GENERIC HEAVY FLYING LEAD 10-6</t>
+          <t>BDK 2.8</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -19493,7 +19750,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19505,17 +19762,17 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 2AWG</t>
+          <t>DR-25-1-0-SP</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19527,17 +19784,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 4AWG</t>
+          <t>DR-25-1-1/2-0-SP</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19549,17 +19806,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 50MM2</t>
+          <t>DR-25-1/2-0-SP</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19571,17 +19828,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 8AWG</t>
+          <t>DR-25-1/4-0-SP</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19593,17 +19850,17 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M8 2AWG</t>
+          <t>DR-25-2-0-SP</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19615,17 +19872,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>GENERIC LUG M8 4AWG</t>
+          <t>DR-25-3/16-0-SP</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19637,17 +19894,17 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M8 8AWG</t>
+          <t>DR-25-3/4-0-SP</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19659,17 +19916,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>GENERIC RING M6 12-10</t>
+          <t>DR-25-3/8-0-SP</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19681,17 +19938,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>GENERIC RING M6 22-16</t>
+          <t>DRB12-102PAE-L018</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19703,17 +19960,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>GENERIC RING M8 22-16</t>
+          <t>DRB16-102SAE-L018</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19725,17 +19982,17 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>GENERIC SOLDER SPLICE</t>
+          <t>DRBF-1A</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19747,17 +20004,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>GENERIC SPADE RECEPTACLE 12-10</t>
+          <t>DT04-08PA-P021</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19769,12 +20026,12 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>HD36-24-33SE</t>
+          <t>DT04-12PA-P021</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -19791,7 +20048,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Jump lugs 1/0</t>
+          <t>GENERIC CRIMP SPLICE 14-10</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -19813,7 +20070,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>LP-16-J05PE-02-001</t>
+          <t>GENERIC FLYING LEAD</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -19823,7 +20080,7 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19835,7 +20092,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-10-2</t>
+          <t>GENERIC HEAVY FLYING LEAD 10-6</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -19845,7 +20102,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19857,7 +20114,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-10-9</t>
+          <t>GENERIC LUG M10 2AWG</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -19867,7 +20124,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19879,7 +20136,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-12-0</t>
+          <t>GENERIC LUG M10 4AWG</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -19889,7 +20146,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19901,7 +20158,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-12-2</t>
+          <t>GENERIC LUG M10 50MM2</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -19911,7 +20168,7 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19923,7 +20180,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>GENERIC LUG M10 8AWG</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -19933,7 +20190,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19945,7 +20202,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-4</t>
+          <t>GENERIC LUG M8 2AWG</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -19955,7 +20212,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19967,7 +20224,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-0</t>
+          <t>GENERIC LUG M8 4AWG</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -19977,7 +20234,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19989,7 +20246,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>GENERIC LUG M8 8AWG</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -19999,7 +20256,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20011,7 +20268,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-4</t>
+          <t>GENERIC RING M6 12-10</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -20021,7 +20278,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20033,7 +20290,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>GENERIC RING M6 22-16</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -20043,7 +20300,7 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20055,7 +20312,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>GENERIC RING M8 22-16</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -20065,7 +20322,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20077,7 +20334,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>GENERIC SOLDER SPLICE</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -20087,7 +20344,7 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20099,7 +20356,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>GENERIC SPADE RECEPTACLE 12-10</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -20109,7 +20366,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20121,17 +20378,17 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>HD36-24-33SE</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -20143,7 +20400,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-6-2</t>
+          <t>Jump lugs 1/0</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -20153,7 +20410,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20165,7 +20422,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-8-0</t>
+          <t>LP-16-J05PE-02-001</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -20175,7 +20432,7 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -20187,7 +20444,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-8-2</t>
+          <t>M22759/16-10-2</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -20209,7 +20466,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>MR-S ZZW30 EHPS pump - A 90980-12068 / B 90980-10897 / C 90980-10942</t>
+          <t>M22759/16-10-9</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -20219,7 +20476,7 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20231,7 +20488,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>RL00801-50BK</t>
+          <t>M22759/16-12-0</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -20241,7 +20498,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20253,7 +20510,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>RL00801-50RE</t>
+          <t>M22759/16-12-2</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -20263,7 +20520,7 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20532,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>RL9080-301-F1</t>
+          <t>M22759/16-14-0</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -20285,7 +20542,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20297,7 +20554,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>RL9080-301-F1RE</t>
+          <t>M22759/16-14-4</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -20307,7 +20564,7 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20319,17 +20576,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-4-STK</t>
+          <t>M22759/16-16-0</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20341,17 +20598,17 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-6-STK</t>
+          <t>M22759/16-16-4</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20363,17 +20620,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-9-STK</t>
+          <t>M22759/16-18-4</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20385,17 +20642,17 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-4-STK</t>
+          <t>M22759/16-18-9</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20407,17 +20664,17 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-6-STK</t>
+          <t>M22759/16-20-0</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20429,17 +20686,17 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-9-STK</t>
+          <t>M22759/16-20-3</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20451,17 +20708,17 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/8-4-STK</t>
+          <t>M22759/16-20-4</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20473,17 +20730,17 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/8-6-STK</t>
+          <t>M22759/16-20-6</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20495,17 +20752,17 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Sumitomo TS 025 6-way</t>
+          <t>M22759/16-20-9</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>seller page seen 2026-10-19 (per foot)</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20517,17 +20774,17 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
+          <t>M22759/16-6-2</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20539,17 +20796,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>M22759/16-8-0</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20561,17 +20818,17 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>M22759/16-8-2</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20583,17 +20840,17 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>V23132-A2001-B200</t>
+          <t>MR-S ZZW30 EHPS pump - A 90980-12068 / B 90980-10897 / C 90980-10942</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20605,12 +20862,12 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>RL00801-50BK</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -20627,12 +20884,12 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>RL00801-50RE</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -20649,12 +20906,12 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>RL9080-301-F1RE</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -20671,12 +20928,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>Sumitomo TS 025 6-way</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -20693,7 +20950,7 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>WB-51PAR</t>
+          <t>V23132-A2001-B200</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
@@ -20715,7 +20972,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>WB-51SAL</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -20737,7 +20994,7 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>WM-6S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -20759,22 +21016,176 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
+          <t>W8S</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>WB-51PAL</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>WB-51PAR</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>WB-51SAL</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>WB-51SAR</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>WM-4S</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>WM-6S</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
           <t>jump-post-M8</t>
         </is>
       </c>
-      <c r="C126" s="2" t="inlineStr">
+      <c r="C133" s="3" t="inlineStr">
         <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="D126" s="2" t="inlineStr">
+      <c r="D133" s="3" t="inlineStr">
         <is>
           <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D126"/>
+  <autoFilter ref="A1:D133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Project BOM: $0 for made-at-work and unpriced lines (R210), To do sheet, first Digi-Key prices (#355)
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Needs Dan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$P$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$P$185</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Needs Dan'!$A$1:$D$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,7 +476,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,7 +507,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>of which printed-material est. USD</t>
+          <t>lines at $0 (made at work / not priced)</t>
         </is>
       </c>
     </row>
@@ -524,13 +524,13 @@
         <v>103</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>469.02</v>
+        <v>309.07</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>153.82</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -546,13 +546,13 @@
         <v>153</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>299.05</v>
+        <v>360.93</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -568,13 +568,13 @@
         <v>256</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>768.0700000000001</v>
+        <v>670</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>153.82</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -1093,16 +1093,16 @@
         <v>1</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>19.04</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>19.04</v>
+        <v>0</v>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1153,16 +1153,16 @@
         <v>1</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>10.74</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>10.74</v>
+        <v>0</v>
       </c>
       <c r="L9" s="3" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1972,14 +1972,22 @@
       <c r="I22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2512,14 +2520,22 @@
       <c r="I32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr"/>
@@ -2564,14 +2580,22 @@
       <c r="I33" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L33" s="3" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr"/>
-      <c r="N33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -2634,7 +2658,7 @@
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 1 per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -2685,10 +2709,10 @@
         <v>22</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>5.5</v>
+        <v>2.2</v>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
@@ -2698,7 +2722,7 @@
       <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 22+ per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
@@ -3797,16 +3821,16 @@
         <v>1</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>40.8</v>
+        <v>0</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>40.8</v>
+        <v>0</v>
       </c>
       <c r="L53" s="3" t="inlineStr"/>
       <c r="M53" s="3" t="inlineStr"/>
       <c r="N53" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -3857,16 +3881,16 @@
         <v>1</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>10.31</v>
+        <v>0</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>10.31</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
@@ -3917,16 +3941,16 @@
         <v>1</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>8.529999999999999</v>
+        <v>0</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>8.529999999999999</v>
+        <v>0</v>
       </c>
       <c r="L55" s="3" t="inlineStr"/>
       <c r="M55" s="3" t="inlineStr"/>
       <c r="N55" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O55" s="3" t="inlineStr">
@@ -4998,7 +5022,7 @@
       <c r="M72" s="2" t="inlineStr"/>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 1 per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
@@ -5049,10 +5073,10 @@
         <v>2</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="L73" s="5" t="inlineStr">
         <is>
@@ -5062,7 +5086,7 @@
       <c r="M73" s="3" t="inlineStr"/>
       <c r="N73" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 22+ per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O73" s="3" t="inlineStr">
@@ -6325,16 +6349,16 @@
         <v>1</v>
       </c>
       <c r="J93" s="3" t="n">
-        <v>36.16</v>
+        <v>0</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>36.16</v>
+        <v>0</v>
       </c>
       <c r="L93" s="3" t="inlineStr"/>
       <c r="M93" s="3" t="inlineStr"/>
       <c r="N93" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O93" s="3" t="inlineStr">
@@ -6385,16 +6409,16 @@
         <v>1</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr"/>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O94" s="2" t="inlineStr">
@@ -6445,16 +6469,16 @@
         <v>1</v>
       </c>
       <c r="J95" s="3" t="n">
-        <v>12.04</v>
+        <v>0</v>
       </c>
       <c r="K95" s="3" t="n">
-        <v>12.04</v>
+        <v>0</v>
       </c>
       <c r="L95" s="3" t="inlineStr"/>
       <c r="M95" s="3" t="inlineStr"/>
       <c r="N95" s="3" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O95" s="3" t="inlineStr">
@@ -6505,16 +6529,16 @@
         <v>1</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="inlineStr"/>
       <c r="M96" s="2" t="inlineStr"/>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>est (printed material)</t>
+          <t>made at work (Dan, R210)</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr">
@@ -6564,12 +6588,8 @@
       <c r="I97" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J97" s="3" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="K97" s="3" t="n">
-        <v>2.53</v>
-      </c>
+      <c r="J97" s="3" t="inlineStr"/>
+      <c r="K97" s="3" t="inlineStr"/>
       <c r="L97" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-1-4-0-STK.html</t>
@@ -7576,14 +7596,22 @@
       <c r="I114" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J114" s="2" t="inlineStr"/>
-      <c r="K114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L114" s="2" t="inlineStr"/>
       <c r="M114" s="2" t="inlineStr"/>
-      <c r="N114" s="2" t="inlineStr"/>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>machined to the drawing (stock supplier not chosen)</t>
+          <t>machined to the drawing (R210: made at work, no buy link)</t>
         </is>
       </c>
       <c r="P114" s="2" t="inlineStr"/>
@@ -7628,11 +7656,19 @@
       <c r="I115" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J115" s="3" t="inlineStr"/>
-      <c r="K115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L115" s="3" t="inlineStr"/>
       <c r="M115" s="3" t="inlineStr"/>
-      <c r="N115" s="3" t="inlineStr"/>
+      <c r="N115" s="3" t="inlineStr">
+        <is>
+          <t>made at work (Dan, R210)</t>
+        </is>
+      </c>
       <c r="O115" s="3" t="inlineStr">
         <is>
           <t>printed on Dan's PA12 printer (R82: no buy link)</t>
@@ -8580,7 +8616,7 @@
       <c r="M15" s="3" t="inlineStr"/>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 1 per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -8631,10 +8667,10 @@
         <v>24</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>6</v>
+        <v>2.4</v>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
@@ -8644,7 +8680,7 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>Mouser qty 22+ per TRUSTED-SOURCES 2026-10-18 (TE page distributor panel)</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -12930,18 +12966,26 @@
       <c r="I95" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J95" s="3" t="inlineStr"/>
-      <c r="K95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K95" s="3" t="n">
+        <v>3.35</v>
+      </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT04-2P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT04-2P/6566582</t>
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
-      <c r="N95" s="3" t="inlineStr"/>
+      <c r="N95" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O95" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P95" s="3" t="inlineStr"/>
@@ -12986,18 +13030,26 @@
       <c r="I96" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J96" s="2" t="inlineStr"/>
-      <c r="K96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="K96" s="2" t="n">
+        <v>0.96</v>
+      </c>
       <c r="L96" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT04-3P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT04-3P/6566583</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr"/>
-      <c r="N96" s="2" t="inlineStr"/>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr"/>
@@ -13042,18 +13094,26 @@
       <c r="I97" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J97" s="3" t="inlineStr"/>
-      <c r="K97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="K97" s="3" t="n">
+        <v>4.68</v>
+      </c>
       <c r="L97" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT04-6P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT04-6P/6566585</t>
         </is>
       </c>
       <c r="M97" s="3" t="inlineStr"/>
-      <c r="N97" s="3" t="inlineStr"/>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O97" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P97" s="3" t="inlineStr"/>
@@ -13098,15 +13158,23 @@
       <c r="I98" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J98" s="2" t="inlineStr"/>
-      <c r="K98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="K98" s="2" t="n">
+        <v>2.34</v>
+      </c>
       <c r="L98" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-DT04-6P-CE03.html</t>
         </is>
       </c>
       <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>family price (DT04-6P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -13154,18 +13222,26 @@
       <c r="I99" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J99" s="3" t="inlineStr"/>
-      <c r="K99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="K99" s="3" t="n">
+        <v>7.62</v>
+      </c>
       <c r="L99" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-08SA.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-08SA/6566565</t>
         </is>
       </c>
       <c r="M99" s="3" t="inlineStr"/>
-      <c r="N99" s="3" t="inlineStr"/>
+      <c r="N99" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O99" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P99" s="3" t="inlineStr"/>
@@ -13258,18 +13334,26 @@
       <c r="I101" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J101" s="3" t="inlineStr"/>
-      <c r="K101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K101" s="3" t="n">
+        <v>0.77</v>
+      </c>
       <c r="L101" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-2S/6566572</t>
         </is>
       </c>
       <c r="M101" s="3" t="inlineStr"/>
-      <c r="N101" s="3" t="inlineStr"/>
+      <c r="N101" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O101" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P101" s="3" t="inlineStr"/>
@@ -13314,15 +13398,23 @@
       <c r="I102" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J102" s="2" t="inlineStr"/>
-      <c r="K102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K102" s="2" t="n">
+        <v>6.16</v>
+      </c>
       <c r="L102" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-DT06-2S-CE05.html</t>
         </is>
       </c>
       <c r="M102" s="2" t="inlineStr"/>
-      <c r="N102" s="2" t="inlineStr"/>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>family price (DT06-2S, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -13418,18 +13510,26 @@
       <c r="I104" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J104" s="2" t="inlineStr"/>
-      <c r="K104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="K104" s="2" t="n">
+        <v>2.06</v>
+      </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-3S-CE05.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-3S-CE05/7219768</t>
         </is>
       </c>
       <c r="M104" s="2" t="inlineStr"/>
-      <c r="N104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P104" s="2" t="inlineStr"/>
@@ -13474,18 +13574,26 @@
       <c r="I105" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J105" s="3" t="inlineStr"/>
-      <c r="K105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="K105" s="3" t="n">
+        <v>5.04</v>
+      </c>
       <c r="L105" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-6S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DT06-6S/6566575</t>
         </is>
       </c>
       <c r="M105" s="3" t="inlineStr"/>
-      <c r="N105" s="3" t="inlineStr"/>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O105" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P105" s="3" t="inlineStr"/>
@@ -13530,18 +13638,26 @@
       <c r="I106" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J106" s="2" t="inlineStr"/>
-      <c r="K106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="K106" s="2" t="n">
+        <v>2.68</v>
+      </c>
       <c r="L106" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DT06-6S-CE05.html</t>
+          <t>https://www.digikey.com/en/products/detail/wee/DT06-6S-CE05/29360522</t>
         </is>
       </c>
       <c r="M106" s="2" t="inlineStr"/>
-      <c r="N106" s="2" t="inlineStr"/>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key listing opened 2026-10-19 (reseller "wee", not TE direct)</t>
         </is>
       </c>
       <c r="P106" s="2" t="inlineStr"/>
@@ -13586,18 +13702,26 @@
       <c r="I107" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J107" s="3" t="inlineStr"/>
-      <c r="K107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="K107" s="3" t="n">
+        <v>13.92</v>
+      </c>
       <c r="L107" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DTHD06-1-8S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/DTHD06-1-8S/9554131</t>
         </is>
       </c>
       <c r="M107" s="3" t="inlineStr"/>
-      <c r="N107" s="3" t="inlineStr"/>
+      <c r="N107" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O107" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P107" s="3" t="inlineStr"/>
@@ -16170,14 +16294,26 @@
       <c r="I154" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J154" s="2" t="inlineStr"/>
-      <c r="K154" s="2" t="inlineStr"/>
-      <c r="L154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="K154" s="2" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="L154" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/amphenol-technical-products-international/RL9080-301-F1/16271602</t>
+        </is>
+      </c>
       <c r="M154" s="2" t="inlineStr"/>
-      <c r="N154" s="2" t="inlineStr"/>
+      <c r="N154" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O154" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P154" s="2" t="inlineStr"/>
@@ -16274,15 +16410,23 @@
       <c r="I156" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J156" s="2" t="inlineStr"/>
-      <c r="K156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L156" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-16-4-STK.html</t>
         </is>
       </c>
       <c r="M156" s="2" t="inlineStr"/>
-      <c r="N156" s="2" t="inlineStr"/>
+      <c r="N156" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16330,15 +16474,23 @@
       <c r="I157" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J157" s="3" t="inlineStr"/>
-      <c r="K157" s="3" t="inlineStr"/>
+      <c r="J157" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L157" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-16-6-STK.html</t>
         </is>
       </c>
       <c r="M157" s="3" t="inlineStr"/>
-      <c r="N157" s="3" t="inlineStr"/>
+      <c r="N157" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O157" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16386,15 +16538,23 @@
       <c r="I158" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J158" s="2" t="inlineStr"/>
-      <c r="K158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L158" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-16-9-STK.html</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr"/>
-      <c r="N158" s="2" t="inlineStr"/>
+      <c r="N158" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O158" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16442,15 +16602,23 @@
       <c r="I159" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J159" s="3" t="inlineStr"/>
-      <c r="K159" s="3" t="inlineStr"/>
+      <c r="J159" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L159" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-32-4-STK.html</t>
         </is>
       </c>
       <c r="M159" s="3" t="inlineStr"/>
-      <c r="N159" s="3" t="inlineStr"/>
+      <c r="N159" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O159" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16498,15 +16666,23 @@
       <c r="I160" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J160" s="2" t="inlineStr"/>
-      <c r="K160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L160" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-32-6-STK.html</t>
         </is>
       </c>
       <c r="M160" s="2" t="inlineStr"/>
-      <c r="N160" s="2" t="inlineStr"/>
+      <c r="N160" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16554,15 +16730,23 @@
       <c r="I161" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J161" s="3" t="inlineStr"/>
-      <c r="K161" s="3" t="inlineStr"/>
+      <c r="J161" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-32-9-STK.html</t>
         </is>
       </c>
       <c r="M161" s="3" t="inlineStr"/>
-      <c r="N161" s="3" t="inlineStr"/>
+      <c r="N161" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O161" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16610,15 +16794,23 @@
       <c r="I162" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J162" s="2" t="inlineStr"/>
-      <c r="K162" s="2" t="inlineStr"/>
+      <c r="J162" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K162" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L162" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-8-4-STK.html</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr"/>
-      <c r="N162" s="2" t="inlineStr"/>
+      <c r="N162" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16666,15 +16858,23 @@
       <c r="I163" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J163" s="3" t="inlineStr"/>
-      <c r="K163" s="3" t="inlineStr"/>
+      <c r="J163" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-RNF-100-3-8-6-STK.html</t>
         </is>
       </c>
       <c r="M163" s="3" t="inlineStr"/>
-      <c r="N163" s="3" t="inlineStr"/>
+      <c r="N163" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O163" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16774,15 +16974,23 @@
       <c r="I165" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="J165" s="3" t="inlineStr"/>
-      <c r="K165" s="3" t="inlineStr"/>
+      <c r="J165" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K165" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-TMS-SCE-1-2-2.0-9.html</t>
         </is>
       </c>
       <c r="M165" s="3" t="inlineStr"/>
-      <c r="N165" s="3" t="inlineStr"/>
+      <c r="N165" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O165" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16830,15 +17038,23 @@
       <c r="I166" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="J166" s="2" t="inlineStr"/>
-      <c r="K166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K166" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L166" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-TMS-SCE-3-16-2.0-9.html</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr"/>
-      <c r="N166" s="2" t="inlineStr"/>
+      <c r="N166" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O166" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -16886,15 +17102,23 @@
       <c r="I167" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="J167" s="3" t="inlineStr"/>
-      <c r="K167" s="3" t="inlineStr"/>
+      <c r="J167" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K167" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="L167" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-TMS-SCE-3-8-2.0-9.html</t>
         </is>
       </c>
       <c r="M167" s="3" t="inlineStr"/>
-      <c r="N167" s="3" t="inlineStr"/>
+      <c r="N167" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="O167" s="3" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -17094,18 +17318,26 @@
       <c r="I171" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J171" s="3" t="inlineStr"/>
-      <c r="K171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K171" s="3" t="n">
+        <v>0.65</v>
+      </c>
       <c r="L171" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="M171" s="3" t="inlineStr"/>
-      <c r="N171" s="3" t="inlineStr"/>
+      <c r="N171" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="O171" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="P171" s="3" t="inlineStr"/>
@@ -17150,15 +17382,23 @@
       <c r="I172" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J172" s="2" t="inlineStr"/>
-      <c r="K172" s="2" t="inlineStr"/>
+      <c r="J172" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K172" s="2" t="n">
+        <v>1.43</v>
+      </c>
       <c r="L172" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr"/>
-      <c r="N172" s="2" t="inlineStr"/>
+      <c r="N172" s="2" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -17206,15 +17446,23 @@
       <c r="I173" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J173" s="3" t="inlineStr"/>
-      <c r="K173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K173" s="3" t="n">
+        <v>0.13</v>
+      </c>
       <c r="L173" s="5" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-W3P.html</t>
         </is>
       </c>
       <c r="M173" s="3" t="inlineStr"/>
-      <c r="N173" s="3" t="inlineStr"/>
+      <c r="N173" s="3" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O173" s="3" t="inlineStr">
         <is>
           <t>te.com page opened 2026-10-19</t>
@@ -17262,15 +17510,23 @@
       <c r="I174" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J174" s="2" t="inlineStr"/>
-      <c r="K174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K174" s="2" t="n">
+        <v>0.26</v>
+      </c>
       <c r="L174" s="4" t="inlineStr">
         <is>
           <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr"/>
-      <c r="N174" s="2" t="inlineStr"/>
+      <c r="N174" s="2" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
           <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
@@ -17955,31 +18211,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L158" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L159" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L160" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L166" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L154" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L158" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L159" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L160" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L166" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -17992,7 +18249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18251,12 +18508,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-1/4-0-STK</t>
+          <t>280919-2</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -18273,12 +18530,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>50M060100P030</t>
+          <t>6-1419137-4</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -18295,17 +18552,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ISO 10642 M3 x 12 A2</t>
+          <t>RNF-100-1/4-0-STK</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18317,7 +18574,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>LP-16-C05SX-02-101</t>
+          <t>50M060100P030</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -18339,7 +18596,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>LP-16-C05SX-02-101</t>
+          <t>ISO 10642 M3 x 12 A2</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -18349,7 +18606,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18361,7 +18618,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Lemu 2990806014</t>
+          <t>LP-16-C05SX-02-101</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -18383,7 +18640,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>N0674-70 2-039</t>
+          <t>LP-16-C05SX-02-101</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -18400,12 +18657,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Wire harness</t>
+          <t>Mechanical assemblies</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>1.8k 1/4W</t>
+          <t>Lemu 2990806014</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -18415,19 +18672,19 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Wire harness</t>
+          <t>Mechanical assemblies</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>10k 1/4W</t>
+          <t>N0674-70 2-039</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -18437,7 +18694,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18449,12 +18706,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>0413-204-2005</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -18471,12 +18728,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>120R 1/4W</t>
+          <t>0413-214-1205</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -18493,12 +18750,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>12110293</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -18515,12 +18772,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>0462-201-2031</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -18537,7 +18794,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>1.8k 1/4W</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -18547,7 +18804,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18559,7 +18816,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>10k 1/4W</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -18569,7 +18826,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18581,12 +18838,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>1N5822</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -18603,17 +18860,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1k 1/4W</t>
+          <t>12084200</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>Waytek listing seen 2026-10-19 (100 pc min, 0 stock; Aptiv sheet not checked)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18625,7 +18882,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1/4W 1%</t>
+          <t>120R 1/4W</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -18635,7 +18892,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18904,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>3.9k 1/4W</t>
+          <t>12110293</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -18657,7 +18914,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18669,12 +18926,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>301A011-25-0</t>
+          <t>12191819</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -18691,12 +18948,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>301A022-25-0</t>
+          <t>15326426</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -18713,12 +18970,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>301A028-25-0</t>
+          <t>15419715</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -18735,12 +18992,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>342A012-25-0</t>
+          <t>1N5822</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -18757,17 +19014,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>342A024-25-0</t>
+          <t>1k 1/4W</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18779,17 +19036,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>342A034-25-0</t>
+          <t>2.2k 1/4W 1%</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18801,12 +19058,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>342A048-25-0</t>
+          <t>280919-2</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -18823,17 +19080,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>382A012-25-0</t>
+          <t>3.9k 1/4W</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -18845,7 +19102,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>382A023-25-0</t>
+          <t>301A011-25-0</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -18867,7 +19124,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>382A034-25-0</t>
+          <t>301A022-25-0</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -18889,12 +19146,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>3R5</t>
+          <t>301A028-25-0</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -18911,12 +19168,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>462A023-25-0</t>
+          <t>320238</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -18933,17 +19190,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>470R 1/4W</t>
+          <t>320575</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -18955,12 +19212,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>52-45780</t>
+          <t>342A012-25-0</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -18977,12 +19234,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>342A024-25-0</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -18999,12 +19256,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>880014175</t>
+          <t>342A034-25-0</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -19021,17 +19278,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>90980-10341</t>
+          <t>342A048-25-0</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19043,17 +19300,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>90980-11062</t>
+          <t>382A012-25-0</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19065,17 +19322,17 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>90980-11143</t>
+          <t>382A023-25-0</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19087,17 +19344,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>90980-11250</t>
+          <t>382A034-25-0</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19109,7 +19366,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>90980-11885</t>
+          <t>3R5</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -19119,7 +19376,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19131,17 +19388,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>ANL/MEGA 300A + holder</t>
+          <t>462A023-25-0</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19153,7 +19410,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>BC-1/0-BLK</t>
+          <t>470R 1/4W</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -19163,7 +19420,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19175,7 +19432,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>BC-1/0-RED</t>
+          <t>52-45780</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -19185,7 +19442,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19197,17 +19454,17 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>BC-2-RED</t>
+          <t>6-1419137-4</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19219,7 +19476,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>BC-4-BLK</t>
+          <t>8100-0461</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -19229,7 +19486,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19241,7 +19498,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>BDK 2.8</t>
+          <t>880014175</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -19263,17 +19520,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1-0-SP</t>
+          <t>90980-10341</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19285,17 +19542,17 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1-1/2-0-SP</t>
+          <t>90980-11062</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19307,17 +19564,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1/2-0-SP</t>
+          <t>90980-11143</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19329,17 +19586,17 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1/4-0-SP</t>
+          <t>90980-11250</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19351,17 +19608,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>DR-25-2-0-SP</t>
+          <t>90980-11885</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -19373,17 +19630,17 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>DR-25-3/16-0-SP</t>
+          <t>ANL/MEGA 300A + holder</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19395,17 +19652,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DR-25-3/4-0-SP</t>
+          <t>BC-1/0-BLK</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19417,17 +19674,17 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>DR-25-3/8-0-SP</t>
+          <t>BC-1/0-RED</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19439,7 +19696,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>GENERIC CRIMP SPLICE 14-10</t>
+          <t>BC-2-RED</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -19449,7 +19706,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19461,7 +19718,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>GENERIC FLYING LEAD</t>
+          <t>BC-4-BLK</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -19471,7 +19728,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -19483,7 +19740,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>GENERIC HEAVY FLYING LEAD 10-6</t>
+          <t>BDK 2.8</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -19493,7 +19750,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19505,17 +19762,17 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 2AWG</t>
+          <t>DR-25-1-0-SP</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19527,17 +19784,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 4AWG</t>
+          <t>DR-25-1-1/2-0-SP</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19549,17 +19806,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 50MM2</t>
+          <t>DR-25-1/2-0-SP</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19571,17 +19828,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>GENERIC LUG M10 8AWG</t>
+          <t>DR-25-1/4-0-SP</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19593,17 +19850,17 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M8 2AWG</t>
+          <t>DR-25-2-0-SP</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19615,17 +19872,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>GENERIC LUG M8 4AWG</t>
+          <t>DR-25-3/16-0-SP</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19637,17 +19894,17 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>GENERIC LUG M8 8AWG</t>
+          <t>DR-25-3/4-0-SP</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19659,17 +19916,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>GENERIC RING M6 12-10</t>
+          <t>DR-25-3/8-0-SP</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19681,17 +19938,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>GENERIC RING M6 22-16</t>
+          <t>DRB12-102PAE-L018</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19703,17 +19960,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>GENERIC RING M8 22-16</t>
+          <t>DRB16-102SAE-L018</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19725,17 +19982,17 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>GENERIC SOLDER SPLICE</t>
+          <t>DRBF-1A</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19747,17 +20004,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>GENERIC SPADE RECEPTACLE 12-10</t>
+          <t>DT04-08PA-P021</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -19769,12 +20026,12 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>HD36-24-33SE</t>
+          <t>DT04-12PA-P021</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -19791,7 +20048,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Jump lugs 1/0</t>
+          <t>GENERIC CRIMP SPLICE 14-10</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -19813,7 +20070,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>LP-16-J05PE-02-001</t>
+          <t>GENERIC FLYING LEAD</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -19823,7 +20080,7 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19835,7 +20092,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-10-2</t>
+          <t>GENERIC HEAVY FLYING LEAD 10-6</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -19845,7 +20102,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19857,7 +20114,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-10-9</t>
+          <t>GENERIC LUG M10 2AWG</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -19867,7 +20124,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19879,7 +20136,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-12-0</t>
+          <t>GENERIC LUG M10 4AWG</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -19889,7 +20146,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19901,7 +20158,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-12-2</t>
+          <t>GENERIC LUG M10 50MM2</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -19911,7 +20168,7 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19923,7 +20180,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>GENERIC LUG M10 8AWG</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -19933,7 +20190,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19945,7 +20202,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-4</t>
+          <t>GENERIC LUG M8 2AWG</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -19955,7 +20212,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19967,7 +20224,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-0</t>
+          <t>GENERIC LUG M8 4AWG</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -19977,7 +20234,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -19989,7 +20246,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>GENERIC LUG M8 8AWG</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -19999,7 +20256,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20011,7 +20268,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-4</t>
+          <t>GENERIC RING M6 12-10</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -20021,7 +20278,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20033,7 +20290,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>GENERIC RING M6 22-16</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -20043,7 +20300,7 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20055,7 +20312,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>GENERIC RING M8 22-16</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -20065,7 +20322,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20077,7 +20334,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>GENERIC SOLDER SPLICE</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -20087,7 +20344,7 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20099,7 +20356,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>GENERIC SPADE RECEPTACLE 12-10</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -20109,7 +20366,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20121,17 +20378,17 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>HD36-24-33SE</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -20143,7 +20400,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-6-2</t>
+          <t>Jump lugs 1/0</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -20153,7 +20410,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20165,7 +20422,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-8-0</t>
+          <t>LP-16-J05PE-02-001</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -20175,7 +20432,7 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -20187,7 +20444,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-8-2</t>
+          <t>M22759/16-10-2</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -20209,7 +20466,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>MR-S ZZW30 EHPS pump - A 90980-12068 / B 90980-10897 / C 90980-10942</t>
+          <t>M22759/16-10-9</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -20219,7 +20476,7 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20231,7 +20488,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>RL00801-50BK</t>
+          <t>M22759/16-12-0</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -20241,7 +20498,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20253,7 +20510,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>RL00801-50RE</t>
+          <t>M22759/16-12-2</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -20263,7 +20520,7 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20532,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>RL9080-301-F1</t>
+          <t>M22759/16-14-0</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -20285,7 +20542,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20297,7 +20554,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>RL9080-301-F1RE</t>
+          <t>M22759/16-14-4</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -20307,7 +20564,7 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20319,17 +20576,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-4-STK</t>
+          <t>M22759/16-16-0</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20341,17 +20598,17 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-6-STK</t>
+          <t>M22759/16-16-4</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20363,17 +20620,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-9-STK</t>
+          <t>M22759/16-18-4</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20385,17 +20642,17 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-4-STK</t>
+          <t>M22759/16-18-9</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20407,17 +20664,17 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-6-STK</t>
+          <t>M22759/16-20-0</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20429,17 +20686,17 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-9-STK</t>
+          <t>M22759/16-20-3</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20451,17 +20708,17 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/8-4-STK</t>
+          <t>M22759/16-20-4</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20473,17 +20730,17 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/8-6-STK</t>
+          <t>M22759/16-20-6</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20495,17 +20752,17 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Sumitomo TS 025 6-way</t>
+          <t>M22759/16-20-9</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>seller page seen 2026-10-19 (per foot)</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20517,17 +20774,17 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
+          <t>M22759/16-6-2</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20539,17 +20796,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>M22759/16-8-0</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20561,17 +20818,17 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>M22759/16-8-2</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -20583,17 +20840,17 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>V23132-A2001-B200</t>
+          <t>MR-S ZZW30 EHPS pump - A 90980-12068 / B 90980-10897 / C 90980-10942</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20605,12 +20862,12 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>RL00801-50BK</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -20627,12 +20884,12 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>RL00801-50RE</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -20649,12 +20906,12 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>RL9080-301-F1RE</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -20671,12 +20928,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>Sumitomo TS 025 6-way</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -20693,7 +20950,7 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>WB-51PAR</t>
+          <t>V23132-A2001-B200</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
@@ -20715,7 +20972,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>WB-51SAL</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -20737,7 +20994,7 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>WM-6S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -20759,22 +21016,176 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
+          <t>W8S</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>WB-51PAL</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>WB-51PAR</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>WB-51SAL</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>WB-51SAR</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>WM-4S</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>WM-6S</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
           <t>jump-post-M8</t>
         </is>
       </c>
-      <c r="C126" s="2" t="inlineStr">
+      <c r="C133" s="3" t="inlineStr">
         <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="D126" s="2" t="inlineStr">
+      <c r="D133" s="3" t="inlineStr">
         <is>
           <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D126"/>
+  <autoFilter ref="A1:D133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
BOM: price 42 more lines from KSV Looms / Custom Connector Kits / Race Spec (Shopify)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$205</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -546,10 +546,10 @@
         <v>193</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3252.25</v>
+        <v>4749.29</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -568,10 +568,10 @@
         <v>296</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>155</v>
+        <v>197</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3663.79</v>
+        <v>5160.83</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>23</v>
@@ -9242,14 +9242,26 @@
       <c r="J17" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/12052641?variant=45536631554366</t>
+        </is>
+      </c>
       <c r="N17" s="3" t="inlineStr"/>
-      <c r="O17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr"/>
@@ -9295,11 +9307,15 @@
       <c r="J18" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>2.24</v>
+      </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>https://waytekwire.com/product/aptiv-12084200-metri-pack-150-series-female</t>
+          <t>https://www.customconnectorkits.com/products/12084200-l?variant=45536283525438</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -9307,10 +9323,14 @@
           <t>https://www.ebay.de/itm/145990327082</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Waytek listing seen 2026-10-19 (100 pc min, 0 stock; Aptiv sheet not checked)</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -9425,14 +9445,26 @@
       <c r="J20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/12110293?variant=45536279953726</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
@@ -9478,14 +9510,26 @@
       <c r="J21" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/12191819-l?variant=45536512966974</t>
+        </is>
+      </c>
       <c r="N21" s="3" t="inlineStr"/>
-      <c r="O21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr"/>
@@ -9531,14 +9575,26 @@
       <c r="J22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/13519047?variant=45536514539838</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
@@ -9584,14 +9640,26 @@
       <c r="J23" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/15326426-l?variant=48621504332094</t>
+        </is>
+      </c>
       <c r="N23" s="3" t="inlineStr"/>
-      <c r="O23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr"/>
@@ -9637,14 +9705,26 @@
       <c r="J24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/15419715?variant=45536627917118</t>
+        </is>
+      </c>
       <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
@@ -11267,14 +11347,26 @@
       <c r="J50" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/8100-0461-l?variant=46049028800830</t>
+        </is>
+      </c>
       <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
@@ -11365,14 +11457,26 @@
       <c r="J52" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/toyota-lexus-90980-10897-8-pin-connector-kit?variant=29504109805610</t>
+        </is>
+      </c>
       <c r="N52" s="2" t="inlineStr"/>
-      <c r="O52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; equivalent connector kit, not the OEM part: confirm it fits</t>
+        </is>
+      </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -11463,14 +11567,26 @@
       <c r="J54" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr"/>
-      <c r="M54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/2-way-connector-kit-for-toyota-lexus-90980-11062-water-temperature-sensor-22-18-awg?variant=11482559741994</t>
+        </is>
+      </c>
       <c r="N54" s="2" t="inlineStr"/>
-      <c r="O54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; equivalent connector kit, not the OEM part: confirm it fits</t>
+        </is>
+      </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
@@ -11948,14 +12064,26 @@
       <c r="J63" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K63" s="3" t="inlineStr"/>
-      <c r="L63" s="3" t="inlineStr"/>
-      <c r="M63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="L63" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/6-way-connector-kit-same-as-bosch-d261-205-358-01-23-20-awg?variant=40430818852899</t>
+        </is>
+      </c>
       <c r="N63" s="3" t="inlineStr"/>
-      <c r="O63" s="3" t="inlineStr"/>
+      <c r="O63" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; equivalent connector kit, not the OEM part: confirm it fits</t>
+        </is>
+      </c>
       <c r="P63" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q63" s="3" t="inlineStr"/>
@@ -12001,14 +12129,26 @@
       <c r="J64" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K64" s="2" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr"/>
-      <c r="M64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="n">
+        <v>20.08</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>60.24</v>
+      </c>
+      <c r="M64" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/1-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443737243683</t>
+        </is>
+      </c>
       <c r="N64" s="2" t="inlineStr"/>
-      <c r="O64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $6.12 per ft</t>
+        </is>
+      </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -12115,14 +12255,26 @@
       <c r="J66" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr"/>
-      <c r="M66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/1-2-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443735736355</t>
+        </is>
+      </c>
       <c r="N66" s="2" t="inlineStr"/>
-      <c r="O66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $4.34 per ft</t>
+        </is>
+      </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
@@ -12172,14 +12324,26 @@
       <c r="J67" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="K67" s="3" t="inlineStr"/>
-      <c r="L67" s="3" t="inlineStr"/>
-      <c r="M67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="L67" s="3" t="n">
+        <v>78.54000000000001</v>
+      </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/1-4-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443735113763</t>
+        </is>
+      </c>
       <c r="N67" s="3" t="inlineStr"/>
-      <c r="O67" s="3" t="inlineStr"/>
+      <c r="O67" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $1.71 per ft</t>
+        </is>
+      </c>
       <c r="P67" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q67" s="3" t="inlineStr">
@@ -12286,14 +12450,26 @@
       <c r="J69" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="K69" s="3" t="inlineStr"/>
-      <c r="L69" s="3" t="inlineStr"/>
-      <c r="M69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="L69" s="3" t="n">
+        <v>72.02</v>
+      </c>
+      <c r="M69" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/3-16-raychem-dr-25-yellow-label-heat-shrink-tubing-per-foot?variant=40443733803043</t>
+        </is>
+      </c>
       <c r="N69" s="3" t="inlineStr"/>
-      <c r="O69" s="3" t="inlineStr"/>
+      <c r="O69" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $1.69 per ft</t>
+        </is>
+      </c>
       <c r="P69" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q69" s="3" t="inlineStr">
@@ -12343,14 +12519,26 @@
       <c r="J70" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/3-4-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443737112611</t>
+        </is>
+      </c>
       <c r="N70" s="2" t="inlineStr"/>
-      <c r="O70" s="2" t="inlineStr"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $4.57 per ft</t>
+        </is>
+      </c>
       <c r="P70" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q70" s="2" t="inlineStr">
@@ -12400,14 +12588,26 @@
       <c r="J71" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="K71" s="3" t="inlineStr"/>
-      <c r="L71" s="3" t="inlineStr"/>
-      <c r="M71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>129.96</v>
+      </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/3-8-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443735343139</t>
+        </is>
+      </c>
       <c r="N71" s="3" t="inlineStr"/>
-      <c r="O71" s="3" t="inlineStr"/>
+      <c r="O71" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $3.30 per ft</t>
+        </is>
+      </c>
       <c r="P71" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q71" s="3" t="inlineStr">
@@ -13529,18 +13729,26 @@
       <c r="J88" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>2.48</v>
+      </c>
       <c r="M88" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DTM06-6S.html</t>
+          <t>https://www.ksvlooms.com/products/dtm06-6s-deutsch-dtm-housing?variant=43643315290147</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr"/>
-      <c r="O88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P88" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q88" s="2" t="inlineStr"/>
@@ -13692,14 +13900,26 @@
       <c r="J91" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K91" s="3" t="inlineStr"/>
-      <c r="L91" s="3" t="inlineStr"/>
-      <c r="M91" s="3" t="inlineStr"/>
+      <c r="K91" s="3" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="L91" s="3" t="n">
+        <v>16.32</v>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/10-awg-black-tefzel-wire-m22759-16-10-0-cut-length?variant=40451551199267</t>
+        </is>
+      </c>
       <c r="N91" s="3" t="inlineStr"/>
-      <c r="O91" s="3" t="inlineStr"/>
+      <c r="O91" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P91" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q91" s="3" t="inlineStr">
@@ -13749,14 +13969,26 @@
       <c r="J92" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr"/>
-      <c r="M92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>21.76</v>
+      </c>
+      <c r="M92" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/10-awg-brown-tefzel-wire-m22759-16-10-1-spool?variant=40423436288035</t>
+        </is>
+      </c>
       <c r="N92" s="2" t="inlineStr"/>
-      <c r="O92" s="2" t="inlineStr"/>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P92" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q92" s="2" t="inlineStr">
@@ -13806,14 +14038,26 @@
       <c r="J93" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="K93" s="3" t="inlineStr"/>
-      <c r="L93" s="3" t="inlineStr"/>
-      <c r="M93" s="3" t="inlineStr"/>
+      <c r="K93" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L93" s="3" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/10-awg-red-tefzel-wire-m22759-16-10-2-cut-length?variant=40451119939619</t>
+        </is>
+      </c>
       <c r="N93" s="3" t="inlineStr"/>
-      <c r="O93" s="3" t="inlineStr"/>
+      <c r="O93" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P93" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q93" s="3" t="inlineStr">
@@ -13863,14 +14107,26 @@
       <c r="J94" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K94" s="2" t="inlineStr"/>
-      <c r="L94" s="2" t="inlineStr"/>
-      <c r="M94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="L94" s="2" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="M94" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/12-awg-black-tefzel-wire-m22759-16-12-0-spool?variant=40415052726307</t>
+        </is>
+      </c>
       <c r="N94" s="2" t="inlineStr"/>
-      <c r="O94" s="2" t="inlineStr"/>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P94" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q94" s="2" t="inlineStr">
@@ -13920,14 +14176,26 @@
       <c r="J95" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="K95" s="3" t="inlineStr"/>
-      <c r="L95" s="3" t="inlineStr"/>
-      <c r="M95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="L95" s="3" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M95" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/12-awg-red-tefzel-wire-m22759-16-12-2-spool?variant=40415053152291</t>
+        </is>
+      </c>
       <c r="N95" s="3" t="inlineStr"/>
-      <c r="O95" s="3" t="inlineStr"/>
+      <c r="O95" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P95" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q95" s="3" t="inlineStr">
@@ -13977,14 +14245,26 @@
       <c r="J96" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K96" s="2" t="inlineStr"/>
-      <c r="L96" s="2" t="inlineStr"/>
-      <c r="M96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/14-awg-black-tefzel-wire-m22759-16-14-0-spool?variant=40415048695843</t>
+        </is>
+      </c>
       <c r="N96" s="2" t="inlineStr"/>
-      <c r="O96" s="2" t="inlineStr"/>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P96" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q96" s="2" t="inlineStr">
@@ -14103,14 +14383,26 @@
       <c r="J98" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K98" s="2" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr"/>
-      <c r="M98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="L98" s="2" t="n">
+        <v>87.36</v>
+      </c>
+      <c r="M98" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/14-awg-blue-tefzel-wire-m22759-16-14-6-spool?variant=40423417708579</t>
+        </is>
+      </c>
       <c r="N98" s="2" t="inlineStr"/>
-      <c r="O98" s="2" t="inlineStr"/>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P98" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q98" s="2" t="inlineStr">
@@ -14388,14 +14680,26 @@
       <c r="J103" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="K103" s="3" t="inlineStr"/>
-      <c r="L103" s="3" t="inlineStr"/>
-      <c r="M103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="L103" s="3" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="M103" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/16-awg-black-tefzel-wire-m22759-16-16-0-spool?variant=40415046434851</t>
+        </is>
+      </c>
       <c r="N103" s="3" t="inlineStr"/>
-      <c r="O103" s="3" t="inlineStr"/>
+      <c r="O103" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P103" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q103" s="3" t="inlineStr">
@@ -14856,14 +15160,26 @@
       <c r="J111" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K111" s="3" t="inlineStr"/>
-      <c r="L111" s="3" t="inlineStr"/>
-      <c r="M111" s="3" t="inlineStr"/>
+      <c r="K111" s="3" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="L111" s="3" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/18-awg-black-tefzel-wire-m22759-16-18-0-spool?variant=40415044370467</t>
+        </is>
+      </c>
       <c r="N111" s="3" t="inlineStr"/>
-      <c r="O111" s="3" t="inlineStr"/>
+      <c r="O111" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P111" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q111" s="3" t="inlineStr">
@@ -15153,14 +15469,26 @@
       <c r="J116" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K116" s="2" t="inlineStr"/>
-      <c r="L116" s="2" t="inlineStr"/>
-      <c r="M116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>38.08</v>
+      </c>
+      <c r="M116" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/18-awg-purple-tefzel-wire-m22759-16-18-7-spool?variant=40423402700835</t>
+        </is>
+      </c>
       <c r="N116" s="2" t="inlineStr"/>
-      <c r="O116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P116" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q116" s="2" t="inlineStr">
@@ -15210,14 +15538,26 @@
       <c r="J117" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="K117" s="3" t="inlineStr"/>
-      <c r="L117" s="3" t="inlineStr"/>
-      <c r="M117" s="3" t="inlineStr"/>
+      <c r="K117" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L117" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="M117" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/18-awg-white-tefzel-wire-m22759-16-18-9-spool?variant=40415044829219</t>
+        </is>
+      </c>
       <c r="N117" s="3" t="inlineStr"/>
-      <c r="O117" s="3" t="inlineStr"/>
+      <c r="O117" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P117" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q117" s="3" t="inlineStr">
@@ -15267,14 +15607,26 @@
       <c r="J118" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="K118" s="2" t="inlineStr"/>
-      <c r="L118" s="2" t="inlineStr"/>
-      <c r="M118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="L118" s="2" t="n">
+        <v>27.72</v>
+      </c>
+      <c r="M118" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-black-tefzel-wire-m22759-16-20-0-spool?variant=40415026577443</t>
+        </is>
+      </c>
       <c r="N118" s="2" t="inlineStr"/>
-      <c r="O118" s="2" t="inlineStr"/>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P118" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q118" s="2" t="inlineStr">
@@ -15438,14 +15790,26 @@
       <c r="J121" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="K121" s="3" t="inlineStr"/>
-      <c r="L121" s="3" t="inlineStr"/>
-      <c r="M121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L121" s="3" t="n">
+        <v>23.52</v>
+      </c>
+      <c r="M121" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-brown-tefzel-wire-m22759-16-20-1-spool?variant=40415026708515</t>
+        </is>
+      </c>
       <c r="N121" s="3" t="inlineStr"/>
-      <c r="O121" s="3" t="inlineStr"/>
+      <c r="O121" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P121" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q121" s="3" t="inlineStr">
@@ -15564,14 +15928,26 @@
       <c r="J123" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="K123" s="3" t="inlineStr"/>
-      <c r="L123" s="3" t="inlineStr"/>
-      <c r="M123" s="3" t="inlineStr"/>
+      <c r="K123" s="3" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L123" s="3" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="M123" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-orange-tefzel-wire-m22759-16-20-3-spool?variant=40415028019235</t>
+        </is>
+      </c>
       <c r="N123" s="3" t="inlineStr"/>
-      <c r="O123" s="3" t="inlineStr"/>
+      <c r="O123" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P123" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q123" s="3" t="inlineStr">
@@ -15678,14 +16054,26 @@
       <c r="J125" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="K125" s="3" t="inlineStr"/>
-      <c r="L125" s="3" t="inlineStr"/>
-      <c r="M125" s="3" t="inlineStr"/>
+      <c r="K125" s="3" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="L125" s="3" t="n">
+        <v>36.96</v>
+      </c>
+      <c r="M125" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-yellow-tefzel-wire-m22759-16-20-4-spool?variant=40415028477987</t>
+        </is>
+      </c>
       <c r="N125" s="3" t="inlineStr"/>
-      <c r="O125" s="3" t="inlineStr"/>
+      <c r="O125" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P125" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q125" s="3" t="inlineStr">
@@ -15735,14 +16123,26 @@
       <c r="J126" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="K126" s="2" t="inlineStr"/>
-      <c r="L126" s="2" t="inlineStr"/>
-      <c r="M126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="M126" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-green-tefzel-wire-m22759-16-20-5-spool?variant=40415028838435</t>
+        </is>
+      </c>
       <c r="N126" s="2" t="inlineStr"/>
-      <c r="O126" s="2" t="inlineStr"/>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
@@ -15792,14 +16192,26 @@
       <c r="J127" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="K127" s="3" t="inlineStr"/>
-      <c r="L127" s="3" t="inlineStr"/>
-      <c r="M127" s="3" t="inlineStr"/>
+      <c r="K127" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L127" s="3" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="M127" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-blue-tefzel-wire-m22759-16-20-6-spool?variant=40415028903971</t>
+        </is>
+      </c>
       <c r="N127" s="3" t="inlineStr"/>
-      <c r="O127" s="3" t="inlineStr"/>
+      <c r="O127" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P127" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q127" s="3" t="inlineStr">
@@ -15849,14 +16261,26 @@
       <c r="J128" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="K128" s="2" t="inlineStr"/>
-      <c r="L128" s="2" t="inlineStr"/>
-      <c r="M128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>24.36</v>
+      </c>
+      <c r="M128" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-purple-tefzel-wire-m22759-16-20-7-spool?variant=40415029198883</t>
+        </is>
+      </c>
       <c r="N128" s="2" t="inlineStr"/>
-      <c r="O128" s="2" t="inlineStr"/>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P128" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q128" s="2" t="inlineStr">
@@ -15906,14 +16330,26 @@
       <c r="J129" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="K129" s="3" t="inlineStr"/>
-      <c r="L129" s="3" t="inlineStr"/>
-      <c r="M129" s="3" t="inlineStr"/>
+      <c r="K129" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L129" s="3" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="M129" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-gray-tefzel-wire-m22759-16-20-8-spool?variant=40415029264419</t>
+        </is>
+      </c>
       <c r="N129" s="3" t="inlineStr"/>
-      <c r="O129" s="3" t="inlineStr"/>
+      <c r="O129" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P129" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q129" s="3" t="inlineStr">
@@ -15963,11 +16399,15 @@
       <c r="J130" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="K130" s="2" t="inlineStr"/>
-      <c r="L130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L130" s="2" t="n">
+        <v>31.68</v>
+      </c>
       <c r="M130" s="4" t="inlineStr">
         <is>
-          <t>https://wingsandwheels.com/tefzel-wire-20-gauge-new.html</t>
+          <t>https://www.ksvlooms.com/products/20-awg-white-tefzel-wire-m22759-16-20-9-spool?variant=40415029297187</t>
         </is>
       </c>
       <c r="N130" s="4" t="inlineStr">
@@ -15975,10 +16415,14 @@
           <t>https://www.flightstore.com.au/M22759/16-Extruded-ETFE-Tefzel-Wire-20AWG-Per-FT</t>
         </is>
       </c>
-      <c r="O130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P130" s="2" t="inlineStr">
         <is>
-          <t>seller page seen 2026-10-19 (per foot)</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
@@ -16028,14 +16472,26 @@
       <c r="J131" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K131" s="3" t="inlineStr"/>
-      <c r="L131" s="3" t="inlineStr"/>
-      <c r="M131" s="3" t="inlineStr"/>
+      <c r="K131" s="3" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="L131" s="3" t="n">
+        <v>64.72</v>
+      </c>
+      <c r="M131" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/6-awg-white-tefzel-wire-m22759-16-6-9-spool?variant=40415058198563</t>
+        </is>
+      </c>
       <c r="N131" s="3" t="inlineStr"/>
-      <c r="O131" s="3" t="inlineStr"/>
+      <c r="O131" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P131" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q131" s="3" t="inlineStr">
@@ -16085,14 +16541,26 @@
       <c r="J132" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="K132" s="2" t="inlineStr"/>
-      <c r="L132" s="2" t="inlineStr"/>
-      <c r="M132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="L132" s="2" t="n">
+        <v>79.04000000000001</v>
+      </c>
+      <c r="M132" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/8-awg-black-tefzel-wire-m22759-16-8-0-cut-length?variant=40451555557411</t>
+        </is>
+      </c>
       <c r="N132" s="2" t="inlineStr"/>
-      <c r="O132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P132" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q132" s="2" t="inlineStr">
@@ -16142,14 +16610,26 @@
       <c r="J133" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="K133" s="3" t="inlineStr"/>
-      <c r="L133" s="3" t="inlineStr"/>
-      <c r="M133" s="3" t="inlineStr"/>
+      <c r="K133" s="3" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="L133" s="3" t="n">
+        <v>183</v>
+      </c>
+      <c r="M133" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/8-awg-red-tefzel-wire-m22759-16-8-2-cut-length?variant=40451557523491</t>
+        </is>
+      </c>
       <c r="N133" s="3" t="inlineStr"/>
-      <c r="O133" s="3" t="inlineStr"/>
+      <c r="O133" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P133" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q133" s="3" t="inlineStr">
@@ -16199,14 +16679,26 @@
       <c r="J134" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="K134" s="2" t="inlineStr"/>
-      <c r="L134" s="2" t="inlineStr"/>
-      <c r="M134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="L134" s="2" t="n">
+        <v>51.52</v>
+      </c>
+      <c r="M134" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/8-awg-white-tefzel-wire-m22759-16-8-9-spool?variant=40415055740963</t>
+        </is>
+      </c>
       <c r="N134" s="2" t="inlineStr"/>
-      <c r="O134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P134" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q134" s="2" t="inlineStr">
@@ -20255,66 +20747,105 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N130" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N130" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId113"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -20327,7 +20858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D142"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20630,7 +21161,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>12052641</t>
+          <t>2.2k 1/4W 1%</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -20640,7 +21171,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20652,12 +21183,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>12084200</t>
+          <t>52-45780</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Waytek listing seen 2026-10-19 (100 pc min, 0 stock; Aptiv sheet not checked)</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -20674,12 +21205,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>12110293</t>
+          <t>55A1811-20-9-9CS2275</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -20696,12 +21227,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>55A1821-20-6/9-9</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -20718,12 +21249,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>13519047</t>
+          <t>55A1831-20-2/4/6-9</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -20740,12 +21271,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>55A1841-20-2/4/5/6-9</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -20762,7 +21293,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>90980-10341</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -20772,7 +21303,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20784,7 +21315,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1/4W 1%</t>
+          <t>90980-10942</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -20794,7 +21325,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20806,7 +21337,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>52-45780</t>
+          <t>90980-11143</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -20816,7 +21347,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20828,17 +21359,17 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>55A1811-20-9-9CS2275</t>
+          <t>90980-11250</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20850,17 +21381,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>55A1821-20-6/9-9</t>
+          <t>90980-11885</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20872,17 +21403,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>55A1831-20-2/4/6-9</t>
+          <t>90980-12068</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20894,17 +21425,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>55A1841-20-2/4/5/6-9</t>
+          <t>BC-1/0-BLK</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20916,7 +21447,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>BC-1/0-RED</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -20926,7 +21457,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20938,7 +21469,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>90980-10341</t>
+          <t>BC-2-RED</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -20948,7 +21479,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20960,7 +21491,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>90980-10897</t>
+          <t>BC-4-BLK</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -20970,7 +21501,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20982,17 +21513,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>90980-10942</t>
+          <t>DR-25-1-1/2-0-SP</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21004,17 +21535,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>90980-11062</t>
+          <t>DR-25-2-0-SP</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21026,17 +21557,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>90980-11143</t>
+          <t>HD36-24-33SE</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21048,7 +21579,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>90980-11250</t>
+          <t>LP-16-J05PE-02-001</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -21058,7 +21589,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21070,7 +21601,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>90980-11885</t>
+          <t>M22759/16-14-60</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -21080,7 +21611,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21092,7 +21623,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>90980-12068</t>
+          <t>M22759/16-14-62</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -21102,7 +21633,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21114,7 +21645,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>BC-1/0-BLK</t>
+          <t>M22759/16-14-63</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -21124,7 +21655,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21136,7 +21667,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>BC-1/0-RED</t>
+          <t>M22759/16-14-69</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -21146,7 +21677,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21158,7 +21689,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>BC-2-RED</t>
+          <t>M22759/16-16-20</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -21168,7 +21699,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21180,7 +21711,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>BC-4-BLK</t>
+          <t>M22759/16-16-26</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -21190,7 +21721,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21202,7 +21733,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>D 261 205 358-01</t>
+          <t>M22759/16-16-50</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -21212,7 +21743,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21224,17 +21755,17 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1-0-SP</t>
+          <t>M22759/16-16-53</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21246,17 +21777,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1-1/2-0-SP</t>
+          <t>M22759/16-16-59</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21268,17 +21799,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1/2-0-SP</t>
+          <t>M22759/16-16-90</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21290,17 +21821,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1/4-0-SP</t>
+          <t>M22759/16-18-29</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21312,17 +21843,17 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>DR-25-2-0-SP</t>
+          <t>M22759/16-18-50</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21334,17 +21865,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>DR-25-3/16-0-SP</t>
+          <t>M22759/16-18-54</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21356,17 +21887,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>DR-25-3/4-0-SP</t>
+          <t>M22759/16-20-06</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21378,17 +21909,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>DR-25-3/8-0-SP</t>
+          <t>M22759/16-20-09</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21400,17 +21931,17 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>DTM06-6S</t>
+          <t>M22759/16-20-39</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21422,12 +21953,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>HD36-24-33SE</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -21444,7 +21975,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>LP-16-J05PE-02-001</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -21466,7 +21997,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-10-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -21476,7 +22007,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21488,7 +22019,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-10-1</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -21498,7 +22029,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21510,7 +22041,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-10-2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -21520,7 +22051,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21532,7 +22063,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-12-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -21542,7 +22073,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21554,7 +22085,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-12-2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -21564,7 +22095,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21576,7 +22107,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -21586,7 +22117,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21598,7 +22129,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-6</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -21608,7 +22139,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21620,7 +22151,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-60</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -21630,7 +22161,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21642,7 +22173,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-62</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -21652,7 +22183,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21664,7 +22195,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-63</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -21674,7 +22205,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21686,7 +22217,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-69</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -21696,7 +22227,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21708,7 +22239,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -21718,7 +22249,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21730,7 +22261,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-20</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -21740,7 +22271,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21752,7 +22283,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-26</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -21762,7 +22293,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21774,7 +22305,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-50</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -21784,7 +22315,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21796,7 +22327,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-53</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -21806,7 +22337,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21818,7 +22349,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-59</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -21828,7 +22359,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21840,7 +22371,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-90</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -21850,7 +22381,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21862,7 +22393,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -21872,7 +22403,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21884,7 +22415,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-29</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -21894,7 +22425,7 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21906,7 +22437,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-50</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -21916,7 +22447,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21928,7 +22459,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-54</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -21938,7 +22469,7 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21950,7 +22481,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-7</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -21960,7 +22491,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21972,7 +22503,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -21982,7 +22513,7 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21994,7 +22525,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -22004,7 +22535,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22016,7 +22547,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -22026,7 +22557,7 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22038,7 +22569,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-09</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -22048,7 +22579,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22060,7 +22591,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-1</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -22070,7 +22601,7 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22082,7 +22613,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -22092,7 +22623,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22104,7 +22635,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-39</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -22114,7 +22645,7 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22126,7 +22657,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -22136,7 +22667,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22148,7 +22679,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-5</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -22158,7 +22689,7 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22170,7 +22701,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -22180,7 +22711,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22192,7 +22723,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-7</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -22202,7 +22733,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22214,7 +22745,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-8</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -22224,7 +22755,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22236,17 +22767,17 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>seller page seen 2026-10-19 (per foot)</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22258,7 +22789,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-6-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -22268,7 +22799,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22280,7 +22811,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-8-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -22290,7 +22821,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22302,7 +22833,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-8-2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -22312,7 +22843,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22324,7 +22855,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-8-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -22334,7 +22865,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22536,932 +23067,8 @@
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C103" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B105" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C105" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C111" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C115" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B117" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C117" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D117" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C119" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D119" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C121" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D121" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C123" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D124" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B125" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C125" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D125" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B127" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C127" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D127" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B129" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C129" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D129" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D130" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B131" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C131" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D131" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B133" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C133" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D133" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B135" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C135" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D135" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B137" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C137" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D137" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B139" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C139" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D139" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B141" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C141" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D142"/>
+  <autoFilter ref="A1:D100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
BOM: 42 more prices from small Shopify vendors (Tefzel wire, DR-25, Aptiv/Sumitomo contacts) (#370)
* BOM: price 42 more lines from KSV Looms / Custom Connector Kits / Race Spec (Shopify)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* BOM xlsx regenerated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$205</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -546,10 +546,10 @@
         <v>193</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3252.25</v>
+        <v>4749.29</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -568,10 +568,10 @@
         <v>296</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>155</v>
+        <v>197</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3663.79</v>
+        <v>5160.83</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>23</v>
@@ -9242,14 +9242,26 @@
       <c r="J17" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/12052641?variant=45536631554366</t>
+        </is>
+      </c>
       <c r="N17" s="3" t="inlineStr"/>
-      <c r="O17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr"/>
@@ -9295,11 +9307,15 @@
       <c r="J18" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>2.24</v>
+      </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>https://waytekwire.com/product/aptiv-12084200-metri-pack-150-series-female</t>
+          <t>https://www.customconnectorkits.com/products/12084200-l?variant=45536283525438</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -9307,10 +9323,14 @@
           <t>https://www.ebay.de/itm/145990327082</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Waytek listing seen 2026-10-19 (100 pc min, 0 stock; Aptiv sheet not checked)</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -9425,14 +9445,26 @@
       <c r="J20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/12110293?variant=45536279953726</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
@@ -9478,14 +9510,26 @@
       <c r="J21" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/12191819-l?variant=45536512966974</t>
+        </is>
+      </c>
       <c r="N21" s="3" t="inlineStr"/>
-      <c r="O21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr"/>
@@ -9531,14 +9575,26 @@
       <c r="J22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/13519047?variant=45536514539838</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
@@ -9584,14 +9640,26 @@
       <c r="J23" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/15326426-l?variant=48621504332094</t>
+        </is>
+      </c>
       <c r="N23" s="3" t="inlineStr"/>
-      <c r="O23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr"/>
@@ -9637,14 +9705,26 @@
       <c r="J24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/15419715?variant=45536627917118</t>
+        </is>
+      </c>
       <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
@@ -11267,14 +11347,26 @@
       <c r="J50" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.customconnectorkits.com/products/8100-0461-l?variant=46049028800830</t>
+        </is>
+      </c>
       <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Custom Connector Kits, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
@@ -11365,14 +11457,26 @@
       <c r="J52" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/toyota-lexus-90980-10897-8-pin-connector-kit?variant=29504109805610</t>
+        </is>
+      </c>
       <c r="N52" s="2" t="inlineStr"/>
-      <c r="O52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; equivalent connector kit, not the OEM part: confirm it fits</t>
+        </is>
+      </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -11463,14 +11567,26 @@
       <c r="J54" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr"/>
-      <c r="M54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/2-way-connector-kit-for-toyota-lexus-90980-11062-water-temperature-sensor-22-18-awg?variant=11482559741994</t>
+        </is>
+      </c>
       <c r="N54" s="2" t="inlineStr"/>
-      <c r="O54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; equivalent connector kit, not the OEM part: confirm it fits</t>
+        </is>
+      </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
@@ -11948,14 +12064,26 @@
       <c r="J63" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K63" s="3" t="inlineStr"/>
-      <c r="L63" s="3" t="inlineStr"/>
-      <c r="M63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="L63" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/6-way-connector-kit-same-as-bosch-d261-205-358-01-23-20-awg?variant=40430818852899</t>
+        </is>
+      </c>
       <c r="N63" s="3" t="inlineStr"/>
-      <c r="O63" s="3" t="inlineStr"/>
+      <c r="O63" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; equivalent connector kit, not the OEM part: confirm it fits</t>
+        </is>
+      </c>
       <c r="P63" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q63" s="3" t="inlineStr"/>
@@ -12001,14 +12129,26 @@
       <c r="J64" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K64" s="2" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr"/>
-      <c r="M64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="n">
+        <v>20.08</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>60.24</v>
+      </c>
+      <c r="M64" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/1-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443737243683</t>
+        </is>
+      </c>
       <c r="N64" s="2" t="inlineStr"/>
-      <c r="O64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $6.12 per ft</t>
+        </is>
+      </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -12115,14 +12255,26 @@
       <c r="J66" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr"/>
-      <c r="M66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/1-2-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443735736355</t>
+        </is>
+      </c>
       <c r="N66" s="2" t="inlineStr"/>
-      <c r="O66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $4.34 per ft</t>
+        </is>
+      </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
@@ -12172,14 +12324,26 @@
       <c r="J67" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="K67" s="3" t="inlineStr"/>
-      <c r="L67" s="3" t="inlineStr"/>
-      <c r="M67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="L67" s="3" t="n">
+        <v>78.54000000000001</v>
+      </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/1-4-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443735113763</t>
+        </is>
+      </c>
       <c r="N67" s="3" t="inlineStr"/>
-      <c r="O67" s="3" t="inlineStr"/>
+      <c r="O67" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $1.71 per ft</t>
+        </is>
+      </c>
       <c r="P67" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q67" s="3" t="inlineStr">
@@ -12286,14 +12450,26 @@
       <c r="J69" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="K69" s="3" t="inlineStr"/>
-      <c r="L69" s="3" t="inlineStr"/>
-      <c r="M69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="L69" s="3" t="n">
+        <v>72.02</v>
+      </c>
+      <c r="M69" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/3-16-raychem-dr-25-yellow-label-heat-shrink-tubing-per-foot?variant=40443733803043</t>
+        </is>
+      </c>
       <c r="N69" s="3" t="inlineStr"/>
-      <c r="O69" s="3" t="inlineStr"/>
+      <c r="O69" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $1.69 per ft</t>
+        </is>
+      </c>
       <c r="P69" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q69" s="3" t="inlineStr">
@@ -12343,14 +12519,26 @@
       <c r="J70" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/3-4-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443737112611</t>
+        </is>
+      </c>
       <c r="N70" s="2" t="inlineStr"/>
-      <c r="O70" s="2" t="inlineStr"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $4.57 per ft</t>
+        </is>
+      </c>
       <c r="P70" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q70" s="2" t="inlineStr">
@@ -12400,14 +12588,26 @@
       <c r="J71" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="K71" s="3" t="inlineStr"/>
-      <c r="L71" s="3" t="inlineStr"/>
-      <c r="M71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>129.96</v>
+      </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/3-8-raychem-dr-25-yellow-label-heat-shrink-tubing?variant=40443735343139</t>
+        </is>
+      </c>
       <c r="N71" s="3" t="inlineStr"/>
-      <c r="O71" s="3" t="inlineStr"/>
+      <c r="O71" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20; $3.30 per ft</t>
+        </is>
+      </c>
       <c r="P71" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q71" s="3" t="inlineStr">
@@ -13529,18 +13729,26 @@
       <c r="J88" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>2.48</v>
+      </c>
       <c r="M88" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-DTM06-6S.html</t>
+          <t>https://www.ksvlooms.com/products/dtm06-6s-deutsch-dtm-housing?variant=43643315290147</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr"/>
-      <c r="O88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P88" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q88" s="2" t="inlineStr"/>
@@ -13692,14 +13900,26 @@
       <c r="J91" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K91" s="3" t="inlineStr"/>
-      <c r="L91" s="3" t="inlineStr"/>
-      <c r="M91" s="3" t="inlineStr"/>
+      <c r="K91" s="3" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="L91" s="3" t="n">
+        <v>16.32</v>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/10-awg-black-tefzel-wire-m22759-16-10-0-cut-length?variant=40451551199267</t>
+        </is>
+      </c>
       <c r="N91" s="3" t="inlineStr"/>
-      <c r="O91" s="3" t="inlineStr"/>
+      <c r="O91" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P91" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q91" s="3" t="inlineStr">
@@ -13749,14 +13969,26 @@
       <c r="J92" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr"/>
-      <c r="M92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>21.76</v>
+      </c>
+      <c r="M92" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/10-awg-brown-tefzel-wire-m22759-16-10-1-spool?variant=40423436288035</t>
+        </is>
+      </c>
       <c r="N92" s="2" t="inlineStr"/>
-      <c r="O92" s="2" t="inlineStr"/>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P92" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q92" s="2" t="inlineStr">
@@ -13806,14 +14038,26 @@
       <c r="J93" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="K93" s="3" t="inlineStr"/>
-      <c r="L93" s="3" t="inlineStr"/>
-      <c r="M93" s="3" t="inlineStr"/>
+      <c r="K93" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L93" s="3" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/10-awg-red-tefzel-wire-m22759-16-10-2-cut-length?variant=40451119939619</t>
+        </is>
+      </c>
       <c r="N93" s="3" t="inlineStr"/>
-      <c r="O93" s="3" t="inlineStr"/>
+      <c r="O93" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P93" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q93" s="3" t="inlineStr">
@@ -13863,14 +14107,26 @@
       <c r="J94" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K94" s="2" t="inlineStr"/>
-      <c r="L94" s="2" t="inlineStr"/>
-      <c r="M94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="L94" s="2" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="M94" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/12-awg-black-tefzel-wire-m22759-16-12-0-spool?variant=40415052726307</t>
+        </is>
+      </c>
       <c r="N94" s="2" t="inlineStr"/>
-      <c r="O94" s="2" t="inlineStr"/>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P94" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q94" s="2" t="inlineStr">
@@ -13920,14 +14176,26 @@
       <c r="J95" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="K95" s="3" t="inlineStr"/>
-      <c r="L95" s="3" t="inlineStr"/>
-      <c r="M95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="L95" s="3" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="M95" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/12-awg-red-tefzel-wire-m22759-16-12-2-spool?variant=40415053152291</t>
+        </is>
+      </c>
       <c r="N95" s="3" t="inlineStr"/>
-      <c r="O95" s="3" t="inlineStr"/>
+      <c r="O95" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P95" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q95" s="3" t="inlineStr">
@@ -13977,14 +14245,26 @@
       <c r="J96" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K96" s="2" t="inlineStr"/>
-      <c r="L96" s="2" t="inlineStr"/>
-      <c r="M96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/14-awg-black-tefzel-wire-m22759-16-14-0-spool?variant=40415048695843</t>
+        </is>
+      </c>
       <c r="N96" s="2" t="inlineStr"/>
-      <c r="O96" s="2" t="inlineStr"/>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P96" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q96" s="2" t="inlineStr">
@@ -14103,14 +14383,26 @@
       <c r="J98" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K98" s="2" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr"/>
-      <c r="M98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="L98" s="2" t="n">
+        <v>87.36</v>
+      </c>
+      <c r="M98" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/14-awg-blue-tefzel-wire-m22759-16-14-6-spool?variant=40423417708579</t>
+        </is>
+      </c>
       <c r="N98" s="2" t="inlineStr"/>
-      <c r="O98" s="2" t="inlineStr"/>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P98" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q98" s="2" t="inlineStr">
@@ -14388,14 +14680,26 @@
       <c r="J103" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="K103" s="3" t="inlineStr"/>
-      <c r="L103" s="3" t="inlineStr"/>
-      <c r="M103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="L103" s="3" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="M103" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/16-awg-black-tefzel-wire-m22759-16-16-0-spool?variant=40415046434851</t>
+        </is>
+      </c>
       <c r="N103" s="3" t="inlineStr"/>
-      <c r="O103" s="3" t="inlineStr"/>
+      <c r="O103" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P103" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q103" s="3" t="inlineStr">
@@ -14856,14 +15160,26 @@
       <c r="J111" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K111" s="3" t="inlineStr"/>
-      <c r="L111" s="3" t="inlineStr"/>
-      <c r="M111" s="3" t="inlineStr"/>
+      <c r="K111" s="3" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="L111" s="3" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/18-awg-black-tefzel-wire-m22759-16-18-0-spool?variant=40415044370467</t>
+        </is>
+      </c>
       <c r="N111" s="3" t="inlineStr"/>
-      <c r="O111" s="3" t="inlineStr"/>
+      <c r="O111" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P111" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q111" s="3" t="inlineStr">
@@ -15153,14 +15469,26 @@
       <c r="J116" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K116" s="2" t="inlineStr"/>
-      <c r="L116" s="2" t="inlineStr"/>
-      <c r="M116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>38.08</v>
+      </c>
+      <c r="M116" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/18-awg-purple-tefzel-wire-m22759-16-18-7-spool?variant=40423402700835</t>
+        </is>
+      </c>
       <c r="N116" s="2" t="inlineStr"/>
-      <c r="O116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P116" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q116" s="2" t="inlineStr">
@@ -15210,14 +15538,26 @@
       <c r="J117" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="K117" s="3" t="inlineStr"/>
-      <c r="L117" s="3" t="inlineStr"/>
-      <c r="M117" s="3" t="inlineStr"/>
+      <c r="K117" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L117" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="M117" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/18-awg-white-tefzel-wire-m22759-16-18-9-spool?variant=40415044829219</t>
+        </is>
+      </c>
       <c r="N117" s="3" t="inlineStr"/>
-      <c r="O117" s="3" t="inlineStr"/>
+      <c r="O117" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P117" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q117" s="3" t="inlineStr">
@@ -15267,14 +15607,26 @@
       <c r="J118" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="K118" s="2" t="inlineStr"/>
-      <c r="L118" s="2" t="inlineStr"/>
-      <c r="M118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="L118" s="2" t="n">
+        <v>27.72</v>
+      </c>
+      <c r="M118" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-black-tefzel-wire-m22759-16-20-0-spool?variant=40415026577443</t>
+        </is>
+      </c>
       <c r="N118" s="2" t="inlineStr"/>
-      <c r="O118" s="2" t="inlineStr"/>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P118" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q118" s="2" t="inlineStr">
@@ -15438,14 +15790,26 @@
       <c r="J121" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="K121" s="3" t="inlineStr"/>
-      <c r="L121" s="3" t="inlineStr"/>
-      <c r="M121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L121" s="3" t="n">
+        <v>23.52</v>
+      </c>
+      <c r="M121" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-brown-tefzel-wire-m22759-16-20-1-spool?variant=40415026708515</t>
+        </is>
+      </c>
       <c r="N121" s="3" t="inlineStr"/>
-      <c r="O121" s="3" t="inlineStr"/>
+      <c r="O121" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P121" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q121" s="3" t="inlineStr">
@@ -15564,14 +15928,26 @@
       <c r="J123" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="K123" s="3" t="inlineStr"/>
-      <c r="L123" s="3" t="inlineStr"/>
-      <c r="M123" s="3" t="inlineStr"/>
+      <c r="K123" s="3" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L123" s="3" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="M123" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-orange-tefzel-wire-m22759-16-20-3-spool?variant=40415028019235</t>
+        </is>
+      </c>
       <c r="N123" s="3" t="inlineStr"/>
-      <c r="O123" s="3" t="inlineStr"/>
+      <c r="O123" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P123" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q123" s="3" t="inlineStr">
@@ -15678,14 +16054,26 @@
       <c r="J125" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="K125" s="3" t="inlineStr"/>
-      <c r="L125" s="3" t="inlineStr"/>
-      <c r="M125" s="3" t="inlineStr"/>
+      <c r="K125" s="3" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="L125" s="3" t="n">
+        <v>36.96</v>
+      </c>
+      <c r="M125" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-yellow-tefzel-wire-m22759-16-20-4-spool?variant=40415028477987</t>
+        </is>
+      </c>
       <c r="N125" s="3" t="inlineStr"/>
-      <c r="O125" s="3" t="inlineStr"/>
+      <c r="O125" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P125" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q125" s="3" t="inlineStr">
@@ -15735,14 +16123,26 @@
       <c r="J126" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="K126" s="2" t="inlineStr"/>
-      <c r="L126" s="2" t="inlineStr"/>
-      <c r="M126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="M126" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-green-tefzel-wire-m22759-16-20-5-spool?variant=40415028838435</t>
+        </is>
+      </c>
       <c r="N126" s="2" t="inlineStr"/>
-      <c r="O126" s="2" t="inlineStr"/>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
@@ -15792,14 +16192,26 @@
       <c r="J127" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="K127" s="3" t="inlineStr"/>
-      <c r="L127" s="3" t="inlineStr"/>
-      <c r="M127" s="3" t="inlineStr"/>
+      <c r="K127" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L127" s="3" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="M127" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-blue-tefzel-wire-m22759-16-20-6-spool?variant=40415028903971</t>
+        </is>
+      </c>
       <c r="N127" s="3" t="inlineStr"/>
-      <c r="O127" s="3" t="inlineStr"/>
+      <c r="O127" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P127" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q127" s="3" t="inlineStr">
@@ -15849,14 +16261,26 @@
       <c r="J128" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="K128" s="2" t="inlineStr"/>
-      <c r="L128" s="2" t="inlineStr"/>
-      <c r="M128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>24.36</v>
+      </c>
+      <c r="M128" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-purple-tefzel-wire-m22759-16-20-7-spool?variant=40415029198883</t>
+        </is>
+      </c>
       <c r="N128" s="2" t="inlineStr"/>
-      <c r="O128" s="2" t="inlineStr"/>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P128" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q128" s="2" t="inlineStr">
@@ -15906,14 +16330,26 @@
       <c r="J129" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="K129" s="3" t="inlineStr"/>
-      <c r="L129" s="3" t="inlineStr"/>
-      <c r="M129" s="3" t="inlineStr"/>
+      <c r="K129" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L129" s="3" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="M129" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/20-awg-gray-tefzel-wire-m22759-16-20-8-spool?variant=40415029264419</t>
+        </is>
+      </c>
       <c r="N129" s="3" t="inlineStr"/>
-      <c r="O129" s="3" t="inlineStr"/>
+      <c r="O129" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P129" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q129" s="3" t="inlineStr">
@@ -15963,11 +16399,15 @@
       <c r="J130" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="K130" s="2" t="inlineStr"/>
-      <c r="L130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L130" s="2" t="n">
+        <v>31.68</v>
+      </c>
       <c r="M130" s="4" t="inlineStr">
         <is>
-          <t>https://wingsandwheels.com/tefzel-wire-20-gauge-new.html</t>
+          <t>https://www.ksvlooms.com/products/20-awg-white-tefzel-wire-m22759-16-20-9-spool?variant=40415029297187</t>
         </is>
       </c>
       <c r="N130" s="4" t="inlineStr">
@@ -15975,10 +16415,14 @@
           <t>https://www.flightstore.com.au/M22759/16-Extruded-ETFE-Tefzel-Wire-20AWG-Per-FT</t>
         </is>
       </c>
-      <c r="O130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P130" s="2" t="inlineStr">
         <is>
-          <t>seller page seen 2026-10-19 (per foot)</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
@@ -16028,14 +16472,26 @@
       <c r="J131" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K131" s="3" t="inlineStr"/>
-      <c r="L131" s="3" t="inlineStr"/>
-      <c r="M131" s="3" t="inlineStr"/>
+      <c r="K131" s="3" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="L131" s="3" t="n">
+        <v>64.72</v>
+      </c>
+      <c r="M131" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/6-awg-white-tefzel-wire-m22759-16-6-9-spool?variant=40415058198563</t>
+        </is>
+      </c>
       <c r="N131" s="3" t="inlineStr"/>
-      <c r="O131" s="3" t="inlineStr"/>
+      <c r="O131" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P131" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q131" s="3" t="inlineStr">
@@ -16085,14 +16541,26 @@
       <c r="J132" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="K132" s="2" t="inlineStr"/>
-      <c r="L132" s="2" t="inlineStr"/>
-      <c r="M132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="L132" s="2" t="n">
+        <v>79.04000000000001</v>
+      </c>
+      <c r="M132" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/8-awg-black-tefzel-wire-m22759-16-8-0-cut-length?variant=40451555557411</t>
+        </is>
+      </c>
       <c r="N132" s="2" t="inlineStr"/>
-      <c r="O132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P132" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q132" s="2" t="inlineStr">
@@ -16142,14 +16610,26 @@
       <c r="J133" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="K133" s="3" t="inlineStr"/>
-      <c r="L133" s="3" t="inlineStr"/>
-      <c r="M133" s="3" t="inlineStr"/>
+      <c r="K133" s="3" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="L133" s="3" t="n">
+        <v>183</v>
+      </c>
+      <c r="M133" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/8-awg-red-tefzel-wire-m22759-16-8-2-cut-length?variant=40451557523491</t>
+        </is>
+      </c>
       <c r="N133" s="3" t="inlineStr"/>
-      <c r="O133" s="3" t="inlineStr"/>
+      <c r="O133" s="3" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P133" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q133" s="3" t="inlineStr">
@@ -16199,14 +16679,26 @@
       <c r="J134" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="K134" s="2" t="inlineStr"/>
-      <c r="L134" s="2" t="inlineStr"/>
-      <c r="M134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="L134" s="2" t="n">
+        <v>51.52</v>
+      </c>
+      <c r="M134" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksvlooms.com/products/8-awg-white-tefzel-wire-m22759-16-8-9-spool?variant=40415055740963</t>
+        </is>
+      </c>
       <c r="N134" s="2" t="inlineStr"/>
-      <c r="O134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>KSV Looms, 2026-10-20</t>
+        </is>
+      </c>
       <c r="P134" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>vendor page read 2026-10-20 (products.json), in stock</t>
         </is>
       </c>
       <c r="Q134" s="2" t="inlineStr">
@@ -20255,66 +20747,105 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N130" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N130" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M202" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M203" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId113"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -20327,7 +20858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D142"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20630,7 +21161,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>12052641</t>
+          <t>2.2k 1/4W 1%</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -20640,7 +21171,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
         </is>
       </c>
     </row>
@@ -20652,12 +21183,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>12084200</t>
+          <t>52-45780</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Waytek listing seen 2026-10-19 (100 pc min, 0 stock; Aptiv sheet not checked)</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -20674,12 +21205,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>12110293</t>
+          <t>55A1811-20-9-9CS2275</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -20696,12 +21227,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>55A1821-20-6/9-9</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -20718,12 +21249,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>13519047</t>
+          <t>55A1831-20-2/4/6-9</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -20740,12 +21271,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>55A1841-20-2/4/5/6-9</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -20762,7 +21293,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>90980-10341</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -20772,7 +21303,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20784,7 +21315,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1/4W 1%</t>
+          <t>90980-10942</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -20794,7 +21325,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>generic part: name a real PN (TE first, then an approved supplier); I propose one on your OK</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20806,7 +21337,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>52-45780</t>
+          <t>90980-11143</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -20816,7 +21347,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20828,17 +21359,17 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>55A1811-20-9-9CS2275</t>
+          <t>90980-11250</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20850,17 +21381,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>55A1821-20-6/9-9</t>
+          <t>90980-11885</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20872,17 +21403,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>55A1831-20-2/4/6-9</t>
+          <t>90980-12068</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20894,17 +21425,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>55A1841-20-2/4/5/6-9</t>
+          <t>BC-1/0-BLK</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20916,7 +21447,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>BC-1/0-RED</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -20926,7 +21457,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20938,7 +21469,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>90980-10341</t>
+          <t>BC-2-RED</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -20948,7 +21479,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20960,7 +21491,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>90980-10897</t>
+          <t>BC-4-BLK</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -20970,7 +21501,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20982,17 +21513,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>90980-10942</t>
+          <t>DR-25-1-1/2-0-SP</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21004,17 +21535,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>90980-11062</t>
+          <t>DR-25-2-0-SP</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21026,17 +21557,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>90980-11143</t>
+          <t>HD36-24-33SE</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21048,7 +21579,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>90980-11250</t>
+          <t>LP-16-J05PE-02-001</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -21058,7 +21589,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21070,7 +21601,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>90980-11885</t>
+          <t>M22759/16-14-60</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -21080,7 +21611,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21092,7 +21623,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>90980-12068</t>
+          <t>M22759/16-14-62</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -21102,7 +21633,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21114,7 +21645,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>BC-1/0-BLK</t>
+          <t>M22759/16-14-63</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -21124,7 +21655,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21136,7 +21667,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>BC-1/0-RED</t>
+          <t>M22759/16-14-69</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -21146,7 +21677,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21158,7 +21689,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>BC-2-RED</t>
+          <t>M22759/16-16-20</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -21168,7 +21699,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21180,7 +21711,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>BC-4-BLK</t>
+          <t>M22759/16-16-26</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -21190,7 +21721,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21202,7 +21733,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>D 261 205 358-01</t>
+          <t>M22759/16-16-50</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -21212,7 +21743,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21224,17 +21755,17 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1-0-SP</t>
+          <t>M22759/16-16-53</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21246,17 +21777,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1-1/2-0-SP</t>
+          <t>M22759/16-16-59</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21268,17 +21799,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>DR-25-1/2-0-SP</t>
+          <t>M22759/16-16-90</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21290,17 +21821,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1/4-0-SP</t>
+          <t>M22759/16-18-29</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21312,17 +21843,17 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>DR-25-2-0-SP</t>
+          <t>M22759/16-18-50</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21334,17 +21865,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>DR-25-3/16-0-SP</t>
+          <t>M22759/16-18-54</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21356,17 +21887,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>DR-25-3/4-0-SP</t>
+          <t>M22759/16-20-06</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21378,17 +21909,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>DR-25-3/8-0-SP</t>
+          <t>M22759/16-20-09</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21400,17 +21931,17 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>DTM06-6S</t>
+          <t>M22759/16-20-39</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21422,12 +21953,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>HD36-24-33SE</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -21444,7 +21975,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>LP-16-J05PE-02-001</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -21466,7 +21997,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-10-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -21476,7 +22007,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21488,7 +22019,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-10-1</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -21498,7 +22029,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21510,7 +22041,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-10-2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -21520,7 +22051,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21532,7 +22063,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-12-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -21542,7 +22073,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21554,7 +22085,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-12-2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -21564,7 +22095,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21576,7 +22107,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -21586,7 +22117,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21598,7 +22129,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-6</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -21608,7 +22139,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21620,7 +22151,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-60</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -21630,7 +22161,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21642,7 +22173,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-62</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -21652,7 +22183,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21664,7 +22195,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-14-63</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -21674,7 +22205,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21686,7 +22217,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-69</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -21696,7 +22227,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21708,7 +22239,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -21718,7 +22249,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21730,7 +22261,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-20</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -21740,7 +22271,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21752,7 +22283,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-26</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -21762,7 +22293,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21774,7 +22305,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-50</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -21784,7 +22315,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21796,7 +22327,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-53</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -21806,7 +22337,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21818,7 +22349,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-16-59</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -21828,7 +22359,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21840,7 +22371,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-90</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -21850,7 +22381,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21862,7 +22393,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -21872,7 +22403,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21884,7 +22415,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-29</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -21894,7 +22425,7 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21906,7 +22437,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-50</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -21916,7 +22447,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21928,7 +22459,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-54</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -21938,7 +22469,7 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21950,7 +22481,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-7</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -21960,7 +22491,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21972,7 +22503,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-18-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -21982,7 +22513,7 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -21994,7 +22525,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -22004,7 +22535,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22016,7 +22547,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -22026,7 +22557,7 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22038,7 +22569,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-09</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -22048,7 +22579,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22060,7 +22591,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-1</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -22070,7 +22601,7 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22082,7 +22613,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-3</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -22092,7 +22623,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22104,7 +22635,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-39</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -22114,7 +22645,7 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22126,7 +22657,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-4</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -22136,7 +22667,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22148,7 +22679,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-5</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -22158,7 +22689,7 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22170,7 +22701,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-6</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -22180,7 +22711,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22192,7 +22723,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-7</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -22202,7 +22733,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22214,7 +22745,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-20-8</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -22224,7 +22755,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22236,17 +22767,17 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-20-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>seller page seen 2026-10-19 (per foot)</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22258,7 +22789,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-6-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -22268,7 +22799,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22280,7 +22811,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-8-0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -22290,7 +22821,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22302,7 +22833,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-8-2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -22312,7 +22843,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22324,7 +22855,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-8-9</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -22334,7 +22865,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -22536,932 +23067,8 @@
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C103" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B105" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C105" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C111" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C115" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B117" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C117" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D117" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C119" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D119" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C121" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D121" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C123" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D124" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B125" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C125" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D125" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B127" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C127" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D127" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B129" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C129" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D129" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D130" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B131" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C131" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D131" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B133" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C133" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D133" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B135" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C135" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D135" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B137" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C137" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D137" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B139" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C139" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D139" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B141" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C141" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D142"/>
+  <autoFilter ref="A1:D100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
A/C defaults (Dan: no preference): SP-AC-SGND for E10, lamp accepted, k_fan2 on Aux 4
Dan answered "no preference" on the four follow-ups, so the recommended
options are applied for his confirmation in #387:
- N63 = A: new cabin splice SP-AC-SGND rebuilds the engine-bay splice E10
  (1993 EWD p.211): Y cowl leads from IQ3 pin 1 (A32 pin 15), IJ1 pin 5
  (A24 pin 3), splice I8 (A21 / A18 pin 2) and the A1 return w_tam_rtn
- N64 = A: the A/C lamp also lights with the blower off; accepted, no part
- row 162 = C: k_fan2 trigger moved Ign 5 (B13) -> Aux 4 (A18), fly-wheeled;
  checked against the PCLink G4X help back-feeding note: coil+ is the SW12
  rail from k_efi, the ECU's own feed
- row 163 left as logged
Drawing set, IO table and BOM regenerated.

Rows: 162

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TQqczMtDLMgNuc99KxpaHx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$115</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,16 +540,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>103</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4787.24</v>
+        <v>4788.32</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>195</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5198.78</v>
+        <v>5199.86</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>23</v>
@@ -8127,7 +8127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q201"/>
+  <dimension ref="A1:Q200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16049,7 +16049,7 @@
         </is>
       </c>
       <c r="G125" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
@@ -16060,13 +16060,13 @@
         <v>0</v>
       </c>
       <c r="J125" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K125" s="3" t="n">
         <v>1.08</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>19.44</v>
+        <v>20.52</v>
       </c>
       <c r="M125" s="5" t="inlineStr">
         <is>
@@ -16086,7 +16086,7 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>4.6 m in the master + 15% margin</t>
+          <t>4.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16963,7 +16963,7 @@
       </c>
       <c r="Q138" s="2" t="inlineStr">
         <is>
-          <t>580 bands of 6 mm, both ends of each wire</t>
+          <t>586 bands of 6 mm, both ends of each wire</t>
         </is>
       </c>
     </row>
@@ -17093,7 +17093,7 @@
       </c>
       <c r="Q140" s="2" t="inlineStr">
         <is>
-          <t>420 bands of 6 mm, both ends of each wire</t>
+          <t>432 bands of 6 mm, both ends of each wire</t>
         </is>
       </c>
     </row>
@@ -17488,11 +17488,11 @@
       <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-A) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -17503,7 +17503,7 @@
         <v>0</v>
       </c>
       <c r="J148" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr"/>
@@ -17541,11 +17541,11 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ETB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G149" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
@@ -17556,7 +17556,7 @@
         <v>0</v>
       </c>
       <c r="J149" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K149" s="3" t="inlineStr"/>
       <c r="L149" s="3" t="inlineStr"/>
@@ -17594,11 +17594,11 @@
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ETB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -17609,7 +17609,7 @@
         <v>0</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
@@ -17647,11 +17647,11 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G151" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
@@ -17662,7 +17662,7 @@
         <v>0</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K151" s="3" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr"/>
@@ -17700,11 +17700,11 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -17715,7 +17715,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
@@ -17753,11 +17753,11 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KNOCK-1) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G153" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
@@ -17768,7 +17768,7 @@
         <v>0</v>
       </c>
       <c r="J153" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K153" s="3" t="inlineStr"/>
       <c r="L153" s="3" t="inlineStr"/>
@@ -17806,7 +17806,7 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KNOCK-1) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-A) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G154" s="2" t="n">
@@ -17859,11 +17859,11 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-A) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G155" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
@@ -17874,7 +17874,7 @@
         <v>0</v>
       </c>
       <c r="J155" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K155" s="3" t="inlineStr"/>
       <c r="L155" s="3" t="inlineStr"/>
@@ -17912,11 +17912,11 @@
       <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -17927,7 +17927,7 @@
         <v>0</v>
       </c>
       <c r="J156" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr"/>
@@ -17965,11 +17965,11 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G157" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
@@ -17980,7 +17980,7 @@
         <v>0</v>
       </c>
       <c r="J157" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K157" s="3" t="inlineStr"/>
       <c r="L157" s="3" t="inlineStr"/>
@@ -18018,7 +18018,7 @@
       <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G158" s="2" t="n">
@@ -18071,7 +18071,7 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G159" s="3" t="n">
@@ -18124,7 +18124,7 @@
       <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G160" s="2" t="n">
@@ -18177,7 +18177,7 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -18230,7 +18230,7 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G162" s="2" t="n">
@@ -18283,7 +18283,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G163" s="3" t="n">
@@ -18336,7 +18336,7 @@
       <c r="E164" s="2" t="inlineStr"/>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (CAM) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G164" s="2" t="n">
@@ -18389,7 +18389,7 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (CAM) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
@@ -18442,7 +18442,7 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G166" s="2" t="n">
@@ -18495,7 +18495,7 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G167" s="3" t="n">
@@ -18548,7 +18548,7 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
@@ -18601,7 +18601,7 @@
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (ENG-GND-RING) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G169" s="3" t="n">
@@ -18654,11 +18654,11 @@
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (ENG-GND-RING) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -18669,7 +18669,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K170" s="2" t="inlineStr"/>
       <c r="L170" s="2" t="inlineStr"/>
@@ -18707,11 +18707,11 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
@@ -18722,7 +18722,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K171" s="3" t="inlineStr"/>
       <c r="L171" s="3" t="inlineStr"/>
@@ -18760,11 +18760,11 @@
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18775,7 +18775,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K172" s="2" t="inlineStr"/>
       <c r="L172" s="2" t="inlineStr"/>
@@ -18813,11 +18813,11 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
@@ -18828,7 +18828,7 @@
         <v>0</v>
       </c>
       <c r="J173" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K173" s="3" t="inlineStr"/>
       <c r="L173" s="3" t="inlineStr"/>
@@ -18866,7 +18866,7 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (STARTER-TRIGGER) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
@@ -18919,7 +18919,7 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (STARTER-TRIGGER) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
@@ -18972,11 +18972,11 @@
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -18987,7 +18987,7 @@
         <v>0</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K176" s="2" t="inlineStr"/>
       <c r="L176" s="2" t="inlineStr"/>
@@ -19025,7 +19025,7 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
@@ -19078,11 +19078,11 @@
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -19093,7 +19093,7 @@
         <v>0</v>
       </c>
       <c r="J178" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K178" s="2" t="inlineStr"/>
       <c r="L178" s="2" t="inlineStr"/>
@@ -19131,7 +19131,7 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
@@ -19184,7 +19184,7 @@
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19237,7 +19237,7 @@
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G181" s="3" t="n">
@@ -19290,7 +19290,7 @@
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-RL-GND-BL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G182" s="2" t="n">
@@ -19343,7 +19343,7 @@
       <c r="E183" s="3" t="inlineStr"/>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-RL-GND-BL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
@@ -19396,7 +19396,7 @@
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G184" s="2" t="n">
@@ -19449,7 +19449,7 @@
       <c r="E185" s="3" t="inlineStr"/>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G185" s="3" t="n">
@@ -19502,7 +19502,7 @@
       <c r="E186" s="2" t="inlineStr"/>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G186" s="2" t="n">
@@ -19555,7 +19555,7 @@
       <c r="E187" s="3" t="inlineStr"/>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G187" s="3" t="n">
@@ -19608,22 +19608,22 @@
       <c r="E188" s="2" t="inlineStr"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>shielded cable, part number not confirmed: CAB-CAN-CLU, CAB-CAN-CSB, CAB-CAN-ECU, CAB-CAN-RD, CAB-CANBH-BC, CAB-ETBM-AE, CAB-LAMCAN-BE</t>
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>ft</t>
         </is>
       </c>
       <c r="I188" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J188" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
       <c r="L188" s="2" t="inlineStr"/>
@@ -19637,7 +19637,7 @@
       </c>
       <c r="Q188" s="2" t="inlineStr">
         <is>
-          <t>no maker document in the repo yet; never guessed</t>
+          <t>OPEN-ITEMS row 140</t>
         </is>
       </c>
     </row>
@@ -19654,45 +19654,53 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D189" s="3" t="inlineStr"/>
+          <t>TMS-SCE-1/2-2.0-9</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E189" s="3" t="inlineStr"/>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>shielded cable, part number not confirmed: CAB-CAN-CLU, CAB-CAN-CSB, CAB-CAN-ECU, CAB-CAN-RD, CAB-CANBH-BC, CAB-ETBM-AE, CAB-LAMCAN-BE</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G189" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>ft</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I189" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J189" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="K189" s="3" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="K189" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L189" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="M189" s="3" t="inlineStr"/>
       <c r="N189" s="3" t="inlineStr"/>
-      <c r="O189" s="3" t="inlineStr"/>
+      <c r="O189" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q189" s="3" t="inlineStr">
-        <is>
-          <t>OPEN-ITEMS row 140</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q189" s="3" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -19707,7 +19715,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
+          <t>TMS-SCE-3/16-2.0-9</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -19718,11 +19726,11 @@
       <c r="E190" s="2" t="inlineStr"/>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -19733,7 +19741,7 @@
         <v>0</v>
       </c>
       <c r="J190" s="2" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="K190" s="2" t="n">
         <v>0</v>
@@ -19768,7 +19776,7 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>TMS-SCE-3/8-2.0-9</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -19779,11 +19787,11 @@
       <c r="E191" s="3" t="inlineStr"/>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G191" s="3" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
@@ -19794,7 +19802,7 @@
         <v>0</v>
       </c>
       <c r="J191" s="3" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="K191" s="3" t="n">
         <v>0</v>
@@ -19829,22 +19837,22 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>W12S</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
+          <t>Deutsch (TE Connectivity)</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr"/>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -19852,27 +19860,31 @@
         </is>
       </c>
       <c r="I192" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="K192" s="2" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="L192" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M192" s="2" t="inlineStr"/>
+        <v>1.26</v>
+      </c>
+      <c r="M192" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
+        </is>
+      </c>
       <c r="N192" s="2" t="inlineStr"/>
       <c r="O192" s="2" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P192" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
         </is>
       </c>
       <c r="Q192" s="2" t="inlineStr"/>
@@ -19890,22 +19902,26 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>W2P</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
-        </is>
-      </c>
-      <c r="E193" s="3" t="inlineStr"/>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G193" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H193" s="3" t="inlineStr">
         <is>
@@ -19913,31 +19929,31 @@
         </is>
       </c>
       <c r="I193" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J193" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J193" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="K193" s="3" t="n">
-        <v>0.42</v>
+        <v>0.13</v>
       </c>
       <c r="L193" s="3" t="n">
-        <v>1.26</v>
+        <v>0.26</v>
       </c>
       <c r="M193" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="N193" s="3" t="inlineStr"/>
       <c r="O193" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 1, 2026-10-19</t>
         </is>
       </c>
       <c r="P193" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q193" s="3" t="inlineStr"/>
@@ -19955,7 +19971,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>W2S</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -19970,11 +19986,11 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -19985,28 +20001,28 @@
         <v>0</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="K194" s="2" t="n">
         <v>0.13</v>
       </c>
       <c r="L194" s="2" t="n">
-        <v>0.26</v>
+        <v>1.43</v>
       </c>
       <c r="M194" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+          <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="N194" s="2" t="inlineStr"/>
       <c r="O194" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q194" s="2" t="inlineStr"/>
@@ -20024,12 +20040,12 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
+          <t>Deutsch</t>
         </is>
       </c>
       <c r="E195" s="3" t="inlineStr">
@@ -20039,11 +20055,11 @@
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G195" s="3" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
@@ -20054,17 +20070,17 @@
         <v>0</v>
       </c>
       <c r="J195" s="3" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K195" s="3" t="n">
         <v>0.13</v>
       </c>
       <c r="L195" s="3" t="n">
-        <v>1.43</v>
+        <v>0.26</v>
       </c>
       <c r="M195" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="N195" s="3" t="inlineStr"/>
@@ -20075,7 +20091,7 @@
       </c>
       <c r="P195" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q195" s="3" t="inlineStr"/>
@@ -20093,12 +20109,12 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -20108,7 +20124,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G196" s="2" t="n">
@@ -20126,25 +20142,25 @@
         <v>2</v>
       </c>
       <c r="K196" s="2" t="n">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="L196" s="2" t="n">
-        <v>0.26</v>
+        <v>0.4</v>
       </c>
       <c r="M196" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
         </is>
       </c>
       <c r="N196" s="2" t="inlineStr"/>
       <c r="O196" s="2" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q196" s="2" t="inlineStr"/>
@@ -20162,7 +20178,7 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -20177,7 +20193,7 @@
       </c>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G197" s="3" t="n">
@@ -20195,14 +20211,14 @@
         <v>2</v>
       </c>
       <c r="K197" s="3" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="L197" s="3" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="M197" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N197" s="3" t="inlineStr"/>
@@ -20213,7 +20229,7 @@
       </c>
       <c r="P197" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q197" s="3" t="inlineStr"/>
@@ -20231,7 +20247,7 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -20246,11 +20262,11 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -20261,28 +20277,28 @@
         <v>0</v>
       </c>
       <c r="J198" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K198" s="2" t="n">
-        <v>0.21</v>
+        <v>0.35</v>
       </c>
       <c r="L198" s="2" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="M198" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N198" s="2" t="inlineStr"/>
       <c r="O198" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
         </is>
       </c>
       <c r="Q198" s="2" t="inlineStr"/>
@@ -20300,7 +20316,7 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>WM-4S</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -20315,7 +20331,7 @@
       </c>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
         </is>
       </c>
       <c r="G199" s="3" t="n">
@@ -20333,14 +20349,14 @@
         <v>1</v>
       </c>
       <c r="K199" s="3" t="n">
-        <v>0.35</v>
+        <v>0.28</v>
       </c>
       <c r="L199" s="3" t="n">
-        <v>0.35</v>
+        <v>0.28</v>
       </c>
       <c r="M199" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
         </is>
       </c>
       <c r="N199" s="3" t="inlineStr"/>
@@ -20351,7 +20367,7 @@
       </c>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
         </is>
       </c>
       <c r="Q199" s="3" t="inlineStr"/>
@@ -20369,12 +20385,12 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>WM-4S</t>
+          <t>WM-6S</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
+          <t>Deutsch</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
@@ -20384,7 +20400,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
         </is>
       </c>
       <c r="G200" s="2" t="n">
@@ -20402,14 +20418,14 @@
         <v>1</v>
       </c>
       <c r="K200" s="2" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="L200" s="2" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="M200" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
         </is>
       </c>
       <c r="N200" s="2" t="inlineStr"/>
@@ -20420,82 +20436,13 @@
       </c>
       <c r="P200" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
         </is>
       </c>
       <c r="Q200" s="2" t="inlineStr"/>
     </row>
-    <row r="201">
-      <c r="A201" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>WM-6S</t>
-        </is>
-      </c>
-      <c r="D201" s="3" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="E201" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F201" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
-        </is>
-      </c>
-      <c r="G201" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H201" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I201" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J201" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K201" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="L201" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="M201" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
-        </is>
-      </c>
-      <c r="N201" s="3" t="inlineStr"/>
-      <c r="O201" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
-      <c r="P201" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
-        </is>
-      </c>
-      <c r="Q201" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q201"/>
+  <autoFilter ref="A1:Q200"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -20599,15 +20546,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M201" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId111"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -20620,7 +20567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22763,30 +22710,8 @@
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D98"/>
+  <autoFilter ref="A1:D97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
D3/D7/D9/D10/D11: C17 clutch tap, CAN branch splice rule, pedal lengths, GT150 plugs, A15 test page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TQqczMtDLMgNuc99KxpaHx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -11247,7 +11247,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -11258,7 +11258,7 @@
         <v>0</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
@@ -11276,7 +11276,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>6 cable runs, 5.9 m + 15% margin</t>
+          <t>6 cable runs, 5.2 m + 15% margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the drawing set and BOM from the master
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TQqczMtDLMgNuc99KxpaHx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$116</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$183</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,16 +540,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4774.69</v>
+        <v>4768.97</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5212.55</v>
+        <v>5206.83</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>24</v>
@@ -8162,7 +8162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q183"/>
+  <dimension ref="A1:Q186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9329,7 +9329,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -9340,13 +9340,13 @@
         <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>0.16</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>2.24</v>
+        <v>0.32</v>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
@@ -9452,7 +9452,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>12110293</t>
+          <t>12191819</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -9463,7 +9463,7 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>CONNECTOR, PLUG, METRI-PACK 150.2, 3 POS, SEALED, SOCKET CONTACTS</t>
+          <t>CONTACT, SOCKET, CRIMP, GT 150, TIN, SEALED, 18-16 AWG, CABLE OD 1.70-2.25 MM</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
@@ -9481,14 +9481,14 @@
         <v>4</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0.95</v>
+        <v>0.18</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>3.8</v>
+        <v>0.72</v>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>https://www.customconnectorkits.com/products/12110293?variant=45536279953726</t>
+          <t>https://www.customconnectorkits.com/products/12191819-l?variant=45536512966974</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
@@ -9517,7 +9517,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>13519047</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -9528,11 +9528,11 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>CONTACT, SOCKET, CRIMP, GT 150, TIN, SEALED, 18-16 AWG, CABLE OD 1.70-2.25 MM</t>
+          <t>CONNECTOR, PLUG, GT 150, 3 POS, SEALED, SOCKET CONTACTS</t>
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
@@ -9543,17 +9543,17 @@
         <v>0</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.18</v>
+        <v>0.95</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>0.72</v>
+        <v>0.95</v>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>https://www.customconnectorkits.com/products/12191819-l?variant=45536512966974</t>
+          <t>https://www.customconnectorkits.com/products/13519047?variant=45536514539838</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr"/>
@@ -9582,7 +9582,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>13519047</t>
+          <t>15326426</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -9593,11 +9593,11 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>CONNECTOR, PLUG, GT 150, 3 POS, SEALED, SOCKET CONTACTS</t>
+          <t>CONTACT, SOCKET, CRIMP, GT 150, GOLD, SEALED, 0.35-0.50 MM2 (22-20 AWG), CABLE OD 1.20-1.85 MM</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -9608,17 +9608,17 @@
         <v>0</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0.95</v>
+        <v>0.45</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>0.95</v>
+        <v>3.15</v>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>https://www.customconnectorkits.com/products/13519047?variant=45536514539838</t>
+          <t>https://www.customconnectorkits.com/products/15326426-l?variant=48621504332094</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
@@ -9647,7 +9647,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>15419715</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -9658,11 +9658,11 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>CONTACT, SOCKET, CRIMP, GT 150, GOLD, SEALED, 0.35-0.50 MM2 (22-20 AWG), CABLE OD 1.20-1.85 MM</t>
+          <t>CONNECTOR, PLUG, GT 150, 2 POS, SEALED, GRAY, USCAR / EV6</t>
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
@@ -9673,17 +9673,17 @@
         <v>0</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0.45</v>
+        <v>1.09</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>3.15</v>
+        <v>4.36</v>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>https://www.customconnectorkits.com/products/15326426-l?variant=48621504332094</t>
+          <t>https://www.customconnectorkits.com/products/15419715?variant=45536627917118</t>
         </is>
       </c>
       <c r="N23" s="3" t="inlineStr"/>
@@ -9712,22 +9712,22 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>1N5822</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Aptiv</t>
+          <t>STMicroelectronics</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>CONNECTOR, PLUG, GT 150, 2 POS, SEALED, GRAY, USCAR / EV6</t>
+          <t>DIODE, SCHOTTKY, RECTIFIER, 40 V, 3 A, DO-201AD AXIAL</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -9738,28 +9738,28 @@
         <v>0</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>1.09</v>
+        <v>0.71</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>4.36</v>
+        <v>0.71</v>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>https://www.customconnectorkits.com/products/15419715?variant=45536627917118</t>
+          <t>https://www.digikey.com/en/products/detail/taiwan-semiconductor-corporation/1N5822/7366597</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Custom Connector Kits, 2026-10-20</t>
+          <t>Digi-Key qty 1 (Cut Tape (CT)), 2026-10-20</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Digi-Key API 2026-10-20: 2377 in stock</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
@@ -9777,18 +9777,18 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>1N5822</t>
+          <t>1k 1/4W</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>STMicroelectronics</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>DIODE, SCHOTTKY, RECTIFIER, 40 V, 3 A, DO-201AD AXIAL</t>
+          <t>RESISTOR, FIXED, METAL FILM, 1 KOHM, 5 PCT, 1/4 W</t>
         </is>
       </c>
       <c r="G25" s="3" t="n">
@@ -9806,25 +9806,25 @@
         <v>1</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.71</v>
+        <v>0.1</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.71</v>
+        <v>0.1</v>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/taiwan-semiconductor-corporation/1N5822/7366597</t>
+          <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/CF14JT1K00/1741314</t>
         </is>
       </c>
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Cut Tape (CT)), 2026-10-20</t>
+          <t>Digi-Key qty 1 (Cut Tape (CT)), 2026-10-20; listed as CF14JT1K00</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2377 in stock</t>
+          <t>Digi-Key API 2026-10-20: 615946 in stock</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr"/>
@@ -9842,7 +9842,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1k 1/4W</t>
+          <t>2.2k 1/4W 1%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -9853,7 +9853,7 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>RESISTOR, FIXED, METAL FILM, 1 KOHM, 5 PCT, 1/4 W</t>
+          <t>RESISTOR, FIXED, METAL FILM, 2.2 KOHM, 1 PCT, 1/4 W</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
@@ -9870,26 +9870,14 @@
       <c r="J26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K26" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L26" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/CF14JT1K00/1741314</t>
-        </is>
-      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Cut Tape (CT)), 2026-10-20; listed as CF14JT1K00</t>
-        </is>
-      </c>
+      <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 615946 in stock</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
@@ -9907,22 +9895,22 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1/4W 1%</t>
+          <t>3-1447221-3</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>TE Connectivity</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>RESISTOR, FIXED, METAL FILM, 2.2 KOHM, 1 PCT, 1/4 W</t>
+          <t>CONTACT, SOCKET, CRIMP, SUPERSEAL 1.0, GOLD, 0.75-0.85 MM2 (18 AWG)</t>
         </is>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
@@ -9930,19 +9918,29 @@
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K27" s="3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <v>0.41</v>
+      </c>
       <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/3-1447221-3/2135580</t>
+        </is>
+      </c>
       <c r="N27" s="3" t="inlineStr"/>
-      <c r="O27" s="3" t="inlineStr"/>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 18 (Cut Tape (CT)), 2026-10-20</t>
+        </is>
+      </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>Digi-Key API 2026-10-20: 10959 in stock</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr"/>
@@ -9960,7 +9958,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>3-1447221-3</t>
+          <t>3-1447221-4</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -9971,11 +9969,11 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>CONTACT, SOCKET, CRIMP, SUPERSEAL 1.0, GOLD, 0.75-0.85 MM2 (18 AWG)</t>
+          <t>CONTACT, SOCKET, CRIMP, SUPERSEAL 1.0, GOLD, 0.5 MM2 (20 AWG), INSUL 1.6-2.2 MM</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -9983,29 +9981,29 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0.41</v>
+        <v>0.28</v>
       </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/3-1447221-3/2135580</t>
+          <t>https://www.digikey.com/en/products/detail/wec/3-1447221-4/29355733</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 18 (Cut Tape (CT)), 2026-10-20</t>
+          <t>Digi-Key qty 7000 (Tape &amp; Reel (TR)), 2026-10-20; reel only at Digi-Key (min 7000), unit price is the reel price</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 10959 in stock</t>
+          <t>Digi-Key API 2026-10-20: 10000 in stock</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr"/>
@@ -10023,22 +10021,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>3-1447221-4</t>
+          <t>3.9k 1/4W</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>generic</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>CONTACT, SOCKET, CRIMP, SUPERSEAL 1.0, GOLD, 0.5 MM2 (20 AWG), INSUL 1.6-2.2 MM</t>
+          <t>RESISTOR, FIXED, METAL FILM, 3.9 KOHM, 5 PCT, 1/4 W</t>
         </is>
       </c>
       <c r="G29" s="3" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
@@ -10046,29 +10044,31 @@
         </is>
       </c>
       <c r="I29" s="3" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="L29" s="3" t="inlineStr"/>
+        <v>0.1</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/wec/3-1447221-4/29355733</t>
+          <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/CF14JT3K90/1741386</t>
         </is>
       </c>
       <c r="N29" s="3" t="inlineStr"/>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 7000 (Tape &amp; Reel (TR)), 2026-10-20; reel only at Digi-Key (min 7000), unit price is the reel price</t>
+          <t>Digi-Key qty 1 (Cut Tape (CT)), 2026-10-20; listed as CF14JT3K90</t>
         </is>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 10000 in stock</t>
+          <t>Digi-Key API 2026-10-20: 44589 in stock</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr"/>
@@ -10086,22 +10086,22 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>3.9k 1/4W</t>
+          <t>301A011-25-0</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>TE Connectivity (Raychem)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>RESISTOR, FIXED, METAL FILM, 3.9 KOHM, 5 PCT, 1/4 W</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, T, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 6.6/3.6 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -10112,28 +10112,28 @@
         <v>0</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0.1</v>
+        <v>27.58</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>0.1</v>
+        <v>82.73999999999999</v>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/CF14JT3K90/1741386</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/301A011-25-0/2394181</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Cut Tape (CT)), 2026-10-20; listed as CF14JT3K90</t>
+          <t>Digi-Key qty 3 (Bulk), 2026-10-20</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 44589 in stock</t>
+          <t>Digi-Key API 2026-10-20: 236 in stock</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>301A011-25-0</t>
+          <t>301A022-25-0</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -10162,11 +10162,11 @@
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, T, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 6.6/3.6 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, T, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 13.2/6.9 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
@@ -10177,28 +10177,28 @@
         <v>0</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>27.58</v>
+        <v>40.77</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>82.73999999999999</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/301A011-25-0/2394181</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/301A022-25-0/2394178</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Bulk), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Bulk), 2026-10-20</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 236 in stock</t>
+          <t>Digi-Key API 2026-10-20: 151 in stock</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr"/>
@@ -10216,7 +10216,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>301A022-25-0</t>
+          <t>301A028-25-0</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -10227,7 +10227,7 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, T, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 13.2/6.9 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, T, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 20/10.2 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
@@ -10245,14 +10245,14 @@
         <v>2</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>40.77</v>
+        <v>37.65</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>81.54000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/301A022-25-0/2394178</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/301A028-25-0/3318081</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 151 in stock</t>
+          <t>Digi-Key API 2026-10-20: 94 in stock</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
@@ -10281,7 +10281,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>301A028-25-0</t>
+          <t>342A012-25-0</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -10292,11 +10292,11 @@
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, T, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 20/10.2 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 13.2/6.9 X 6.6/3.6 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
@@ -10307,28 +10307,28 @@
         <v>0</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>37.65</v>
+        <v>35.59</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>75.3</v>
+        <v>427.08</v>
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/301A028-25-0/3318081</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A012-25-0/2394240</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Bulk), 2026-10-20</t>
+          <t>Digi-Key qty 12 (Bulk), 2026-10-20</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 94 in stock</t>
+          <t>Digi-Key API 2026-10-20: not stocked at Digi-Key now</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr"/>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>342A012-25-0</t>
+          <t>342A024-25-0</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -10357,11 +10357,11 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 13.2/6.9 X 6.6/3.6 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 26.9/12.7 X 6.6/3.6 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -10372,28 +10372,28 @@
         <v>0</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>35.59</v>
+        <v>50.66</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>427.08</v>
+        <v>557.26</v>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A012-25-0/2394240</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A024-25-0/2394208</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 12 (Bulk), 2026-10-20</t>
+          <t>Digi-Key qty 11 (Bulk), 2026-10-20</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: not stocked at Digi-Key now</t>
+          <t>Digi-Key API 2026-10-20: 140 in stock</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr"/>
@@ -10411,7 +10411,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>342A024-25-0</t>
+          <t>342A034-25-0</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -10422,11 +10422,11 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 26.9/12.7 X 6.6/3.6 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 26.9/13.7 X 13.2/6.1 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
@@ -10437,28 +10437,28 @@
         <v>0</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>50.66</v>
+        <v>75.67</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>557.26</v>
+        <v>605.36</v>
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A024-25-0/2394208</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A034-25-0/2394180</t>
         </is>
       </c>
       <c r="N35" s="3" t="inlineStr"/>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 11 (Bulk), 2026-10-20</t>
+          <t>Digi-Key qty 8 (Bulk), 2026-10-20</t>
         </is>
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 140 in stock</t>
+          <t>Digi-Key API 2026-10-20: 57 in stock</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr"/>
@@ -10476,7 +10476,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>342A034-25-0</t>
+          <t>342A048-25-0</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -10487,11 +10487,11 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 26.9/13.7 X 13.2/6.1 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 55.6/26.9 X 13.2/6.9 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -10502,28 +10502,28 @@
         <v>0</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>75.67</v>
+        <v>117.77</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>605.36</v>
+        <v>235.54</v>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A034-25-0/2394180</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A048-25-0/2394190</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 8 (Bulk), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Bulk), 2026-10-20</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 57 in stock</t>
+          <t>Digi-Key API 2026-10-20: 46 in stock</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
@@ -10541,22 +10541,22 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>342A048-25-0</t>
+          <t>354404</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
+          <t>Lowdoller Motorsports</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>TRANSITION, MOULDED, HEAT SHRINK, 45 DEG BREAKOUT, 3 BRANCHES, -25 FLUID RESISTANT ELASTOMER, BLACK, 55.6/26.9 X 13.2/6.9 MM SUPPLIED / RECOVERED, -75 TO 150 C</t>
+          <t>CONNECTOR KIT, PRESSURE / MAP SENSOR, 3 PIN, DELPHI GT150 (PLUG, PINS, SEALS)</t>
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
@@ -10567,28 +10567,20 @@
         <v>0</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K37" s="3" t="n">
-        <v>117.77</v>
-      </c>
-      <c r="L37" s="3" t="n">
-        <v>235.54</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr"/>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-aerospace-defense-and-marine/342A048-25-0/2394190</t>
+          <t>https://lowdoller-motorsports.com/products/3-pin-connector-pins-and-grommets-for-pressure-sensor</t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr"/>
-      <c r="O37" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 2 (Bulk), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O37" s="3" t="inlineStr"/>
       <c r="P37" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 46 in stock</t>
+          <t>maker page read 2026-10-25 (one ships with each Lowdoller sensor)</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr"/>
@@ -16067,11 +16059,11 @@
       <c r="E124" s="2" t="inlineStr"/>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-1) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (CLNT-P) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16082,7 +16074,7 @@
         <v>0</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K124" s="2" t="inlineStr"/>
       <c r="L124" s="2" t="inlineStr"/>
@@ -16120,7 +16112,7 @@
       <c r="E125" s="3" t="inlineStr"/>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (COIL-1) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G125" s="3" t="n">
@@ -16173,7 +16165,7 @@
       <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (COIL-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G126" s="2" t="n">
@@ -16226,7 +16218,7 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-4) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (COIL-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G127" s="3" t="n">
@@ -16279,11 +16271,11 @@
       <c r="E128" s="2" t="inlineStr"/>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (COIL-4) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -16294,7 +16286,7 @@
         <v>0</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K128" s="2" t="inlineStr"/>
       <c r="L128" s="2" t="inlineStr"/>
@@ -16332,11 +16324,11 @@
       <c r="E129" s="3" t="inlineStr"/>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ETB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G129" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
@@ -16347,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="J129" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K129" s="3" t="inlineStr"/>
       <c r="L129" s="3" t="inlineStr"/>
@@ -16385,11 +16377,11 @@
       <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ETB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -16400,7 +16392,7 @@
         <v>0</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K130" s="2" t="inlineStr"/>
       <c r="L130" s="2" t="inlineStr"/>
@@ -16438,11 +16430,11 @@
       <c r="E131" s="3" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G131" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
@@ -16453,7 +16445,7 @@
         <v>0</v>
       </c>
       <c r="J131" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K131" s="3" t="inlineStr"/>
       <c r="L131" s="3" t="inlineStr"/>
@@ -16491,11 +16483,11 @@
       <c r="E132" s="2" t="inlineStr"/>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -16506,7 +16498,7 @@
         <v>0</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K132" s="2" t="inlineStr"/>
       <c r="L132" s="2" t="inlineStr"/>
@@ -16544,11 +16536,11 @@
       <c r="E133" s="3" t="inlineStr"/>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KNOCK-1) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G133" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
@@ -16559,7 +16551,7 @@
         <v>0</v>
       </c>
       <c r="J133" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K133" s="3" t="inlineStr"/>
       <c r="L133" s="3" t="inlineStr"/>
@@ -16597,7 +16589,7 @@
       <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-A) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KNOCK-1) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G134" s="2" t="n">
@@ -16650,11 +16642,11 @@
       <c r="E135" s="3" t="inlineStr"/>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-A) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G135" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
@@ -16665,7 +16657,7 @@
         <v>0</v>
       </c>
       <c r="J135" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K135" s="3" t="inlineStr"/>
       <c r="L135" s="3" t="inlineStr"/>
@@ -16703,11 +16695,11 @@
       <c r="E136" s="2" t="inlineStr"/>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -16718,7 +16710,7 @@
         <v>0</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K136" s="2" t="inlineStr"/>
       <c r="L136" s="2" t="inlineStr"/>
@@ -16756,11 +16748,11 @@
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G137" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
@@ -16771,7 +16763,7 @@
         <v>0</v>
       </c>
       <c r="J137" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K137" s="3" t="inlineStr"/>
       <c r="L137" s="3" t="inlineStr"/>
@@ -16809,7 +16801,7 @@
       <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G138" s="2" t="n">
@@ -16862,7 +16854,7 @@
       <c r="E139" s="3" t="inlineStr"/>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G139" s="3" t="n">
@@ -16915,7 +16907,7 @@
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G140" s="2" t="n">
@@ -16968,7 +16960,7 @@
       <c r="E141" s="3" t="inlineStr"/>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G141" s="3" t="n">
@@ -17021,7 +17013,7 @@
       <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G142" s="2" t="n">
@@ -17074,7 +17066,7 @@
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G143" s="3" t="n">
@@ -17127,7 +17119,7 @@
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (CAM) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G144" s="2" t="n">
@@ -17180,7 +17172,7 @@
       <c r="E145" s="3" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (CAM) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G145" s="3" t="n">
@@ -17233,7 +17225,7 @@
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (CLNT-P) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G146" s="2" t="n">
@@ -17286,7 +17278,7 @@
       <c r="E147" s="3" t="inlineStr"/>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G147" s="3" t="n">
@@ -17339,7 +17331,7 @@
       <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G148" s="2" t="n">
@@ -17392,7 +17384,7 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (ENG-GND-RING) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G149" s="3" t="n">
@@ -17445,11 +17437,11 @@
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -17460,7 +17452,7 @@
         <v>0</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
@@ -17498,11 +17490,11 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (ENG-GND-RING) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G151" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
@@ -17513,7 +17505,7 @@
         <v>0</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K151" s="3" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr"/>
@@ -17551,11 +17543,11 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -17566,7 +17558,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
@@ -17604,11 +17596,11 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G153" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
@@ -17619,7 +17611,7 @@
         <v>0</v>
       </c>
       <c r="J153" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K153" s="3" t="inlineStr"/>
       <c r="L153" s="3" t="inlineStr"/>
@@ -17657,11 +17649,11 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (STARTER-TRIGGER) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -17672,7 +17664,7 @@
         <v>0</v>
       </c>
       <c r="J154" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr"/>
@@ -17710,7 +17702,7 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AC-BTN) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G155" s="3" t="n">
@@ -17763,7 +17755,7 @@
       <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (STARTER-TRIGGER) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G156" s="2" t="n">
@@ -17816,11 +17808,11 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AC-BTN) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G157" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
@@ -17831,7 +17823,7 @@
         <v>0</v>
       </c>
       <c r="J157" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K157" s="3" t="inlineStr"/>
       <c r="L157" s="3" t="inlineStr"/>
@@ -17869,11 +17861,11 @@
       <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -17884,7 +17876,7 @@
         <v>0</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr"/>
@@ -17922,11 +17914,11 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G159" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H159" s="3" t="inlineStr">
         <is>
@@ -17937,7 +17929,7 @@
         <v>0</v>
       </c>
       <c r="J159" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K159" s="3" t="inlineStr"/>
       <c r="L159" s="3" t="inlineStr"/>
@@ -17975,11 +17967,11 @@
       <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -17990,7 +17982,7 @@
         <v>0</v>
       </c>
       <c r="J160" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K160" s="2" t="inlineStr"/>
       <c r="L160" s="2" t="inlineStr"/>
@@ -18028,7 +18020,7 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -18081,7 +18073,7 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G162" s="2" t="n">
@@ -18134,7 +18126,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-EVAP-RTN) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G163" s="3" t="n">
@@ -18187,7 +18179,7 @@
       <c r="E164" s="2" t="inlineStr"/>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-EVAP-TEMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G164" s="2" t="n">
@@ -18240,7 +18232,7 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-RL-GND-BL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-EVAP-RTN) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
@@ -18293,7 +18285,7 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-EVAP-TEMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G166" s="2" t="n">
@@ -18346,7 +18338,7 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-RL-GND-BL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G167" s="3" t="n">
@@ -18399,7 +18391,7 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
@@ -18452,7 +18444,7 @@
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G169" s="3" t="n">
@@ -18505,7 +18497,7 @@
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G170" s="2" t="n">
@@ -18558,22 +18550,22 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>shielded cable, part number not confirmed: CAB-CAN-CLU, CAB-CAN-CSB, CAB-CAN-ECU, CAB-CAN-RD, CAB-CANBH-BC, CAB-ETBM-AE, CAB-LAMCAN-BE</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>ft</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I171" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K171" s="3" t="inlineStr"/>
       <c r="L171" s="3" t="inlineStr"/>
@@ -18587,7 +18579,7 @@
       </c>
       <c r="Q171" s="3" t="inlineStr">
         <is>
-          <t>OPEN-ITEMS row 140</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -18604,22 +18596,18 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
-        </is>
-      </c>
-      <c r="D172" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr"/>
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18630,27 +18618,23 @@
         <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L172" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K172" s="2" t="inlineStr"/>
+      <c r="L172" s="2" t="inlineStr"/>
       <c r="M172" s="2" t="inlineStr"/>
       <c r="N172" s="2" t="inlineStr"/>
-      <c r="O172" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O172" s="2" t="inlineStr"/>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
-        </is>
-      </c>
-      <c r="Q172" s="2" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q172" s="2" t="inlineStr">
+        <is>
+          <t>no maker document in the repo yet; never guessed</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -18665,53 +18649,45 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
-        </is>
-      </c>
-      <c r="D173" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr"/>
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>shielded cable, part number not confirmed: CAB-CAN-CLU, CAB-CAN-CSB, CAB-CAN-ECU, CAB-CAN-RD, CAB-CANBH-BC, CAB-ETBM-AE, CAB-LAMCAN-BE</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>ft</t>
         </is>
       </c>
       <c r="I173" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J173" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="K173" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L173" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K173" s="3" t="inlineStr"/>
+      <c r="L173" s="3" t="inlineStr"/>
       <c r="M173" s="3" t="inlineStr"/>
       <c r="N173" s="3" t="inlineStr"/>
-      <c r="O173" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O173" s="3" t="inlineStr"/>
       <c r="P173" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
-        </is>
-      </c>
-      <c r="Q173" s="3" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q173" s="3" t="inlineStr">
+        <is>
+          <t>OPEN-ITEMS row 140</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -18726,7 +18702,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>TMS-SCE-1/2-2.0-9</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -18737,11 +18713,11 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -18752,7 +18728,7 @@
         <v>0</v>
       </c>
       <c r="J174" s="2" t="n">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="K174" s="2" t="n">
         <v>0</v>
@@ -18787,22 +18763,22 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>TMS-SCE-3/16-2.0-9</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
+          <t>TE Connectivity (Raychem)</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
@@ -18810,31 +18786,27 @@
         </is>
       </c>
       <c r="I175" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J175" s="3" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="K175" s="3" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L175" s="3" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="M175" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M175" s="3" t="inlineStr"/>
       <c r="N175" s="3" t="inlineStr"/>
       <c r="O175" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>not priced (Dan)</t>
         </is>
       </c>
       <c r="P175" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="Q175" s="3" t="inlineStr"/>
@@ -18852,26 +18824,22 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>TMS-SCE-3/8-2.0-9</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E176" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -18882,28 +18850,24 @@
         <v>0</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="K176" s="2" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="L176" s="2" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="M176" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M176" s="2" t="inlineStr"/>
       <c r="N176" s="2" t="inlineStr"/>
       <c r="O176" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>not priced (Dan)</t>
         </is>
       </c>
       <c r="P176" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="Q176" s="2" t="inlineStr"/>
@@ -18921,26 +18885,22 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>W12S</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E177" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
+          <t>Deutsch (TE Connectivity)</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
@@ -18948,31 +18908,31 @@
         </is>
       </c>
       <c r="I177" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J177" s="3" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K177" s="3" t="n">
-        <v>0.13</v>
+        <v>0.42</v>
       </c>
       <c r="L177" s="3" t="n">
-        <v>1.43</v>
+        <v>1.26</v>
       </c>
       <c r="M177" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
         </is>
       </c>
       <c r="N177" s="3" t="inlineStr"/>
       <c r="O177" s="3" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P177" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
         </is>
       </c>
       <c r="Q177" s="3" t="inlineStr"/>
@@ -18990,12 +18950,12 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>W2P</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -19005,7 +18965,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
@@ -19030,18 +18990,18 @@
       </c>
       <c r="M178" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="N178" s="2" t="inlineStr"/>
       <c r="O178" s="2" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1, 2026-10-19</t>
         </is>
       </c>
       <c r="P178" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q178" s="2" t="inlineStr"/>
@@ -19059,7 +19019,7 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>W2S</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -19074,11 +19034,11 @@
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
@@ -19089,28 +19049,28 @@
         <v>0</v>
       </c>
       <c r="J179" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="K179" s="3" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="L179" s="3" t="n">
-        <v>0.4</v>
+        <v>1.43</v>
       </c>
       <c r="M179" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+          <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="N179" s="3" t="inlineStr"/>
       <c r="O179" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P179" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q179" s="3" t="inlineStr"/>
@@ -19128,12 +19088,12 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
+          <t>Deutsch</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -19143,7 +19103,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19161,25 +19121,25 @@
         <v>2</v>
       </c>
       <c r="K180" s="2" t="n">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="L180" s="2" t="n">
-        <v>0.42</v>
+        <v>0.26</v>
       </c>
       <c r="M180" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
+          <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="N180" s="2" t="inlineStr"/>
       <c r="O180" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P180" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q180" s="2" t="inlineStr"/>
@@ -19197,7 +19157,7 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -19212,11 +19172,11 @@
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G181" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
@@ -19227,28 +19187,28 @@
         <v>0</v>
       </c>
       <c r="J181" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K181" s="3" t="n">
-        <v>0.35</v>
+        <v>0.2</v>
       </c>
       <c r="L181" s="3" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="M181" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
         </is>
       </c>
       <c r="N181" s="3" t="inlineStr"/>
       <c r="O181" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P181" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q181" s="3" t="inlineStr"/>
@@ -19266,7 +19226,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>WM-4S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -19281,11 +19241,11 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -19296,28 +19256,28 @@
         <v>0</v>
       </c>
       <c r="J182" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K182" s="2" t="n">
-        <v>0.28</v>
+        <v>0.21</v>
       </c>
       <c r="L182" s="2" t="n">
-        <v>0.28</v>
+        <v>0.42</v>
       </c>
       <c r="M182" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N182" s="2" t="inlineStr"/>
       <c r="O182" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q182" s="2" t="inlineStr"/>
@@ -19335,12 +19295,12 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>WM-6S</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E183" s="3" t="inlineStr">
@@ -19350,7 +19310,7 @@
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
@@ -19368,14 +19328,14 @@
         <v>1</v>
       </c>
       <c r="K183" s="3" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="L183" s="3" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="M183" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N183" s="3" t="inlineStr"/>
@@ -19386,13 +19346,196 @@
       </c>
       <c r="P183" s="3" t="inlineStr">
         <is>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
+        </is>
+      </c>
+      <c r="Q183" s="3" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>All harnesses (master wire list)</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>WM-4S</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K184" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L184" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="M184" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="inlineStr"/>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+        </is>
+      </c>
+      <c r="P184" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+        </is>
+      </c>
+      <c r="Q184" s="2" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>All harnesses (master wire list)</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>WM-6S</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J185" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K185" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="L185" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="M185" s="5" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+        </is>
+      </c>
+      <c r="N185" s="3" t="inlineStr"/>
+      <c r="O185" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+        </is>
+      </c>
+      <c r="P185" s="3" t="inlineStr">
+        <is>
           <t>Digi-Key API 2026-10-20: 2478 in stock</t>
         </is>
       </c>
-      <c r="Q183" s="3" t="inlineStr"/>
+      <c r="Q185" s="3" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>All harnesses (master wire list)</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>in kit 354404</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr"/>
+      <c r="E186" s="2" t="inlineStr"/>
+      <c r="F186" s="2" t="inlineStr"/>
+      <c r="G186" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J186" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr"/>
+      <c r="M186" s="2" t="inlineStr"/>
+      <c r="N186" s="2" t="inlineStr"/>
+      <c r="O186" s="2" t="inlineStr"/>
+      <c r="P186" s="2" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q183"/>
+  <autoFilter ref="A1:Q186"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -19418,7 +19561,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId28"/>
@@ -19488,15 +19631,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -19509,7 +19652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -19878,12 +20021,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>52-45780</t>
+          <t>354404</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>maker page read 2026-10-25 (one ships with each Lowdoller sensor)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -19900,12 +20043,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>55A1811-20-9-9CS2275</t>
+          <t>52-45780</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -19922,7 +20065,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>55A1821-20-6/9-9</t>
+          <t>55A1811-20-9-9CS2275</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -19944,7 +20087,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>55A1831-20-2/4/6-9</t>
+          <t>55A1821-20-6/9-9</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -19966,7 +20109,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>55A1841-20-2/4/5/6-9</t>
+          <t>55A1831-20-2/4/6-9</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -19988,17 +20131,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>90980-10341</t>
+          <t>55A1841-20-2/4/5/6-9</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -20010,7 +20153,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>90980-10942</t>
+          <t>90980-10341</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -20032,7 +20175,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>90980-11143</t>
+          <t>90980-10942</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -20054,7 +20197,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>90980-11250</t>
+          <t>90980-11143</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -20076,7 +20219,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>90980-11885</t>
+          <t>90980-11250</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -20098,7 +20241,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>90980-12068</t>
+          <t>90980-11885</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -20120,7 +20263,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>BC-1/0-BLK</t>
+          <t>90980-12068</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -20130,7 +20273,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
+          <t>OEM Toyota part: buy from a Toyota parts dealer; confirm it is not already on the car</t>
         </is>
       </c>
     </row>
@@ -20142,7 +20285,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>BC-1/0-RED</t>
+          <t>BC-1/0-BLK</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -20164,7 +20307,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>BC-2-RED</t>
+          <t>BC-1/0-RED</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -20186,7 +20329,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>BC-4-BLK</t>
+          <t>BC-2-RED</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -20208,17 +20351,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>DR-25-1-1/2-0-SP</t>
+          <t>BC-4-BLK</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>pick a welding / battery cable supplier (no PN exists for this drawn wire); recommend ProWire USA</t>
         </is>
       </c>
     </row>
@@ -20230,7 +20373,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>HD36-24-33SE</t>
+          <t>DR-25-1-1/2-0-SP</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -20252,12 +20395,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>LP-16-J05PE-02-001</t>
+          <t>HD36-24-33SE</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -20274,7 +20417,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-10-9</t>
+          <t>LP-16-J05PE-02-001</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -20284,7 +20427,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
+          <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
@@ -20296,7 +20439,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-14-4</t>
+          <t>M22759/16-10-9</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -20318,7 +20461,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-16-4</t>
+          <t>M22759/16-14-4</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -20340,7 +20483,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>M22759/16-18-4</t>
+          <t>M22759/16-16-4</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -20362,7 +20505,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>M22759/16-6-2</t>
+          <t>M22759/16-18-4</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -20384,7 +20527,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>M22759/16-6-2</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -20394,7 +20537,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>I find and validate a maker page or approved-supplier listing</t>
+          <t>buy by the foot (Wings and Wheels / Flight Store); confirm the supplier and the colour code page</t>
         </is>
       </c>
     </row>
@@ -21498,8 +21641,96 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>in kit 354404</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D90"/>
+  <autoFilter ref="A1:D94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Stop treating C11 as an ECU input; keep C17 as the one clutch tap
C11 only completes the starter circuit in hardware. Remove the C11-to-Aux-8
wire, leave Aux 8 spare, and record the factory trinary A/C switch and unused
brake-fluid switch in the existing wiring docs. Drawings Rev E and the BOM
follow the master.

Co-authored-by: living-relation <living-relation@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>84</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4637.41</v>
+        <v>4635.81</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -571,7 +571,7 @@
         <v>175</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5075.27</v>
+        <v>5073.67</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>24</v>
@@ -9806,7 +9806,7 @@
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
@@ -9814,7 +9814,7 @@
         </is>
       </c>
       <c r="I25" s="3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>0</v>
@@ -14612,7 +14612,7 @@
         </is>
       </c>
       <c r="G101" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -14623,13 +14623,13 @@
         <v>0</v>
       </c>
       <c r="J101" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K101" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="L101" s="3" t="n">
-        <v>40</v>
+        <v>38.4</v>
       </c>
       <c r="M101" s="5" t="inlineStr">
         <is>
@@ -14649,7 +14649,7 @@
       </c>
       <c r="Q101" s="3" t="inlineStr">
         <is>
-          <t>6.6 m in the master + 15% margin</t>
+          <t>6.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="Q116" s="2" t="inlineStr">
         <is>
-          <t>562 bands of 6 mm, both ends of each wire</t>
+          <t>560 bands of 6 mm, both ends of each wire</t>
         </is>
       </c>
     </row>
@@ -15782,7 +15782,7 @@
       </c>
       <c r="Q118" s="2" t="inlineStr">
         <is>
-          <t>402 bands of 6 mm, both ends of each wire</t>
+          <t>400 bands of 6 mm, both ends of each wire</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Per-harness From/To wire lists for AB-cabin and AB-engine (Rev H)
- build_drawings.py writes docs/harness/wirelists/ST185-<harness>-wirelist.xlsx from the master
  (Wires / Connectors / Splices / Spare Cavities / Key; harness.design Excel-import column names);
  --check fails when one is stale. Layout file lists which harnesses get one.
- Master: spare rows for ECU A26 (Aux 8), B31 / B32 (An Volt 10 / 11); IO table detail rows and pin
  budget now show them spare; BOM regenerated.
- B27: fuse boxes follow the harnesses (Dan). Fuse-box CAD input note points at Route 17.
- README: wirelists folder; AB-cabin drawn left to right without a route (Dan).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$116</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$181</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,10 +540,10 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>84</v>
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>175</v>
@@ -8162,7 +8162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q181"/>
+  <dimension ref="A1:Q182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16230,11 +16230,11 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-A) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G127" s="3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H127" s="3" t="inlineStr">
         <is>
@@ -16245,7 +16245,7 @@
         <v>0</v>
       </c>
       <c r="J127" s="3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K127" s="3" t="inlineStr"/>
       <c r="L127" s="3" t="inlineStr"/>
@@ -16283,11 +16283,11 @@
       <c r="E128" s="2" t="inlineStr"/>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ETB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -16298,7 +16298,7 @@
         <v>0</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K128" s="2" t="inlineStr"/>
       <c r="L128" s="2" t="inlineStr"/>
@@ -16336,11 +16336,11 @@
       <c r="E129" s="3" t="inlineStr"/>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ETB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G129" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
@@ -16351,7 +16351,7 @@
         <v>0</v>
       </c>
       <c r="J129" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K129" s="3" t="inlineStr"/>
       <c r="L129" s="3" t="inlineStr"/>
@@ -16389,11 +16389,11 @@
       <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -16404,7 +16404,7 @@
         <v>0</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K130" s="2" t="inlineStr"/>
       <c r="L130" s="2" t="inlineStr"/>
@@ -16442,11 +16442,11 @@
       <c r="E131" s="3" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G131" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
@@ -16457,7 +16457,7 @@
         <v>0</v>
       </c>
       <c r="J131" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K131" s="3" t="inlineStr"/>
       <c r="L131" s="3" t="inlineStr"/>
@@ -16495,11 +16495,11 @@
       <c r="E132" s="2" t="inlineStr"/>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KNOCK-1) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -16510,7 +16510,7 @@
         <v>0</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K132" s="2" t="inlineStr"/>
       <c r="L132" s="2" t="inlineStr"/>
@@ -16548,7 +16548,7 @@
       <c r="E133" s="3" t="inlineStr"/>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-A) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KNOCK-1) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G133" s="3" t="n">
@@ -16601,11 +16601,11 @@
       <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-A) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -16616,7 +16616,7 @@
         <v>0</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K134" s="2" t="inlineStr"/>
       <c r="L134" s="2" t="inlineStr"/>
@@ -16654,11 +16654,11 @@
       <c r="E135" s="3" t="inlineStr"/>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G135" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
@@ -16669,7 +16669,7 @@
         <v>0</v>
       </c>
       <c r="J135" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K135" s="3" t="inlineStr"/>
       <c r="L135" s="3" t="inlineStr"/>
@@ -16707,11 +16707,11 @@
       <c r="E136" s="2" t="inlineStr"/>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -16722,7 +16722,7 @@
         <v>0</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K136" s="2" t="inlineStr"/>
       <c r="L136" s="2" t="inlineStr"/>
@@ -16760,7 +16760,7 @@
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G137" s="3" t="n">
@@ -16813,7 +16813,7 @@
       <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G138" s="2" t="n">
@@ -16866,7 +16866,7 @@
       <c r="E139" s="3" t="inlineStr"/>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G139" s="3" t="n">
@@ -16919,7 +16919,7 @@
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G140" s="2" t="n">
@@ -16972,7 +16972,7 @@
       <c r="E141" s="3" t="inlineStr"/>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G141" s="3" t="n">
@@ -17025,7 +17025,7 @@
       <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G142" s="2" t="n">
@@ -17078,7 +17078,7 @@
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (CAM) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G143" s="3" t="n">
@@ -17131,7 +17131,7 @@
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (CLNT-P) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (CAM) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G144" s="2" t="n">
@@ -17184,7 +17184,7 @@
       <c r="E145" s="3" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (CLNT-P) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G145" s="3" t="n">
@@ -17237,7 +17237,7 @@
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G146" s="2" t="n">
@@ -17290,7 +17290,7 @@
       <c r="E147" s="3" t="inlineStr"/>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G147" s="3" t="n">
@@ -17343,7 +17343,7 @@
       <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G148" s="2" t="n">
@@ -17396,7 +17396,7 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (ENG-GND-RING) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G149" s="3" t="n">
@@ -17449,11 +17449,11 @@
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (ENG-GND-RING) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -17464,7 +17464,7 @@
         <v>0</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
@@ -17502,11 +17502,11 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G151" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
@@ -17517,7 +17517,7 @@
         <v>0</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K151" s="3" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr"/>
@@ -17555,11 +17555,11 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -17570,7 +17570,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
@@ -17608,11 +17608,11 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G153" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
@@ -17623,7 +17623,7 @@
         <v>0</v>
       </c>
       <c r="J153" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K153" s="3" t="inlineStr"/>
       <c r="L153" s="3" t="inlineStr"/>
@@ -17661,7 +17661,7 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (STARTER-TRIGGER) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G154" s="2" t="n">
@@ -17714,7 +17714,7 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (STARTER-TRIGGER) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G155" s="3" t="n">
@@ -17767,11 +17767,11 @@
       <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -17782,7 +17782,7 @@
         <v>0</v>
       </c>
       <c r="J156" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr"/>
@@ -17820,7 +17820,7 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G157" s="3" t="n">
@@ -17873,11 +17873,11 @@
       <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -17888,7 +17888,7 @@
         <v>0</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr"/>
@@ -17926,7 +17926,7 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G159" s="3" t="n">
@@ -17979,7 +17979,7 @@
       <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G160" s="2" t="n">
@@ -18032,7 +18032,7 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -18085,7 +18085,7 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G162" s="2" t="n">
@@ -18138,7 +18138,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G163" s="3" t="n">
@@ -18191,7 +18191,7 @@
       <c r="E164" s="2" t="inlineStr"/>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G164" s="2" t="n">
@@ -18244,7 +18244,7 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
@@ -18297,7 +18297,7 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G166" s="2" t="n">
@@ -18350,7 +18350,7 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G167" s="3" t="n">
@@ -18403,22 +18403,22 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>shielded cable, part number not confirmed: CAB-CAN-CLU, CAB-CAN-CSB, CAB-CAN-ECU, CAB-CAN-RD, CAB-CANBH-BC, CAB-ETBM-AE, CAB-LAMCAN-BE</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>ft</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I168" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J168" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K168" s="2" t="inlineStr"/>
       <c r="L168" s="2" t="inlineStr"/>
@@ -18432,7 +18432,7 @@
       </c>
       <c r="Q168" s="2" t="inlineStr">
         <is>
-          <t>OPEN-ITEMS row 140</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -18449,53 +18449,45 @@
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
-        </is>
-      </c>
-      <c r="D169" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr"/>
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>shielded cable, part number not confirmed: CAB-CAN-CLU, CAB-CAN-CSB, CAB-CAN-ECU, CAB-CAN-RD, CAB-CANBH-BC, CAB-ETBM-AE, CAB-LAMCAN-BE</t>
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>ft</t>
         </is>
       </c>
       <c r="I169" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="K169" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L169" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K169" s="3" t="inlineStr"/>
+      <c r="L169" s="3" t="inlineStr"/>
       <c r="M169" s="3" t="inlineStr"/>
       <c r="N169" s="3" t="inlineStr"/>
-      <c r="O169" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O169" s="3" t="inlineStr"/>
       <c r="P169" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
-        </is>
-      </c>
-      <c r="Q169" s="3" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q169" s="3" t="inlineStr">
+        <is>
+          <t>OPEN-ITEMS row 140</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -18510,7 +18502,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>TMS-SCE-1/2-2.0-9</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -18521,11 +18513,11 @@
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -18536,7 +18528,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="K170" s="2" t="n">
         <v>0</v>
@@ -18571,7 +18563,7 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>TMS-SCE-3/16-2.0-9</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -18582,11 +18574,11 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
@@ -18597,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="K171" s="3" t="n">
         <v>0</v>
@@ -18632,22 +18624,22 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>TMS-SCE-3/8-2.0-9</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
+          <t>TE Connectivity (Raychem)</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18655,31 +18647,27 @@
         </is>
       </c>
       <c r="I172" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="K172" s="2" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L172" s="2" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="M172" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M172" s="2" t="inlineStr"/>
       <c r="N172" s="2" t="inlineStr"/>
       <c r="O172" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>not priced (Dan)</t>
         </is>
       </c>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="Q172" s="2" t="inlineStr"/>
@@ -18697,58 +18685,54 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>W12S</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
+          <t>Deutsch (TE Connectivity)</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H173" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I173" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="J173" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K173" s="3" t="n">
-        <v>0.13</v>
+        <v>0.42</v>
       </c>
       <c r="L173" s="3" t="n">
-        <v>0.26</v>
+        <v>1.26</v>
       </c>
       <c r="M173" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
         </is>
       </c>
       <c r="N173" s="3" t="inlineStr"/>
       <c r="O173" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P173" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
         </is>
       </c>
       <c r="Q173" s="3" t="inlineStr"/>
@@ -18766,7 +18750,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>W2P</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -18781,11 +18765,11 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -18796,28 +18780,28 @@
         <v>0</v>
       </c>
       <c r="J174" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K174" s="2" t="n">
         <v>0.13</v>
       </c>
       <c r="L174" s="2" t="n">
-        <v>1.43</v>
+        <v>0.26</v>
       </c>
       <c r="M174" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="N174" s="2" t="inlineStr"/>
       <c r="O174" s="2" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1, 2026-10-19</t>
         </is>
       </c>
       <c r="P174" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q174" s="2" t="inlineStr"/>
@@ -18835,12 +18819,12 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>W2S</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr">
@@ -18850,11 +18834,11 @@
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
@@ -18865,17 +18849,17 @@
         <v>0</v>
       </c>
       <c r="J175" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="K175" s="3" t="n">
         <v>0.13</v>
       </c>
       <c r="L175" s="3" t="n">
-        <v>0.26</v>
+        <v>1.43</v>
       </c>
       <c r="M175" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
+          <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="N175" s="3" t="inlineStr"/>
@@ -18886,7 +18870,7 @@
       </c>
       <c r="P175" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q175" s="3" t="inlineStr"/>
@@ -18904,12 +18888,12 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
+          <t>Deutsch</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
@@ -18919,7 +18903,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
@@ -18937,25 +18921,25 @@
         <v>2</v>
       </c>
       <c r="K176" s="2" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="L176" s="2" t="n">
-        <v>0.4</v>
+        <v>0.26</v>
       </c>
       <c r="M176" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+          <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="N176" s="2" t="inlineStr"/>
       <c r="O176" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P176" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q176" s="2" t="inlineStr"/>
@@ -18973,7 +18957,7 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -18988,7 +18972,7 @@
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
@@ -19006,14 +18990,14 @@
         <v>2</v>
       </c>
       <c r="K177" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="L177" s="3" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="M177" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
         </is>
       </c>
       <c r="N177" s="3" t="inlineStr"/>
@@ -19024,7 +19008,7 @@
       </c>
       <c r="P177" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q177" s="3" t="inlineStr"/>
@@ -19042,7 +19026,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -19057,11 +19041,11 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -19072,28 +19056,28 @@
         <v>0</v>
       </c>
       <c r="J178" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K178" s="2" t="n">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="L178" s="2" t="n">
-        <v>0.35</v>
+        <v>0.42</v>
       </c>
       <c r="M178" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N178" s="2" t="inlineStr"/>
       <c r="O178" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P178" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q178" s="2" t="inlineStr"/>
@@ -19111,7 +19095,7 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>WM-4S</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -19126,7 +19110,7 @@
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
@@ -19144,14 +19128,14 @@
         <v>1</v>
       </c>
       <c r="K179" s="3" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="L179" s="3" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="M179" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N179" s="3" t="inlineStr"/>
@@ -19162,7 +19146,7 @@
       </c>
       <c r="P179" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
         </is>
       </c>
       <c r="Q179" s="3" t="inlineStr"/>
@@ -19180,12 +19164,12 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>WM-6S</t>
+          <t>WM-4S</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -19195,7 +19179,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19213,14 +19197,14 @@
         <v>1</v>
       </c>
       <c r="K180" s="2" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="L180" s="2" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="M180" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
         </is>
       </c>
       <c r="N180" s="2" t="inlineStr"/>
@@ -19231,7 +19215,7 @@
       </c>
       <c r="P180" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
         </is>
       </c>
       <c r="Q180" s="2" t="inlineStr"/>
@@ -19249,44 +19233,113 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
+          <t>WM-6S</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+        </is>
+      </c>
+      <c r="G181" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J181" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K181" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="L181" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="M181" s="5" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+        </is>
+      </c>
+      <c r="N181" s="3" t="inlineStr"/>
+      <c r="O181" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+        </is>
+      </c>
+      <c r="P181" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
+        </is>
+      </c>
+      <c r="Q181" s="3" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>All harnesses (master wire list)</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
           <t>in kit 354404</t>
         </is>
       </c>
-      <c r="D181" s="3" t="inlineStr"/>
-      <c r="E181" s="3" t="inlineStr"/>
-      <c r="F181" s="3" t="inlineStr"/>
-      <c r="G181" s="3" t="n">
+      <c r="D182" s="2" t="inlineStr"/>
+      <c r="E182" s="2" t="inlineStr"/>
+      <c r="F182" s="2" t="inlineStr"/>
+      <c r="G182" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H181" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I181" s="3" t="n">
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J181" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K181" s="3" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr"/>
-      <c r="M181" s="3" t="inlineStr"/>
-      <c r="N181" s="3" t="inlineStr"/>
-      <c r="O181" s="3" t="inlineStr"/>
-      <c r="P181" s="3" t="inlineStr">
+      <c r="J182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="2" t="inlineStr"/>
+      <c r="M182" s="2" t="inlineStr"/>
+      <c r="N182" s="2" t="inlineStr"/>
+      <c r="O182" s="2" t="inlineStr"/>
+      <c r="P182" s="2" t="inlineStr">
         <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q181" s="3" t="inlineStr">
+      <c r="Q182" s="2" t="inlineStr">
         <is>
           <t>on hand (sensor plug / terminal: never a buy)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q181"/>
+  <autoFilter ref="A1:Q182"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -19380,15 +19433,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M172" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M173" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M174" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M173" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M174" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M175" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M176" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M177" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M178" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M179" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M180" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId101"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -19401,7 +19454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -21302,8 +21355,30 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D86"/>
+  <autoFilter ref="A1:D87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Layout tree: starter S post on the engine tree from bulkhead cavity 3 (Bugbot finding)
The FW_STR -> STARTER segment carried the old cabin-side starter wire; w_strl_e now routes
BH_ENG -> BP_ENG_A2 -> STARTER (450 mm estimate). FW_STR keeps only the RADLOK pair.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>85</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4638.46</v>
+        <v>4618.81</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -571,7 +571,7 @@
         <v>176</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5076.32</v>
+        <v>5056.67</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>24</v>
@@ -12043,7 +12043,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -12054,13 +12054,13 @@
         <v>0</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>20.08</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>60.24</v>
+        <v>40.16</v>
       </c>
       <c r="M62" s="4" t="inlineStr">
         <is>
@@ -12080,7 +12080,7 @@
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>1.9 m of bundle + 10 % cut / recovery margin</t>
+          <t>0.9 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -12169,7 +12169,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -12180,13 +12180,13 @@
         <v>0</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>14.24</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>170.88</v>
+        <v>156.64</v>
       </c>
       <c r="M64" s="4" t="inlineStr">
         <is>
@@ -12206,7 +12206,7 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>10.6 m of bundle + 10 % cut / recovery margin</t>
+          <t>9.2 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
         </is>
       </c>
       <c r="G65" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -12249,13 +12249,13 @@
         <v>0</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K65" s="3" t="n">
         <v>5.61</v>
       </c>
       <c r="L65" s="3" t="n">
-        <v>22.44</v>
+        <v>16.83</v>
       </c>
       <c r="M65" s="5" t="inlineStr">
         <is>
@@ -12275,7 +12275,7 @@
       </c>
       <c r="Q65" s="3" t="inlineStr">
         <is>
-          <t>2.9 m of bundle + 10 % cut / recovery margin</t>
+          <t>2.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -12307,7 +12307,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -12318,13 +12318,13 @@
         <v>0</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>5.54</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>83.09999999999999</v>
+        <v>77.56</v>
       </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
@@ -12344,7 +12344,7 @@
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>13.6 m of bundle + 10 % cut / recovery margin</t>
+          <t>11.9 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -12376,7 +12376,7 @@
         </is>
       </c>
       <c r="G67" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -12387,13 +12387,13 @@
         <v>0</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K67" s="3" t="n">
         <v>14.99</v>
       </c>
       <c r="L67" s="3" t="n">
-        <v>74.95</v>
+        <v>89.94</v>
       </c>
       <c r="M67" s="5" t="inlineStr">
         <is>
@@ -12413,7 +12413,7 @@
       </c>
       <c r="Q67" s="3" t="inlineStr">
         <is>
-          <t>4.0 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.9 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -12445,7 +12445,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -12456,13 +12456,13 @@
         <v>0</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>10.83</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>75.81</v>
+        <v>86.64</v>
       </c>
       <c r="M68" s="4" t="inlineStr">
         <is>
@@ -12482,7 +12482,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>6.8 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fans 10 AWG / 30 A for a 12 in 18 A fan (N78); FP fuse stays 40 A (N79)
- Fan feeds and grounds 8 -> 10 AWG; AMI FAN 40 -> 30 A (FAN2 already 30 A)
- Relay 30/87 FASTON 280755-4 -> 280756-4 (12-10 AWG, 3.4-5.1 mm insulation; check_terminal_holes G1)
- AMI stud rings Klauke 2R5 (10 mm2) -> TE 36161 (12-10 AWG) on the fan and FP fuse 10 AWG leads
- Fuse-box wiring plan follows the master; DECISIONS B12 cases; tracker; drawings and BOM regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>86</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4649.18</v>
+        <v>4597.1</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>9</v>
@@ -571,7 +571,7 @@
         <v>177</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5087.04</v>
+        <v>5034.96</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>24</v>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>3.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>2.8 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13078,7 +13078,7 @@
         </is>
       </c>
       <c r="G79" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -13089,13 +13089,13 @@
         <v>0</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K79" s="3" t="n">
         <v>14.99</v>
       </c>
       <c r="L79" s="3" t="n">
-        <v>59.96</v>
+        <v>74.95</v>
       </c>
       <c r="M79" s="5" t="inlineStr">
         <is>
@@ -13115,7 +13115,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>3.6 m of bundle + 10 % cut / recovery margin</t>
+          <t>3.9 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13147,7 +13147,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13158,13 +13158,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>10.83</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>64.98</v>
+        <v>75.81</v>
       </c>
       <c r="M80" s="4" t="inlineStr">
         <is>
@@ -13184,7 +13184,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>5.3 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.6 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -14534,7 +14534,7 @@
         </is>
       </c>
       <c r="G101" s="3" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
@@ -14545,13 +14545,13 @@
         <v>0</v>
       </c>
       <c r="J101" s="3" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="K101" s="3" t="n">
         <v>4.08</v>
       </c>
       <c r="L101" s="3" t="n">
-        <v>20.4</v>
+        <v>44.88</v>
       </c>
       <c r="M101" s="5" t="inlineStr">
         <is>
@@ -14571,7 +14571,7 @@
       </c>
       <c r="Q101" s="3" t="inlineStr">
         <is>
-          <t>1.2 m in the master + 15% margin</t>
+          <t>2.8 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -14603,7 +14603,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -14614,13 +14614,13 @@
         <v>0</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>3.5</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>91</v>
+        <v>171.5</v>
       </c>
       <c r="M102" s="4" t="inlineStr">
         <is>
@@ -14640,7 +14640,7 @@
       </c>
       <c r="Q102" s="2" t="inlineStr">
         <is>
-          <t>6.6 m in the master + 15% margin</t>
+          <t>12.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15996,7 +15996,7 @@
         </is>
       </c>
       <c r="G123" s="3" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
@@ -16007,13 +16007,13 @@
         <v>0</v>
       </c>
       <c r="J123" s="3" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="K123" s="3" t="n">
         <v>6.08</v>
       </c>
       <c r="L123" s="3" t="n">
-        <v>79.04000000000001</v>
+        <v>42.56</v>
       </c>
       <c r="M123" s="5" t="inlineStr">
         <is>
@@ -16033,7 +16033,7 @@
       </c>
       <c r="Q123" s="3" t="inlineStr">
         <is>
-          <t>3.2 m in the master + 15% margin</t>
+          <t>1.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16065,7 +16065,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16076,13 +16076,13 @@
         <v>0</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>6.1</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>231.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="M124" s="4" t="inlineStr">
         <is>
@@ -16102,7 +16102,7 @@
       </c>
       <c r="Q124" s="2" t="inlineStr">
         <is>
-          <t>9.9 m in the master + 15% margin</t>
+          <t>3.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Row 176: drawing generator without bands or pinout sheet; BOM and pin chart regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$199</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -540,19 +540,19 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>4286.18</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -562,19 +562,19 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>4724.04</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -8333,7 +8333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q205"/>
+  <dimension ref="A1:Q199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17121,55 +17121,43 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-4-STK</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr"/>
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, YELLOW, 2:1, 4.8 MM EXPANDED ID, 2.4 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (ALT-PLUG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I140" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K140" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L140" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr"/>
       <c r="M140" s="2" t="inlineStr"/>
       <c r="N140" s="2" t="inlineStr"/>
-      <c r="O140" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O140" s="2" t="inlineStr"/>
       <c r="P140" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q140" s="2" t="inlineStr">
         <is>
-          <t>34 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17186,55 +17174,43 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-6-STK</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr"/>
       <c r="E141" s="3" t="inlineStr"/>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, BLUE, 2:1, 4.8 MM EXPANDED ID, 2.4 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G141" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I141" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J141" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K141" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L141" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="3" t="inlineStr"/>
       <c r="M141" s="3" t="inlineStr"/>
       <c r="N141" s="3" t="inlineStr"/>
-      <c r="O141" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O141" s="3" t="inlineStr"/>
       <c r="P141" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q141" s="3" t="inlineStr">
         <is>
-          <t>58 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17251,55 +17227,43 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-9-STK</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr"/>
       <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, WHITE, 2:1, 4.8 MM EXPANDED ID, 2.4 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-1) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I142" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K142" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L142" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K142" s="2" t="inlineStr"/>
+      <c r="L142" s="2" t="inlineStr"/>
       <c r="M142" s="2" t="inlineStr"/>
       <c r="N142" s="2" t="inlineStr"/>
-      <c r="O142" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O142" s="2" t="inlineStr"/>
       <c r="P142" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q142" s="2" t="inlineStr">
         <is>
-          <t>52 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17316,18 +17280,14 @@
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-4-STK</t>
-        </is>
-      </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr"/>
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, YELLOW, 2:1, 2.4 MM EXPANDED ID, 1.2 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G143" s="3" t="n">
@@ -17335,7 +17295,7 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I143" s="3" t="n">
@@ -17344,27 +17304,19 @@
       <c r="J143" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K143" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L143" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="3" t="inlineStr"/>
       <c r="M143" s="3" t="inlineStr"/>
       <c r="N143" s="3" t="inlineStr"/>
-      <c r="O143" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O143" s="3" t="inlineStr"/>
       <c r="P143" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q143" s="3" t="inlineStr">
         <is>
-          <t>570 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17381,55 +17333,43 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-6-STK</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr"/>
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, BLUE, 2:1, 2.4 MM EXPANDED ID, 1.2 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I144" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J144" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K144" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L144" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr"/>
       <c r="M144" s="2" t="inlineStr"/>
       <c r="N144" s="2" t="inlineStr"/>
-      <c r="O144" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O144" s="2" t="inlineStr"/>
       <c r="P144" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q144" s="2" t="inlineStr">
         <is>
-          <t>820 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17446,55 +17386,43 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-9-STK</t>
-        </is>
-      </c>
-      <c r="D145" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr"/>
       <c r="E145" s="3" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, WHITE, 2:1, 2.4 MM EXPANDED ID, 1.2 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-4) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G145" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I145" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J145" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="K145" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L145" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="3" t="inlineStr"/>
       <c r="M145" s="3" t="inlineStr"/>
       <c r="N145" s="3" t="inlineStr"/>
-      <c r="O145" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O145" s="3" t="inlineStr"/>
       <c r="P145" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q145" s="3" t="inlineStr">
         <is>
-          <t>408 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17518,11 +17446,11 @@
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ALT-PLUG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-A) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -17533,7 +17461,7 @@
         <v>0</v>
       </c>
       <c r="J146" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr"/>
@@ -17571,11 +17499,11 @@
       <c r="E147" s="3" t="inlineStr"/>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G147" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
@@ -17586,7 +17514,7 @@
         <v>0</v>
       </c>
       <c r="J147" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K147" s="3" t="inlineStr"/>
       <c r="L147" s="3" t="inlineStr"/>
@@ -17624,11 +17552,11 @@
       <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-1) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -17639,7 +17567,7 @@
         <v>0</v>
       </c>
       <c r="J148" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr"/>
@@ -17677,11 +17605,11 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G149" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
@@ -17692,7 +17620,7 @@
         <v>0</v>
       </c>
       <c r="J149" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K149" s="3" t="inlineStr"/>
       <c r="L149" s="3" t="inlineStr"/>
@@ -17730,11 +17658,11 @@
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -17745,7 +17673,7 @@
         <v>0</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
@@ -17783,11 +17711,11 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-4) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G151" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
@@ -17798,7 +17726,7 @@
         <v>0</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K151" s="3" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr"/>
@@ -17836,11 +17764,11 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-A) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -17851,7 +17779,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
@@ -17889,11 +17817,11 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G153" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
@@ -17904,7 +17832,7 @@
         <v>0</v>
       </c>
       <c r="J153" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K153" s="3" t="inlineStr"/>
       <c r="L153" s="3" t="inlineStr"/>
@@ -17942,11 +17870,11 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -17957,7 +17885,7 @@
         <v>0</v>
       </c>
       <c r="J154" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr"/>
@@ -17995,7 +17923,7 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G155" s="3" t="n">
@@ -18048,11 +17976,11 @@
       <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -18063,7 +17991,7 @@
         <v>0</v>
       </c>
       <c r="J156" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr"/>
@@ -18101,11 +18029,11 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G157" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
@@ -18116,7 +18044,7 @@
         <v>0</v>
       </c>
       <c r="J157" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K157" s="3" t="inlineStr"/>
       <c r="L157" s="3" t="inlineStr"/>
@@ -18154,11 +18082,11 @@
       <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -18169,7 +18097,7 @@
         <v>0</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr"/>
@@ -18207,7 +18135,7 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G159" s="3" t="n">
@@ -18260,7 +18188,7 @@
       <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G160" s="2" t="n">
@@ -18313,7 +18241,7 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -18366,7 +18294,7 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G162" s="2" t="n">
@@ -18419,7 +18347,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G163" s="3" t="n">
@@ -18472,11 +18400,11 @@
       <c r="E164" s="2" t="inlineStr"/>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -18487,7 +18415,7 @@
         <v>0</v>
       </c>
       <c r="J164" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K164" s="2" t="inlineStr"/>
       <c r="L164" s="2" t="inlineStr"/>
@@ -18525,11 +18453,11 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
@@ -18540,7 +18468,7 @@
         <v>0</v>
       </c>
       <c r="J165" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K165" s="3" t="inlineStr"/>
       <c r="L165" s="3" t="inlineStr"/>
@@ -18578,11 +18506,11 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -18593,7 +18521,7 @@
         <v>0</v>
       </c>
       <c r="J166" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K166" s="2" t="inlineStr"/>
       <c r="L166" s="2" t="inlineStr"/>
@@ -18631,7 +18559,7 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G167" s="3" t="n">
@@ -18684,7 +18612,7 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
@@ -18737,11 +18665,11 @@
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
@@ -18752,7 +18680,7 @@
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K169" s="3" t="inlineStr"/>
       <c r="L169" s="3" t="inlineStr"/>
@@ -18790,11 +18718,11 @@
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -18805,7 +18733,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K170" s="2" t="inlineStr"/>
       <c r="L170" s="2" t="inlineStr"/>
@@ -18843,11 +18771,11 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
@@ -18858,7 +18786,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K171" s="3" t="inlineStr"/>
       <c r="L171" s="3" t="inlineStr"/>
@@ -18896,11 +18824,11 @@
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18911,7 +18839,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K172" s="2" t="inlineStr"/>
       <c r="L172" s="2" t="inlineStr"/>
@@ -18949,7 +18877,7 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
@@ -19002,7 +18930,7 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
@@ -19055,11 +18983,11 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
@@ -19070,7 +18998,7 @@
         <v>0</v>
       </c>
       <c r="J175" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K175" s="3" t="inlineStr"/>
       <c r="L175" s="3" t="inlineStr"/>
@@ -19108,11 +19036,11 @@
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -19123,7 +19051,7 @@
         <v>0</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K176" s="2" t="inlineStr"/>
       <c r="L176" s="2" t="inlineStr"/>
@@ -19161,7 +19089,7 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
@@ -19214,7 +19142,7 @@
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
@@ -19267,7 +19195,7 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
@@ -19320,7 +19248,7 @@
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19366,18 +19294,22 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr"/>
+          <t>TMS-SCE-1/2-2.0-9</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G181" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
@@ -19388,23 +19320,27 @@
         <v>0</v>
       </c>
       <c r="J181" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K181" s="3" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="K181" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="M181" s="3" t="inlineStr"/>
       <c r="N181" s="3" t="inlineStr"/>
-      <c r="O181" s="3" t="inlineStr"/>
+      <c r="O181" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P181" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q181" s="3" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q181" s="3" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -19419,18 +19355,22 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr"/>
+          <t>TMS-SCE-3/16-2.0-9</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -19441,23 +19381,27 @@
         <v>0</v>
       </c>
       <c r="J182" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="2" t="inlineStr"/>
+        <v>34</v>
+      </c>
+      <c r="K182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L182" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M182" s="2" t="inlineStr"/>
       <c r="N182" s="2" t="inlineStr"/>
-      <c r="O182" s="2" t="inlineStr"/>
+      <c r="O182" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q182" s="2" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -19472,18 +19416,22 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D183" s="3" t="inlineStr"/>
+          <t>TMS-SCE-3/8-2.0-9</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E183" s="3" t="inlineStr"/>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
@@ -19494,23 +19442,27 @@
         <v>0</v>
       </c>
       <c r="J183" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K183" s="3" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="K183" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L183" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="M183" s="3" t="inlineStr"/>
       <c r="N183" s="3" t="inlineStr"/>
-      <c r="O183" s="3" t="inlineStr"/>
+      <c r="O183" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P183" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q183" s="3" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -19525,18 +19477,22 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D184" s="2" t="inlineStr"/>
+          <t>W12S</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Deutsch (TE Connectivity)</t>
+        </is>
+      </c>
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -19544,26 +19500,34 @@
         </is>
       </c>
       <c r="I184" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J184" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="2" t="inlineStr"/>
-      <c r="M184" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="K184" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L184" s="2" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="M184" s="5" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
+        </is>
+      </c>
       <c r="N184" s="2" t="inlineStr"/>
-      <c r="O184" s="2" t="inlineStr"/>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+        </is>
+      </c>
       <c r="P184" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q184" s="2" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+        </is>
+      </c>
+      <c r="Q184" s="2" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -19578,18 +19542,26 @@
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D185" s="3" t="inlineStr"/>
-      <c r="E185" s="3" t="inlineStr"/>
+          <t>W2P</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G185" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
@@ -19600,23 +19572,31 @@
         <v>0</v>
       </c>
       <c r="J185" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K185" s="3" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr"/>
-      <c r="M185" s="3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K185" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L185" s="3" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="M185" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+        </is>
+      </c>
       <c r="N185" s="3" t="inlineStr"/>
-      <c r="O185" s="3" t="inlineStr"/>
+      <c r="O185" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="P185" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q185" s="3" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>Digi-Key product page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -19631,18 +19611,26 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr"/>
-      <c r="E186" s="2" t="inlineStr"/>
+          <t>W2S</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -19653,23 +19641,31 @@
         <v>0</v>
       </c>
       <c r="J186" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="2" t="inlineStr"/>
-      <c r="M186" s="2" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="K186" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L186" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M186" s="5" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-W2S.html</t>
+        </is>
+      </c>
       <c r="N186" s="2" t="inlineStr"/>
-      <c r="O186" s="2" t="inlineStr"/>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="P186" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q186" s="2" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -19684,22 +19680,26 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
+          <t>W3P</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
-      <c r="E187" s="3" t="inlineStr"/>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
         </is>
       </c>
       <c r="G187" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
@@ -19710,24 +19710,28 @@
         <v>0</v>
       </c>
       <c r="J187" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K187" s="3" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L187" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M187" s="3" t="inlineStr"/>
+        <v>0.13</v>
+      </c>
+      <c r="M187" s="4" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-W3P.html</t>
+        </is>
+      </c>
       <c r="N187" s="3" t="inlineStr"/>
       <c r="O187" s="3" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P187" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q187" s="3" t="inlineStr"/>
@@ -19745,22 +19749,26 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
-      <c r="E188" s="2" t="inlineStr"/>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -19771,24 +19779,28 @@
         <v>0</v>
       </c>
       <c r="J188" s="2" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="K188" s="2" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L188" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M188" s="2" t="inlineStr"/>
+        <v>0.39</v>
+      </c>
+      <c r="M188" s="5" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-W3S.html</t>
+        </is>
+      </c>
       <c r="N188" s="2" t="inlineStr"/>
       <c r="O188" s="2" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P188" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q188" s="2" t="inlineStr"/>
@@ -19806,22 +19818,26 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
-      <c r="E189" s="3" t="inlineStr"/>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G189" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
@@ -19832,24 +19848,28 @@
         <v>0</v>
       </c>
       <c r="J189" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="K189" s="3" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L189" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M189" s="3" t="inlineStr"/>
+        <v>0.4</v>
+      </c>
+      <c r="M189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+        </is>
+      </c>
       <c r="N189" s="3" t="inlineStr"/>
       <c r="O189" s="3" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q189" s="3" t="inlineStr"/>
@@ -19867,22 +19887,26 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr"/>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -19890,31 +19914,31 @@
         </is>
       </c>
       <c r="I190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J190" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="K190" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="L190" s="2" t="n">
         <v>0.42</v>
       </c>
-      <c r="L190" s="2" t="n">
-        <v>1.26</v>
-      </c>
       <c r="M190" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N190" s="2" t="inlineStr"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr"/>
@@ -19932,7 +19956,7 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -19947,11 +19971,11 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G191" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
@@ -19962,28 +19986,28 @@
         <v>0</v>
       </c>
       <c r="J191" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K191" s="3" t="n">
-        <v>0.13</v>
+        <v>0.35</v>
       </c>
       <c r="L191" s="3" t="n">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="M191" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N191" s="3" t="inlineStr"/>
       <c r="O191" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P191" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
         </is>
       </c>
       <c r="Q191" s="3" t="inlineStr"/>
@@ -20001,7 +20025,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>WM-4S</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -20016,11 +20040,11 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -20031,28 +20055,28 @@
         <v>0</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K192" s="2" t="n">
-        <v>0.13</v>
+        <v>0.28</v>
       </c>
       <c r="L192" s="2" t="n">
-        <v>1.3</v>
+        <v>0.28</v>
       </c>
       <c r="M192" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
         </is>
       </c>
       <c r="N192" s="2" t="inlineStr"/>
       <c r="O192" s="2" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P192" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
         </is>
       </c>
       <c r="Q192" s="2" t="inlineStr"/>
@@ -20070,7 +20094,7 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>W3P</t>
+          <t>WM-6S</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -20085,7 +20109,7 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
         </is>
       </c>
       <c r="G193" s="3" t="n">
@@ -20103,25 +20127,25 @@
         <v>1</v>
       </c>
       <c r="K193" s="3" t="n">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
       <c r="L193" s="3" t="n">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
       <c r="M193" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
         </is>
       </c>
       <c r="N193" s="3" t="inlineStr"/>
       <c r="O193" s="3" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P193" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
         </is>
       </c>
       <c r="Q193" s="3" t="inlineStr"/>
@@ -20139,26 +20163,14 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>W3S</t>
-        </is>
-      </c>
-      <c r="D194" s="2" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="E194" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
-        </is>
-      </c>
+          <t>in kit 354404</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr"/>
+      <c r="E194" s="2" t="inlineStr"/>
+      <c r="F194" s="2" t="inlineStr"/>
       <c r="G194" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -20166,34 +20178,26 @@
         </is>
       </c>
       <c r="I194" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K194" s="2" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="L194" s="2" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="M194" s="5" t="inlineStr">
-        <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="2" t="inlineStr"/>
+      <c r="M194" s="2" t="inlineStr"/>
       <c r="N194" s="2" t="inlineStr"/>
-      <c r="O194" s="2" t="inlineStr">
-        <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
-        </is>
-      </c>
+      <c r="O194" s="2" t="inlineStr"/>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
-        </is>
-      </c>
-      <c r="Q194" s="2" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -20208,24 +20212,12 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>W6P</t>
-        </is>
-      </c>
-      <c r="D195" s="3" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E195" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F195" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
-        </is>
-      </c>
+          <t>in kit CONN-75800</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr"/>
+      <c r="E195" s="3" t="inlineStr"/>
+      <c r="F195" s="3" t="inlineStr"/>
       <c r="G195" s="3" t="n">
         <v>2</v>
       </c>
@@ -20235,34 +20227,26 @@
         </is>
       </c>
       <c r="I195" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J195" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K195" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L195" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="M195" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K195" s="3" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr"/>
+      <c r="M195" s="3" t="inlineStr"/>
       <c r="N195" s="3" t="inlineStr"/>
-      <c r="O195" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O195" s="3" t="inlineStr"/>
       <c r="P195" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
-        </is>
-      </c>
-      <c r="Q195" s="3" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q195" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -20277,26 +20261,14 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>W6S</t>
-        </is>
-      </c>
-      <c r="D196" s="2" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E196" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F196" s="2" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
-        </is>
-      </c>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr"/>
+      <c r="E196" s="2" t="inlineStr"/>
+      <c r="F196" s="2" t="inlineStr"/>
       <c r="G196" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -20307,28 +20279,16 @@
         <v>0</v>
       </c>
       <c r="J196" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K196" s="2" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="L196" s="2" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="M196" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="2" t="inlineStr"/>
+      <c r="M196" s="2" t="inlineStr"/>
       <c r="N196" s="2" t="inlineStr"/>
-      <c r="O196" s="2" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O196" s="2" t="inlineStr"/>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q196" s="2" t="inlineStr"/>
@@ -20346,26 +20306,14 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>W8S</t>
-        </is>
-      </c>
-      <c r="D197" s="3" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E197" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F197" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
-        </is>
-      </c>
+          <t>in kit CONN-76270</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr"/>
+      <c r="E197" s="3" t="inlineStr"/>
+      <c r="F197" s="3" t="inlineStr"/>
       <c r="G197" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H197" s="3" t="inlineStr">
         <is>
@@ -20373,34 +20321,26 @@
         </is>
       </c>
       <c r="I197" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J197" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K197" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="L197" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="M197" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K197" s="3" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr"/>
+      <c r="M197" s="3" t="inlineStr"/>
       <c r="N197" s="3" t="inlineStr"/>
-      <c r="O197" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O197" s="3" t="inlineStr"/>
       <c r="P197" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
-        </is>
-      </c>
-      <c r="Q197" s="3" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q197" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -20415,26 +20355,14 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>WM-4S</t>
-        </is>
-      </c>
-      <c r="D198" s="2" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E198" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
-        </is>
-      </c>
+          <t>in kit D 261 205 358-01</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr"/>
+      <c r="E198" s="2" t="inlineStr"/>
+      <c r="F198" s="2" t="inlineStr"/>
       <c r="G198" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -20445,28 +20373,16 @@
         <v>0</v>
       </c>
       <c r="J198" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K198" s="2" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="L198" s="2" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="M198" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="2" t="inlineStr"/>
+      <c r="M198" s="2" t="inlineStr"/>
       <c r="N198" s="2" t="inlineStr"/>
-      <c r="O198" s="2" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O198" s="2" t="inlineStr"/>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q198" s="2" t="inlineStr"/>
@@ -20484,24 +20400,12 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>WM-6S</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="E199" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F199" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
-        </is>
-      </c>
+          <t>pigtail supplied with the sensor (owned)</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr"/>
+      <c r="E199" s="3" t="inlineStr"/>
+      <c r="F199" s="3" t="inlineStr"/>
       <c r="G199" s="3" t="n">
         <v>1</v>
       </c>
@@ -20511,323 +20415,29 @@
         </is>
       </c>
       <c r="I199" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J199" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K199" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="L199" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="M199" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K199" s="3" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr"/>
+      <c r="M199" s="3" t="inlineStr"/>
       <c r="N199" s="3" t="inlineStr"/>
-      <c r="O199" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O199" s="3" t="inlineStr"/>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
-        </is>
-      </c>
-      <c r="Q199" s="3" t="inlineStr"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B200" s="2" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C200" s="2" t="inlineStr">
-        <is>
-          <t>in kit 354404</t>
-        </is>
-      </c>
-      <c r="D200" s="2" t="inlineStr"/>
-      <c r="E200" s="2" t="inlineStr"/>
-      <c r="F200" s="2" t="inlineStr"/>
-      <c r="G200" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="H200" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I200" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="J200" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="2" t="inlineStr"/>
-      <c r="M200" s="2" t="inlineStr"/>
-      <c r="N200" s="2" t="inlineStr"/>
-      <c r="O200" s="2" t="inlineStr"/>
-      <c r="P200" s="2" t="inlineStr">
-        <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q200" s="2" t="inlineStr">
+      <c r="Q199" s="3" t="inlineStr">
         <is>
           <t>on hand (sensor plug / terminal: never a buy)</t>
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>in kit CONN-75800</t>
-        </is>
-      </c>
-      <c r="D201" s="3" t="inlineStr"/>
-      <c r="E201" s="3" t="inlineStr"/>
-      <c r="F201" s="3" t="inlineStr"/>
-      <c r="G201" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H201" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I201" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J201" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K201" s="3" t="inlineStr"/>
-      <c r="L201" s="3" t="inlineStr"/>
-      <c r="M201" s="3" t="inlineStr"/>
-      <c r="N201" s="3" t="inlineStr"/>
-      <c r="O201" s="3" t="inlineStr"/>
-      <c r="P201" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q201" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B202" s="2" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C202" s="2" t="inlineStr">
-        <is>
-          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr"/>
-      <c r="E202" s="2" t="inlineStr"/>
-      <c r="F202" s="2" t="inlineStr"/>
-      <c r="G202" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H202" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I202" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J202" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K202" s="2" t="inlineStr"/>
-      <c r="L202" s="2" t="inlineStr"/>
-      <c r="M202" s="2" t="inlineStr"/>
-      <c r="N202" s="2" t="inlineStr"/>
-      <c r="O202" s="2" t="inlineStr"/>
-      <c r="P202" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q202" s="2" t="inlineStr"/>
-    </row>
-    <row r="203">
-      <c r="A203" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B203" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C203" s="3" t="inlineStr">
-        <is>
-          <t>in kit CONN-76270</t>
-        </is>
-      </c>
-      <c r="D203" s="3" t="inlineStr"/>
-      <c r="E203" s="3" t="inlineStr"/>
-      <c r="F203" s="3" t="inlineStr"/>
-      <c r="G203" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="H203" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I203" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="J203" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K203" s="3" t="inlineStr"/>
-      <c r="L203" s="3" t="inlineStr"/>
-      <c r="M203" s="3" t="inlineStr"/>
-      <c r="N203" s="3" t="inlineStr"/>
-      <c r="O203" s="3" t="inlineStr"/>
-      <c r="P203" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q203" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B204" s="2" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C204" s="2" t="inlineStr">
-        <is>
-          <t>in kit D 261 205 358-01</t>
-        </is>
-      </c>
-      <c r="D204" s="2" t="inlineStr"/>
-      <c r="E204" s="2" t="inlineStr"/>
-      <c r="F204" s="2" t="inlineStr"/>
-      <c r="G204" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H204" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I204" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J204" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K204" s="2" t="inlineStr"/>
-      <c r="L204" s="2" t="inlineStr"/>
-      <c r="M204" s="2" t="inlineStr"/>
-      <c r="N204" s="2" t="inlineStr"/>
-      <c r="O204" s="2" t="inlineStr"/>
-      <c r="P204" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q204" s="2" t="inlineStr"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B205" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C205" s="3" t="inlineStr">
-        <is>
-          <t>pigtail supplied with the sensor (owned)</t>
-        </is>
-      </c>
-      <c r="D205" s="3" t="inlineStr"/>
-      <c r="E205" s="3" t="inlineStr"/>
-      <c r="F205" s="3" t="inlineStr"/>
-      <c r="G205" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H205" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I205" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J205" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K205" s="3" t="inlineStr"/>
-      <c r="L205" s="3" t="inlineStr"/>
-      <c r="M205" s="3" t="inlineStr"/>
-      <c r="N205" s="3" t="inlineStr"/>
-      <c r="O205" s="3" t="inlineStr"/>
-      <c r="P205" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q205" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q205"/>
+  <autoFilter ref="A1:Q199"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -20927,16 +20537,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Row 176: no ident bands anywhere; the pin chart is the one pinout (#442)
* WIP row 176: no ident bands, drop the drawing-set pinout PDF (generator edit in progress)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

* Row 176: drawing generator without bands or pinout sheet; BOM and pin chart regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$199</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -540,19 +540,19 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>4286.18</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -562,19 +562,19 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>4724.04</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -8333,7 +8333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q205"/>
+  <dimension ref="A1:Q199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17121,55 +17121,43 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-4-STK</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr"/>
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, YELLOW, 2:1, 4.8 MM EXPANDED ID, 2.4 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (ALT-PLUG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I140" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K140" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L140" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr"/>
       <c r="M140" s="2" t="inlineStr"/>
       <c r="N140" s="2" t="inlineStr"/>
-      <c r="O140" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O140" s="2" t="inlineStr"/>
       <c r="P140" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q140" s="2" t="inlineStr">
         <is>
-          <t>34 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17186,55 +17174,43 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-6-STK</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr"/>
       <c r="E141" s="3" t="inlineStr"/>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, BLUE, 2:1, 4.8 MM EXPANDED ID, 2.4 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G141" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I141" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J141" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K141" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L141" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="3" t="inlineStr"/>
       <c r="M141" s="3" t="inlineStr"/>
       <c r="N141" s="3" t="inlineStr"/>
-      <c r="O141" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O141" s="3" t="inlineStr"/>
       <c r="P141" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q141" s="3" t="inlineStr">
         <is>
-          <t>58 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17251,55 +17227,43 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/16-9-STK</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr"/>
       <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, WHITE, 2:1, 4.8 MM EXPANDED ID, 2.4 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-1) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I142" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K142" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L142" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K142" s="2" t="inlineStr"/>
+      <c r="L142" s="2" t="inlineStr"/>
       <c r="M142" s="2" t="inlineStr"/>
       <c r="N142" s="2" t="inlineStr"/>
-      <c r="O142" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O142" s="2" t="inlineStr"/>
       <c r="P142" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q142" s="2" t="inlineStr">
         <is>
-          <t>52 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17316,18 +17280,14 @@
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-4-STK</t>
-        </is>
-      </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr"/>
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, YELLOW, 2:1, 2.4 MM EXPANDED ID, 1.2 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G143" s="3" t="n">
@@ -17335,7 +17295,7 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I143" s="3" t="n">
@@ -17344,27 +17304,19 @@
       <c r="J143" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K143" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L143" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="3" t="inlineStr"/>
       <c r="M143" s="3" t="inlineStr"/>
       <c r="N143" s="3" t="inlineStr"/>
-      <c r="O143" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O143" s="3" t="inlineStr"/>
       <c r="P143" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q143" s="3" t="inlineStr">
         <is>
-          <t>570 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17381,55 +17333,43 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-6-STK</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr"/>
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, BLUE, 2:1, 2.4 MM EXPANDED ID, 1.2 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I144" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J144" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K144" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L144" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr"/>
       <c r="M144" s="2" t="inlineStr"/>
       <c r="N144" s="2" t="inlineStr"/>
-      <c r="O144" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O144" s="2" t="inlineStr"/>
       <c r="P144" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q144" s="2" t="inlineStr">
         <is>
-          <t>820 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17446,55 +17386,43 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>RNF-100-3/32-9-STK</t>
-        </is>
-      </c>
-      <c r="D145" s="3" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr"/>
       <c r="E145" s="3" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>TUBING, HEAT SHRINK, RNF-100, WHITE, 2:1, 2.4 MM EXPANDED ID, 1.2 MM RECOVERED ID, 1.2 M STICK</t>
+          <t>part number not confirmed yet: contact / plug (COIL-4) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G145" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>stick</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="I145" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J145" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="K145" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L145" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="3" t="inlineStr"/>
       <c r="M145" s="3" t="inlineStr"/>
       <c r="N145" s="3" t="inlineStr"/>
-      <c r="O145" s="3" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O145" s="3" t="inlineStr"/>
       <c r="P145" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q145" s="3" t="inlineStr">
         <is>
-          <t>408 bands of 6 mm, both ends of each wire</t>
+          <t>no maker document in the repo yet; never guessed</t>
         </is>
       </c>
     </row>
@@ -17518,11 +17446,11 @@
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ALT-PLUG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-A) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -17533,7 +17461,7 @@
         <v>0</v>
       </c>
       <c r="J146" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr"/>
@@ -17571,11 +17499,11 @@
       <c r="E147" s="3" t="inlineStr"/>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G147" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
@@ -17586,7 +17514,7 @@
         <v>0</v>
       </c>
       <c r="J147" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K147" s="3" t="inlineStr"/>
       <c r="L147" s="3" t="inlineStr"/>
@@ -17624,11 +17552,11 @@
       <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-1) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -17639,7 +17567,7 @@
         <v>0</v>
       </c>
       <c r="J148" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr"/>
@@ -17677,11 +17605,11 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G149" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
@@ -17692,7 +17620,7 @@
         <v>0</v>
       </c>
       <c r="J149" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K149" s="3" t="inlineStr"/>
       <c r="L149" s="3" t="inlineStr"/>
@@ -17730,11 +17658,11 @@
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -17745,7 +17673,7 @@
         <v>0</v>
       </c>
       <c r="J150" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
@@ -17783,11 +17711,11 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (COIL-4) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G151" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
@@ -17798,7 +17726,7 @@
         <v>0</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K151" s="3" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr"/>
@@ -17836,11 +17764,11 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-A) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -17851,7 +17779,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
@@ -17889,11 +17817,11 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (ECU-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G153" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
@@ -17904,7 +17832,7 @@
         <v>0</v>
       </c>
       <c r="J153" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K153" s="3" t="inlineStr"/>
       <c r="L153" s="3" t="inlineStr"/>
@@ -17942,11 +17870,11 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -17957,7 +17885,7 @@
         <v>0</v>
       </c>
       <c r="J154" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr"/>
@@ -17995,7 +17923,7 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G155" s="3" t="n">
@@ -18048,11 +17976,11 @@
       <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (KILL-SW) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -18063,7 +17991,7 @@
         <v>0</v>
       </c>
       <c r="J156" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr"/>
@@ -18101,11 +18029,11 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G157" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
@@ -18116,7 +18044,7 @@
         <v>0</v>
       </c>
       <c r="J157" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K157" s="3" t="inlineStr"/>
       <c r="L157" s="3" t="inlineStr"/>
@@ -18154,11 +18082,11 @@
       <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: contact / plug (MRS-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -18169,7 +18097,7 @@
         <v>0</v>
       </c>
       <c r="J158" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr"/>
@@ -18207,7 +18135,7 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-CHG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G159" s="3" t="n">
@@ -18260,7 +18188,7 @@
       <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-HB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G160" s="2" t="n">
@@ -18313,7 +18241,7 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-OIL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -18366,7 +18294,7 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-PK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G162" s="2" t="n">
@@ -18419,7 +18347,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G163" s="3" t="n">
@@ -18472,11 +18400,11 @@
       <c r="E164" s="2" t="inlineStr"/>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: diode (D-TR) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -18487,7 +18415,7 @@
         <v>0</v>
       </c>
       <c r="J164" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K164" s="2" t="inlineStr"/>
       <c r="L164" s="2" t="inlineStr"/>
@@ -18525,11 +18453,11 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (APS-PEDAL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
@@ -18540,7 +18468,7 @@
         <v>0</v>
       </c>
       <c r="J165" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K165" s="3" t="inlineStr"/>
       <c r="L165" s="3" t="inlineStr"/>
@@ -18578,11 +18506,11 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (FUEL-PUMP) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -18593,7 +18521,7 @@
         <v>0</v>
       </c>
       <c r="J166" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K166" s="2" t="inlineStr"/>
       <c r="L166" s="2" t="inlineStr"/>
@@ -18631,7 +18559,7 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (JUMP-POST) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G167" s="3" t="n">
@@ -18684,7 +18612,7 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: housing (OPTO-8) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
@@ -18737,11 +18665,11 @@
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (BATT-POS) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
@@ -18752,7 +18680,7 @@
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K169" s="3" t="inlineStr"/>
       <c r="L169" s="3" t="inlineStr"/>
@@ -18790,11 +18718,11 @@
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EA) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -18805,7 +18733,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K170" s="2" t="inlineStr"/>
       <c r="L170" s="2" t="inlineStr"/>
@@ -18843,11 +18771,11 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-EB) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
@@ -18858,7 +18786,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K171" s="3" t="inlineStr"/>
       <c r="L171" s="3" t="inlineStr"/>
@@ -18896,11 +18824,11 @@
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18911,7 +18839,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K172" s="2" t="inlineStr"/>
       <c r="L172" s="2" t="inlineStr"/>
@@ -18949,7 +18877,7 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
@@ -19002,7 +18930,7 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
@@ -19055,11 +18983,11 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
@@ -19070,7 +18998,7 @@
         <v>0</v>
       </c>
       <c r="J175" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K175" s="3" t="inlineStr"/>
       <c r="L175" s="3" t="inlineStr"/>
@@ -19108,11 +19036,11 @@
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -19123,7 +19051,7 @@
         <v>0</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K176" s="2" t="inlineStr"/>
       <c r="L176" s="2" t="inlineStr"/>
@@ -19161,7 +19089,7 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
@@ -19214,7 +19142,7 @@
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
@@ -19267,7 +19195,7 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
@@ -19320,7 +19248,7 @@
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19366,18 +19294,22 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr"/>
+          <t>TMS-SCE-1/2-2.0-9</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G181" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
@@ -19388,23 +19320,27 @@
         <v>0</v>
       </c>
       <c r="J181" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K181" s="3" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="K181" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="M181" s="3" t="inlineStr"/>
       <c r="N181" s="3" t="inlineStr"/>
-      <c r="O181" s="3" t="inlineStr"/>
+      <c r="O181" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P181" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q181" s="3" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q181" s="3" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -19419,18 +19355,22 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr"/>
+          <t>TMS-SCE-3/16-2.0-9</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -19441,23 +19381,27 @@
         <v>0</v>
       </c>
       <c r="J182" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="2" t="inlineStr"/>
+        <v>34</v>
+      </c>
+      <c r="K182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L182" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M182" s="2" t="inlineStr"/>
       <c r="N182" s="2" t="inlineStr"/>
-      <c r="O182" s="2" t="inlineStr"/>
+      <c r="O182" s="2" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q182" s="2" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -19472,18 +19416,22 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D183" s="3" t="inlineStr"/>
+          <t>TMS-SCE-3/8-2.0-9</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>TE Connectivity (Raychem)</t>
+        </is>
+      </c>
       <c r="E183" s="3" t="inlineStr"/>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
@@ -19494,23 +19442,27 @@
         <v>0</v>
       </c>
       <c r="J183" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K183" s="3" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="K183" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L183" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="M183" s="3" t="inlineStr"/>
       <c r="N183" s="3" t="inlineStr"/>
-      <c r="O183" s="3" t="inlineStr"/>
+      <c r="O183" s="3" t="inlineStr">
+        <is>
+          <t>not priced (Dan)</t>
+        </is>
+      </c>
       <c r="P183" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q183" s="3" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+        </is>
+      </c>
+      <c r="Q183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -19525,18 +19477,22 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D184" s="2" t="inlineStr"/>
+          <t>W12S</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Deutsch (TE Connectivity)</t>
+        </is>
+      </c>
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -19544,26 +19500,34 @@
         </is>
       </c>
       <c r="I184" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J184" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="2" t="inlineStr"/>
-      <c r="M184" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="K184" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L184" s="2" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="M184" s="5" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
+        </is>
+      </c>
       <c r="N184" s="2" t="inlineStr"/>
-      <c r="O184" s="2" t="inlineStr"/>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+        </is>
+      </c>
       <c r="P184" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q184" s="2" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+        </is>
+      </c>
+      <c r="Q184" s="2" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -19578,18 +19542,26 @@
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D185" s="3" t="inlineStr"/>
-      <c r="E185" s="3" t="inlineStr"/>
+          <t>W2P</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G185" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
@@ -19600,23 +19572,31 @@
         <v>0</v>
       </c>
       <c r="J185" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K185" s="3" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr"/>
-      <c r="M185" s="3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K185" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L185" s="3" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="M185" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+        </is>
+      </c>
       <c r="N185" s="3" t="inlineStr"/>
-      <c r="O185" s="3" t="inlineStr"/>
+      <c r="O185" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1, 2026-10-19</t>
+        </is>
+      </c>
       <c r="P185" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q185" s="3" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>Digi-Key product page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -19631,18 +19611,26 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr"/>
-      <c r="E186" s="2" t="inlineStr"/>
+          <t>W2S</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -19653,23 +19641,31 @@
         <v>0</v>
       </c>
       <c r="J186" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="2" t="inlineStr"/>
-      <c r="M186" s="2" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="K186" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L186" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M186" s="5" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-W2S.html</t>
+        </is>
+      </c>
       <c r="N186" s="2" t="inlineStr"/>
-      <c r="O186" s="2" t="inlineStr"/>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+        </is>
+      </c>
       <c r="P186" s="2" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q186" s="2" t="inlineStr">
-        <is>
-          <t>no maker document in the repo yet; never guessed</t>
-        </is>
-      </c>
+          <t>te.com page opened 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -19684,22 +19680,26 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
+          <t>W3P</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
-      <c r="E187" s="3" t="inlineStr"/>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
         </is>
       </c>
       <c r="G187" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
@@ -19710,24 +19710,28 @@
         <v>0</v>
       </c>
       <c r="J187" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K187" s="3" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L187" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M187" s="3" t="inlineStr"/>
+        <v>0.13</v>
+      </c>
+      <c r="M187" s="4" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-W3P.html</t>
+        </is>
+      </c>
       <c r="N187" s="3" t="inlineStr"/>
       <c r="O187" s="3" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P187" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q187" s="3" t="inlineStr"/>
@@ -19745,22 +19749,26 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
-      <c r="E188" s="2" t="inlineStr"/>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -19771,24 +19779,28 @@
         <v>0</v>
       </c>
       <c r="J188" s="2" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="K188" s="2" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L188" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M188" s="2" t="inlineStr"/>
+        <v>0.39</v>
+      </c>
+      <c r="M188" s="5" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-W3S.html</t>
+        </is>
+      </c>
       <c r="N188" s="2" t="inlineStr"/>
       <c r="O188" s="2" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P188" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q188" s="2" t="inlineStr"/>
@@ -19806,22 +19818,26 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
-      <c r="E189" s="3" t="inlineStr"/>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G189" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
@@ -19832,24 +19848,28 @@
         <v>0</v>
       </c>
       <c r="J189" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="K189" s="3" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L189" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M189" s="3" t="inlineStr"/>
+        <v>0.4</v>
+      </c>
+      <c r="M189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+        </is>
+      </c>
       <c r="N189" s="3" t="inlineStr"/>
       <c r="O189" s="3" t="inlineStr">
         <is>
-          <t>not priced (Dan)</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q189" s="3" t="inlineStr"/>
@@ -19867,22 +19887,26 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr"/>
+          <t>TE DEUTSCH</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -19890,31 +19914,31 @@
         </is>
       </c>
       <c r="I190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J190" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="K190" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="L190" s="2" t="n">
         <v>0.42</v>
       </c>
-      <c r="L190" s="2" t="n">
-        <v>1.26</v>
-      </c>
       <c r="M190" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N190" s="2" t="inlineStr"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr"/>
@@ -19932,7 +19956,7 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -19947,11 +19971,11 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G191" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
@@ -19962,28 +19986,28 @@
         <v>0</v>
       </c>
       <c r="J191" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K191" s="3" t="n">
-        <v>0.13</v>
+        <v>0.35</v>
       </c>
       <c r="L191" s="3" t="n">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="M191" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N191" s="3" t="inlineStr"/>
       <c r="O191" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P191" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
         </is>
       </c>
       <c r="Q191" s="3" t="inlineStr"/>
@@ -20001,7 +20025,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>WM-4S</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -20016,11 +20040,11 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -20031,28 +20055,28 @@
         <v>0</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K192" s="2" t="n">
-        <v>0.13</v>
+        <v>0.28</v>
       </c>
       <c r="L192" s="2" t="n">
-        <v>1.3</v>
+        <v>0.28</v>
       </c>
       <c r="M192" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
         </is>
       </c>
       <c r="N192" s="2" t="inlineStr"/>
       <c r="O192" s="2" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P192" s="2" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
         </is>
       </c>
       <c r="Q192" s="2" t="inlineStr"/>
@@ -20070,7 +20094,7 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>W3P</t>
+          <t>WM-6S</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -20085,7 +20109,7 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
         </is>
       </c>
       <c r="G193" s="3" t="n">
@@ -20103,25 +20127,25 @@
         <v>1</v>
       </c>
       <c r="K193" s="3" t="n">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
       <c r="L193" s="3" t="n">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
       <c r="M193" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3P.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
         </is>
       </c>
       <c r="N193" s="3" t="inlineStr"/>
       <c r="O193" s="3" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P193" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
         </is>
       </c>
       <c r="Q193" s="3" t="inlineStr"/>
@@ -20139,26 +20163,14 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>W3S</t>
-        </is>
-      </c>
-      <c r="D194" s="2" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="E194" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
-        </is>
-      </c>
+          <t>in kit 354404</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr"/>
+      <c r="E194" s="2" t="inlineStr"/>
+      <c r="F194" s="2" t="inlineStr"/>
       <c r="G194" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -20166,34 +20178,26 @@
         </is>
       </c>
       <c r="I194" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K194" s="2" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="L194" s="2" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="M194" s="5" t="inlineStr">
-        <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="2" t="inlineStr"/>
+      <c r="M194" s="2" t="inlineStr"/>
       <c r="N194" s="2" t="inlineStr"/>
-      <c r="O194" s="2" t="inlineStr">
-        <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
-        </is>
-      </c>
+      <c r="O194" s="2" t="inlineStr"/>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
-        </is>
-      </c>
-      <c r="Q194" s="2" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -20208,24 +20212,12 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>W6P</t>
-        </is>
-      </c>
-      <c r="D195" s="3" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E195" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F195" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
-        </is>
-      </c>
+          <t>in kit CONN-75800</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr"/>
+      <c r="E195" s="3" t="inlineStr"/>
+      <c r="F195" s="3" t="inlineStr"/>
       <c r="G195" s="3" t="n">
         <v>2</v>
       </c>
@@ -20235,34 +20227,26 @@
         </is>
       </c>
       <c r="I195" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J195" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K195" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L195" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="M195" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K195" s="3" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr"/>
+      <c r="M195" s="3" t="inlineStr"/>
       <c r="N195" s="3" t="inlineStr"/>
-      <c r="O195" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O195" s="3" t="inlineStr"/>
       <c r="P195" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
-        </is>
-      </c>
-      <c r="Q195" s="3" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q195" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -20277,26 +20261,14 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>W6S</t>
-        </is>
-      </c>
-      <c r="D196" s="2" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E196" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F196" s="2" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
-        </is>
-      </c>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr"/>
+      <c r="E196" s="2" t="inlineStr"/>
+      <c r="F196" s="2" t="inlineStr"/>
       <c r="G196" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -20307,28 +20279,16 @@
         <v>0</v>
       </c>
       <c r="J196" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K196" s="2" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="L196" s="2" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="M196" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="2" t="inlineStr"/>
+      <c r="M196" s="2" t="inlineStr"/>
       <c r="N196" s="2" t="inlineStr"/>
-      <c r="O196" s="2" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O196" s="2" t="inlineStr"/>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q196" s="2" t="inlineStr"/>
@@ -20346,26 +20306,14 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>W8S</t>
-        </is>
-      </c>
-      <c r="D197" s="3" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E197" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F197" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
-        </is>
-      </c>
+          <t>in kit CONN-76270</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr"/>
+      <c r="E197" s="3" t="inlineStr"/>
+      <c r="F197" s="3" t="inlineStr"/>
       <c r="G197" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H197" s="3" t="inlineStr">
         <is>
@@ -20373,34 +20321,26 @@
         </is>
       </c>
       <c r="I197" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J197" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K197" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="L197" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="M197" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K197" s="3" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr"/>
+      <c r="M197" s="3" t="inlineStr"/>
       <c r="N197" s="3" t="inlineStr"/>
-      <c r="O197" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O197" s="3" t="inlineStr"/>
       <c r="P197" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
-        </is>
-      </c>
-      <c r="Q197" s="3" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q197" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -20415,26 +20355,14 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>WM-4S</t>
-        </is>
-      </c>
-      <c r="D198" s="2" t="inlineStr">
-        <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E198" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
-        </is>
-      </c>
+          <t>in kit D 261 205 358-01</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr"/>
+      <c r="E198" s="2" t="inlineStr"/>
+      <c r="F198" s="2" t="inlineStr"/>
       <c r="G198" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -20445,28 +20373,16 @@
         <v>0</v>
       </c>
       <c r="J198" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K198" s="2" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="L198" s="2" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="M198" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="2" t="inlineStr"/>
+      <c r="M198" s="2" t="inlineStr"/>
       <c r="N198" s="2" t="inlineStr"/>
-      <c r="O198" s="2" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O198" s="2" t="inlineStr"/>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>NO LINK</t>
         </is>
       </c>
       <c r="Q198" s="2" t="inlineStr"/>
@@ -20484,24 +20400,12 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>WM-6S</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="E199" s="3" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
-      <c r="F199" s="3" t="inlineStr">
-        <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
-        </is>
-      </c>
+          <t>pigtail supplied with the sensor (owned)</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr"/>
+      <c r="E199" s="3" t="inlineStr"/>
+      <c r="F199" s="3" t="inlineStr"/>
       <c r="G199" s="3" t="n">
         <v>1</v>
       </c>
@@ -20511,323 +20415,29 @@
         </is>
       </c>
       <c r="I199" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J199" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K199" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="L199" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="M199" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K199" s="3" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr"/>
+      <c r="M199" s="3" t="inlineStr"/>
       <c r="N199" s="3" t="inlineStr"/>
-      <c r="O199" s="3" t="inlineStr">
-        <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
-        </is>
-      </c>
+      <c r="O199" s="3" t="inlineStr"/>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
-        </is>
-      </c>
-      <c r="Q199" s="3" t="inlineStr"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B200" s="2" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C200" s="2" t="inlineStr">
-        <is>
-          <t>in kit 354404</t>
-        </is>
-      </c>
-      <c r="D200" s="2" t="inlineStr"/>
-      <c r="E200" s="2" t="inlineStr"/>
-      <c r="F200" s="2" t="inlineStr"/>
-      <c r="G200" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="H200" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I200" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="J200" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="2" t="inlineStr"/>
-      <c r="M200" s="2" t="inlineStr"/>
-      <c r="N200" s="2" t="inlineStr"/>
-      <c r="O200" s="2" t="inlineStr"/>
-      <c r="P200" s="2" t="inlineStr">
-        <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q200" s="2" t="inlineStr">
+      <c r="Q199" s="3" t="inlineStr">
         <is>
           <t>on hand (sensor plug / terminal: never a buy)</t>
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>in kit CONN-75800</t>
-        </is>
-      </c>
-      <c r="D201" s="3" t="inlineStr"/>
-      <c r="E201" s="3" t="inlineStr"/>
-      <c r="F201" s="3" t="inlineStr"/>
-      <c r="G201" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H201" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I201" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J201" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K201" s="3" t="inlineStr"/>
-      <c r="L201" s="3" t="inlineStr"/>
-      <c r="M201" s="3" t="inlineStr"/>
-      <c r="N201" s="3" t="inlineStr"/>
-      <c r="O201" s="3" t="inlineStr"/>
-      <c r="P201" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q201" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B202" s="2" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C202" s="2" t="inlineStr">
-        <is>
-          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr"/>
-      <c r="E202" s="2" t="inlineStr"/>
-      <c r="F202" s="2" t="inlineStr"/>
-      <c r="G202" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H202" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I202" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J202" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K202" s="2" t="inlineStr"/>
-      <c r="L202" s="2" t="inlineStr"/>
-      <c r="M202" s="2" t="inlineStr"/>
-      <c r="N202" s="2" t="inlineStr"/>
-      <c r="O202" s="2" t="inlineStr"/>
-      <c r="P202" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q202" s="2" t="inlineStr"/>
-    </row>
-    <row r="203">
-      <c r="A203" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B203" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C203" s="3" t="inlineStr">
-        <is>
-          <t>in kit CONN-76270</t>
-        </is>
-      </c>
-      <c r="D203" s="3" t="inlineStr"/>
-      <c r="E203" s="3" t="inlineStr"/>
-      <c r="F203" s="3" t="inlineStr"/>
-      <c r="G203" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="H203" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I203" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="J203" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K203" s="3" t="inlineStr"/>
-      <c r="L203" s="3" t="inlineStr"/>
-      <c r="M203" s="3" t="inlineStr"/>
-      <c r="N203" s="3" t="inlineStr"/>
-      <c r="O203" s="3" t="inlineStr"/>
-      <c r="P203" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q203" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="2" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B204" s="2" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C204" s="2" t="inlineStr">
-        <is>
-          <t>in kit D 261 205 358-01</t>
-        </is>
-      </c>
-      <c r="D204" s="2" t="inlineStr"/>
-      <c r="E204" s="2" t="inlineStr"/>
-      <c r="F204" s="2" t="inlineStr"/>
-      <c r="G204" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H204" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I204" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J204" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K204" s="2" t="inlineStr"/>
-      <c r="L204" s="2" t="inlineStr"/>
-      <c r="M204" s="2" t="inlineStr"/>
-      <c r="N204" s="2" t="inlineStr"/>
-      <c r="O204" s="2" t="inlineStr"/>
-      <c r="P204" s="2" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q204" s="2" t="inlineStr"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="3" t="inlineStr">
-        <is>
-          <t>Wire harness</t>
-        </is>
-      </c>
-      <c r="B205" s="3" t="inlineStr">
-        <is>
-          <t>All harnesses (master wire list)</t>
-        </is>
-      </c>
-      <c r="C205" s="3" t="inlineStr">
-        <is>
-          <t>pigtail supplied with the sensor (owned)</t>
-        </is>
-      </c>
-      <c r="D205" s="3" t="inlineStr"/>
-      <c r="E205" s="3" t="inlineStr"/>
-      <c r="F205" s="3" t="inlineStr"/>
-      <c r="G205" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H205" s="3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I205" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J205" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K205" s="3" t="inlineStr"/>
-      <c r="L205" s="3" t="inlineStr"/>
-      <c r="M205" s="3" t="inlineStr"/>
-      <c r="N205" s="3" t="inlineStr"/>
-      <c r="O205" s="3" t="inlineStr"/>
-      <c r="P205" s="3" t="inlineStr">
-        <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q205" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q205"/>
+  <autoFilter ref="A1:Q199"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -20927,16 +20537,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Ground studs EA / EB on Route 17 at their factory spots; their wire lengths from the tree (Rev N, Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4492.35</v>
+        <v>4550.26</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4930.21</v>
+        <v>4988.12</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -12550,7 +12550,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -12561,7 +12561,7 @@
         <v>0</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
@@ -12575,7 +12575,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>3.2 m in the master + 15% margin</t>
+          <t>4.3 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -12937,7 +12937,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>3.1 m of bundle + 10 % cut / recovery margin</t>
+          <t>2.8 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13063,7 +13063,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>7.2 m of bundle + 10 % cut / recovery margin</t>
+          <t>6.4 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13164,7 +13164,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -13175,13 +13175,13 @@
         <v>0</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>5.54</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>55.4</v>
+        <v>60.94</v>
       </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>8.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>9.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13270,7 +13270,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>4.1 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.2 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13302,7 +13302,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13313,13 +13313,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>10.83</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>108.3</v>
+        <v>97.47</v>
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
@@ -13339,7 +13339,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>8.7 m of bundle + 10 % cut / recovery margin</t>
+          <t>7.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -15829,7 +15829,7 @@
         </is>
       </c>
       <c r="G121" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
@@ -15840,13 +15840,13 @@
         <v>0</v>
       </c>
       <c r="J121" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K121" s="3" t="n">
         <v>4.08</v>
       </c>
       <c r="L121" s="3" t="n">
-        <v>32.64</v>
+        <v>48.96</v>
       </c>
       <c r="M121" s="4" t="inlineStr">
         <is>
@@ -15866,7 +15866,7 @@
       </c>
       <c r="Q121" s="3" t="inlineStr">
         <is>
-          <t>1.9 m in the master + 15% margin</t>
+          <t>3.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16024,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16035,13 +16035,13 @@
         <v>0</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>3.56</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>14.24</v>
+        <v>46.28</v>
       </c>
       <c r="M124" s="5" t="inlineStr">
         <is>
@@ -16061,7 +16061,7 @@
       </c>
       <c r="Q124" s="2" t="inlineStr">
         <is>
-          <t>1.0 m in the master + 15% margin</t>
+          <t>3.4 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16162,7 +16162,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -16173,13 +16173,13 @@
         <v>0</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>2.56</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>20.48</v>
+        <v>40.96</v>
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
@@ -16199,7 +16199,7 @@
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>2.0 m in the master + 15% margin</t>
+          <t>4.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16357,7 +16357,7 @@
         </is>
       </c>
       <c r="G129" s="3" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
@@ -16368,13 +16368,13 @@
         <v>0</v>
       </c>
       <c r="J129" s="3" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K129" s="3" t="n">
         <v>1.88</v>
       </c>
       <c r="L129" s="3" t="n">
-        <v>45.12</v>
+        <v>39.48</v>
       </c>
       <c r="M129" s="4" t="inlineStr">
         <is>
@@ -16394,7 +16394,7 @@
       </c>
       <c r="Q129" s="3" t="inlineStr">
         <is>
-          <t>6.3 m in the master + 15% margin</t>
+          <t>5.5 m in the master + 15% margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ground studs EA / EB on Route 17 at their factory spots; their wire lengths from the tree (Rev N, Dan 2026-11-01) (#450)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4492.35</v>
+        <v>4550.26</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4930.21</v>
+        <v>4988.12</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -12550,7 +12550,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -12561,7 +12561,7 @@
         <v>0</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
@@ -12575,7 +12575,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>3.2 m in the master + 15% margin</t>
+          <t>4.3 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -12937,7 +12937,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>3.1 m of bundle + 10 % cut / recovery margin</t>
+          <t>2.8 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13063,7 +13063,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>7.2 m of bundle + 10 % cut / recovery margin</t>
+          <t>6.4 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13164,7 +13164,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -13175,13 +13175,13 @@
         <v>0</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>5.54</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>55.4</v>
+        <v>60.94</v>
       </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>8.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>9.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13270,7 +13270,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>4.1 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.2 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13302,7 +13302,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13313,13 +13313,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>10.83</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>108.3</v>
+        <v>97.47</v>
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
@@ -13339,7 +13339,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>8.7 m of bundle + 10 % cut / recovery margin</t>
+          <t>7.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -15829,7 +15829,7 @@
         </is>
       </c>
       <c r="G121" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
@@ -15840,13 +15840,13 @@
         <v>0</v>
       </c>
       <c r="J121" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K121" s="3" t="n">
         <v>4.08</v>
       </c>
       <c r="L121" s="3" t="n">
-        <v>32.64</v>
+        <v>48.96</v>
       </c>
       <c r="M121" s="4" t="inlineStr">
         <is>
@@ -15866,7 +15866,7 @@
       </c>
       <c r="Q121" s="3" t="inlineStr">
         <is>
-          <t>1.9 m in the master + 15% margin</t>
+          <t>3.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16024,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16035,13 +16035,13 @@
         <v>0</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>3.56</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>14.24</v>
+        <v>46.28</v>
       </c>
       <c r="M124" s="5" t="inlineStr">
         <is>
@@ -16061,7 +16061,7 @@
       </c>
       <c r="Q124" s="2" t="inlineStr">
         <is>
-          <t>1.0 m in the master + 15% margin</t>
+          <t>3.4 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16162,7 +16162,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -16173,13 +16173,13 @@
         <v>0</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>2.56</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>20.48</v>
+        <v>40.96</v>
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
@@ -16199,7 +16199,7 @@
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>2.0 m in the master + 15% margin</t>
+          <t>4.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16357,7 +16357,7 @@
         </is>
       </c>
       <c r="G129" s="3" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
@@ -16368,13 +16368,13 @@
         <v>0</v>
       </c>
       <c r="J129" s="3" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K129" s="3" t="n">
         <v>1.88</v>
       </c>
       <c r="L129" s="3" t="n">
-        <v>45.12</v>
+        <v>39.48</v>
       </c>
       <c r="M129" s="4" t="inlineStr">
         <is>
@@ -16394,7 +16394,7 @@
       </c>
       <c r="Q129" s="3" t="inlineStr">
         <is>
-          <t>6.3 m in the master + 15% margin</t>
+          <t>5.5 m in the master + 15% margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tefzel buy links to Corsa Technic; row 169 waits on the bench test (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aA8s41WDmzkdeUSzti3t8
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4550.26</v>
+        <v>4326.14</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4988.12</v>
+        <v>4764</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -4398,21 +4398,29 @@
       </c>
       <c r="M59" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=432&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-14</t>
         </is>
       </c>
-      <c r="N59" s="3" t="inlineStr"/>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P59" s="3" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4463,21 +4471,29 @@
       </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=429&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N60" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-16</t>
         </is>
       </c>
-      <c r="N60" s="2" t="inlineStr"/>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q60" s="2" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -4528,21 +4544,29 @@
       </c>
       <c r="M61" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=798&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-18</t>
         </is>
       </c>
-      <c r="N61" s="3" t="inlineStr"/>
       <c r="O61" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P61" s="3" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q61" s="3" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4593,21 +4617,29 @@
       </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N62" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-20</t>
         </is>
       </c>
-      <c r="N62" s="2" t="inlineStr"/>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q62" s="2" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -8275,52 +8307,56 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId92"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -15843,25 +15879,29 @@
         <v>12</v>
       </c>
       <c r="K121" s="3" t="n">
-        <v>4.08</v>
+        <v>1.95</v>
       </c>
       <c r="L121" s="3" t="n">
-        <v>48.96</v>
+        <v>23.4</v>
       </c>
       <c r="M121" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=425&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N121" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/10-awg-black-tefzel-wire-m22759-16-10-0-cut-length?variant=40451551199267</t>
         </is>
       </c>
-      <c r="N121" s="3" t="inlineStr"/>
       <c r="O121" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P121" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q121" s="3" t="inlineStr">
@@ -15912,25 +15952,29 @@
         <v>38</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>3.5</v>
+        <v>1.95</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>133</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="M122" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=425&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N122" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/10-awg-red-tefzel-wire-m22759-16-10-2-cut-length?variant=40451119939619</t>
         </is>
       </c>
-      <c r="N122" s="2" t="inlineStr"/>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P122" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q122" s="2" t="inlineStr">
@@ -16038,25 +16082,29 @@
         <v>13</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>3.56</v>
+        <v>1.8</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>46.28</v>
+        <v>23.4</v>
       </c>
       <c r="M124" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=404&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N124" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/12-awg-black-tefzel-wire-m22759-16-12-0-spool?variant=40415052726307</t>
         </is>
       </c>
-      <c r="N124" s="2" t="inlineStr"/>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P124" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q124" s="2" t="inlineStr">
@@ -16107,25 +16155,29 @@
         <v>41</v>
       </c>
       <c r="K125" s="3" t="n">
-        <v>3.56</v>
+        <v>1.8</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>145.96</v>
+        <v>73.8</v>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=404&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N125" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/12-awg-red-tefzel-wire-m22759-16-12-2-spool?variant=40415053152291</t>
         </is>
       </c>
-      <c r="N125" s="3" t="inlineStr"/>
       <c r="O125" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P125" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q125" s="3" t="inlineStr">
@@ -16183,18 +16235,22 @@
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=432&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N126" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/14-awg-black-tefzel-wire-m22759-16-14-0-spool?variant=40415048695843</t>
         </is>
       </c>
-      <c r="N126" s="2" t="inlineStr"/>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
@@ -16252,18 +16308,22 @@
       </c>
       <c r="M127" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=432&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N127" s="4" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-14</t>
         </is>
       </c>
-      <c r="N127" s="3" t="inlineStr"/>
       <c r="O127" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P127" s="3" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q127" s="3" t="inlineStr">
@@ -16378,18 +16438,22 @@
       </c>
       <c r="M129" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=429&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N129" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/16-awg-black-tefzel-wire-m22759-16-16-0-spool?variant=40415046434851</t>
         </is>
       </c>
-      <c r="N129" s="3" t="inlineStr"/>
       <c r="O129" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P129" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q129" s="3" t="inlineStr">
@@ -16447,18 +16511,22 @@
       </c>
       <c r="M130" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=429&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N130" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-16</t>
         </is>
       </c>
-      <c r="N130" s="2" t="inlineStr"/>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P130" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
@@ -16573,18 +16641,22 @@
       </c>
       <c r="M132" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=798&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N132" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-18</t>
         </is>
       </c>
-      <c r="N132" s="2" t="inlineStr"/>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P132" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q132" s="2" t="inlineStr">
@@ -16642,18 +16714,22 @@
       </c>
       <c r="M133" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=798&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N133" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/18-awg-white-tefzel-wire-m22759-16-18-9-spool?variant=40415044829219</t>
         </is>
       </c>
-      <c r="N133" s="3" t="inlineStr"/>
       <c r="O133" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P133" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q133" s="3" t="inlineStr">
@@ -16711,18 +16787,22 @@
       </c>
       <c r="M134" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N134" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-20</t>
         </is>
       </c>
-      <c r="N134" s="2" t="inlineStr"/>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q134" s="2" t="inlineStr">
@@ -16780,18 +16860,22 @@
       </c>
       <c r="M135" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N135" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-orange-tefzel-wire-m22759-16-20-3-spool?variant=40415028019235</t>
         </is>
       </c>
-      <c r="N135" s="3" t="inlineStr"/>
       <c r="O135" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P135" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q135" s="3" t="inlineStr">
@@ -16849,18 +16933,22 @@
       </c>
       <c r="M136" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N136" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-yellow-tefzel-wire-m22759-16-20-4-spool?variant=40415028477987</t>
         </is>
       </c>
-      <c r="N136" s="2" t="inlineStr"/>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P136" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q136" s="2" t="inlineStr">
@@ -16918,18 +17006,22 @@
       </c>
       <c r="M137" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N137" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-green-tefzel-wire-m22759-16-20-5-spool?variant=40415028838435</t>
         </is>
       </c>
-      <c r="N137" s="3" t="inlineStr"/>
       <c r="O137" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P137" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q137" s="3" t="inlineStr">
@@ -16987,18 +17079,22 @@
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N138" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-blue-tefzel-wire-m22759-16-20-6-spool?variant=40415028903971</t>
         </is>
       </c>
-      <c r="N138" s="2" t="inlineStr"/>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P138" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q138" s="2" t="inlineStr">
@@ -17056,7 +17152,7 @@
       </c>
       <c r="M139" s="4" t="inlineStr">
         <is>
-          <t>https://www.ksvlooms.com/products/20-awg-white-tefzel-wire-m22759-16-20-9-spool?variant=40415029297187</t>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
         </is>
       </c>
       <c r="N139" s="4" t="inlineStr">
@@ -17066,12 +17162,12 @@
       </c>
       <c r="O139" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P139" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q139" s="3" t="inlineStr">
@@ -17122,25 +17218,29 @@
         <v>9</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>6.08</v>
+        <v>3.86</v>
       </c>
       <c r="L140" s="2" t="n">
-        <v>54.72</v>
+        <v>34.74</v>
       </c>
       <c r="M140" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=2454&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N140" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/8-awg-black-tefzel-wire-m22759-16-8-0-cut-length?variant=40451555557411</t>
         </is>
       </c>
-      <c r="N140" s="2" t="inlineStr"/>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P140" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q140" s="2" t="inlineStr">
@@ -17191,25 +17291,29 @@
         <v>11</v>
       </c>
       <c r="K141" s="3" t="n">
-        <v>6.1</v>
+        <v>3.86</v>
       </c>
       <c r="L141" s="3" t="n">
-        <v>67.09999999999999</v>
+        <v>42.46</v>
       </c>
       <c r="M141" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=2454&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N141" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/8-awg-red-tefzel-wire-m22759-16-8-2-cut-length?variant=40451557523491</t>
         </is>
       </c>
-      <c r="N141" s="3" t="inlineStr"/>
       <c r="O141" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P141" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q141" s="3" t="inlineStr">
@@ -20758,36 +20862,53 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N139" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N121" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N122" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N124" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N125" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N126" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N127" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N129" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N130" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N132" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N133" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N134" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N135" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N136" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N137" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N138" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N139" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N140" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N141" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId126"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Tefzel buy links to Corsa Technic; row 169 waits on the bench test (Dan 2026-11-01) (#458)
Claude-Session: https://claude.ai/code/session_014aA8s41WDmzkdeUSzti3t8

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4550.26</v>
+        <v>4326.14</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4988.12</v>
+        <v>4764</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -4398,21 +4398,29 @@
       </c>
       <c r="M59" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=432&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-14</t>
         </is>
       </c>
-      <c r="N59" s="3" t="inlineStr"/>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P59" s="3" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4463,21 +4471,29 @@
       </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=429&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N60" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-16</t>
         </is>
       </c>
-      <c r="N60" s="2" t="inlineStr"/>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q60" s="2" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -4528,21 +4544,29 @@
       </c>
       <c r="M61" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=798&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-18</t>
         </is>
       </c>
-      <c r="N61" s="3" t="inlineStr"/>
       <c r="O61" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P61" s="3" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q61" s="3" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4593,21 +4617,29 @@
       </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N62" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-20</t>
         </is>
       </c>
-      <c r="N62" s="2" t="inlineStr"/>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
-        </is>
-      </c>
-      <c r="Q62" s="2" t="inlineStr"/>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>preferred Tefzel supplier (Dan 2026-11-01)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -8275,52 +8307,56 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId92"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -15843,25 +15879,29 @@
         <v>12</v>
       </c>
       <c r="K121" s="3" t="n">
-        <v>4.08</v>
+        <v>1.95</v>
       </c>
       <c r="L121" s="3" t="n">
-        <v>48.96</v>
+        <v>23.4</v>
       </c>
       <c r="M121" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=425&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N121" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/10-awg-black-tefzel-wire-m22759-16-10-0-cut-length?variant=40451551199267</t>
         </is>
       </c>
-      <c r="N121" s="3" t="inlineStr"/>
       <c r="O121" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P121" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q121" s="3" t="inlineStr">
@@ -15912,25 +15952,29 @@
         <v>38</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>3.5</v>
+        <v>1.95</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>133</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="M122" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=425&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N122" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/10-awg-red-tefzel-wire-m22759-16-10-2-cut-length?variant=40451119939619</t>
         </is>
       </c>
-      <c r="N122" s="2" t="inlineStr"/>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P122" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q122" s="2" t="inlineStr">
@@ -16038,25 +16082,29 @@
         <v>13</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>3.56</v>
+        <v>1.8</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>46.28</v>
+        <v>23.4</v>
       </c>
       <c r="M124" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=404&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N124" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/12-awg-black-tefzel-wire-m22759-16-12-0-spool?variant=40415052726307</t>
         </is>
       </c>
-      <c r="N124" s="2" t="inlineStr"/>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P124" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q124" s="2" t="inlineStr">
@@ -16107,25 +16155,29 @@
         <v>41</v>
       </c>
       <c r="K125" s="3" t="n">
-        <v>3.56</v>
+        <v>1.8</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>145.96</v>
+        <v>73.8</v>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=404&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N125" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/12-awg-red-tefzel-wire-m22759-16-12-2-spool?variant=40415053152291</t>
         </is>
       </c>
-      <c r="N125" s="3" t="inlineStr"/>
       <c r="O125" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P125" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q125" s="3" t="inlineStr">
@@ -16183,18 +16235,22 @@
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=432&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N126" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/14-awg-black-tefzel-wire-m22759-16-14-0-spool?variant=40415048695843</t>
         </is>
       </c>
-      <c r="N126" s="2" t="inlineStr"/>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
@@ -16252,18 +16308,22 @@
       </c>
       <c r="M127" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=432&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N127" s="4" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-14</t>
         </is>
       </c>
-      <c r="N127" s="3" t="inlineStr"/>
       <c r="O127" s="3" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P127" s="3" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q127" s="3" t="inlineStr">
@@ -16378,18 +16438,22 @@
       </c>
       <c r="M129" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=429&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N129" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/16-awg-black-tefzel-wire-m22759-16-16-0-spool?variant=40415046434851</t>
         </is>
       </c>
-      <c r="N129" s="3" t="inlineStr"/>
       <c r="O129" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P129" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q129" s="3" t="inlineStr">
@@ -16447,18 +16511,22 @@
       </c>
       <c r="M130" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=429&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N130" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-16</t>
         </is>
       </c>
-      <c r="N130" s="2" t="inlineStr"/>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P130" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
@@ -16573,18 +16641,22 @@
       </c>
       <c r="M132" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=798&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N132" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-18</t>
         </is>
       </c>
-      <c r="N132" s="2" t="inlineStr"/>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P132" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q132" s="2" t="inlineStr">
@@ -16642,18 +16714,22 @@
       </c>
       <c r="M133" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=798&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N133" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/18-awg-white-tefzel-wire-m22759-16-18-9-spool?variant=40415044829219</t>
         </is>
       </c>
-      <c r="N133" s="3" t="inlineStr"/>
       <c r="O133" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P133" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q133" s="3" t="inlineStr">
@@ -16711,18 +16787,22 @@
       </c>
       <c r="M134" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N134" s="5" t="inlineStr">
+        <is>
           <t>https://www.awcwire.com/product/m22759_16-20</t>
         </is>
       </c>
-      <c r="N134" s="2" t="inlineStr"/>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>est</t>
+          <t>est; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr">
         <is>
-          <t>from cad/fusebox parts list (R82 checked)</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q134" s="2" t="inlineStr">
@@ -16780,18 +16860,22 @@
       </c>
       <c r="M135" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N135" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-orange-tefzel-wire-m22759-16-20-3-spool?variant=40415028019235</t>
         </is>
       </c>
-      <c r="N135" s="3" t="inlineStr"/>
       <c r="O135" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P135" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q135" s="3" t="inlineStr">
@@ -16849,18 +16933,22 @@
       </c>
       <c r="M136" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N136" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-yellow-tefzel-wire-m22759-16-20-4-spool?variant=40415028477987</t>
         </is>
       </c>
-      <c r="N136" s="2" t="inlineStr"/>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P136" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q136" s="2" t="inlineStr">
@@ -16918,18 +17006,22 @@
       </c>
       <c r="M137" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N137" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-green-tefzel-wire-m22759-16-20-5-spool?variant=40415028838435</t>
         </is>
       </c>
-      <c r="N137" s="3" t="inlineStr"/>
       <c r="O137" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P137" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q137" s="3" t="inlineStr">
@@ -16987,18 +17079,22 @@
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N138" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/20-awg-blue-tefzel-wire-m22759-16-20-6-spool?variant=40415028903971</t>
         </is>
       </c>
-      <c r="N138" s="2" t="inlineStr"/>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P138" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q138" s="2" t="inlineStr">
@@ -17056,7 +17152,7 @@
       </c>
       <c r="M139" s="4" t="inlineStr">
         <is>
-          <t>https://www.ksvlooms.com/products/20-awg-white-tefzel-wire-m22759-16-20-9-spool?variant=40415029297187</t>
+          <t>https://www.corsa-technic.com/item.php?item_id=381&amp;category_id=62</t>
         </is>
       </c>
       <c r="N139" s="4" t="inlineStr">
@@ -17066,12 +17162,12 @@
       </c>
       <c r="O139" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>KSV Looms, 2026-10-20; Corsa base price not shown on its page (only %% breaks), old price kept</t>
         </is>
       </c>
       <c r="P139" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q139" s="3" t="inlineStr">
@@ -17122,25 +17218,29 @@
         <v>9</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>6.08</v>
+        <v>3.86</v>
       </c>
       <c r="L140" s="2" t="n">
-        <v>54.72</v>
+        <v>34.74</v>
       </c>
       <c r="M140" s="5" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=2454&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N140" s="5" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/8-awg-black-tefzel-wire-m22759-16-8-0-cut-length?variant=40451555557411</t>
         </is>
       </c>
-      <c r="N140" s="2" t="inlineStr"/>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P140" s="2" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q140" s="2" t="inlineStr">
@@ -17191,25 +17291,29 @@
         <v>11</v>
       </c>
       <c r="K141" s="3" t="n">
-        <v>6.1</v>
+        <v>3.86</v>
       </c>
       <c r="L141" s="3" t="n">
-        <v>67.09999999999999</v>
+        <v>42.46</v>
       </c>
       <c r="M141" s="4" t="inlineStr">
         <is>
+          <t>https://www.corsa-technic.com/item.php?item_id=2454&amp;category_id=62</t>
+        </is>
+      </c>
+      <c r="N141" s="4" t="inlineStr">
+        <is>
           <t>https://www.ksvlooms.com/products/8-awg-red-tefzel-wire-m22759-16-8-2-cut-length?variant=40451557523491</t>
         </is>
       </c>
-      <c r="N141" s="3" t="inlineStr"/>
       <c r="O141" s="3" t="inlineStr">
         <is>
-          <t>KSV Looms, 2026-10-20</t>
+          <t>Corsa Technic per ft, 1-99 ft, 2026-11-01</t>
         </is>
       </c>
       <c r="P141" s="3" t="inlineStr">
         <is>
-          <t>vendor page read 2026-10-20 (products.json), in stock</t>
+          <t>Corsa Technic category page read 2026-11-01 (colour picked on the page)</t>
         </is>
       </c>
       <c r="Q141" s="3" t="inlineStr">
@@ -20758,36 +20862,53 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N139" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N121" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N122" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N124" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N125" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N126" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N127" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N129" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N130" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N132" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N133" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N134" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N135" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N136" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N137" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N138" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N139" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N140" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N141" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId126"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Gearbox speed sensor: plain wires, no shield (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4326.14</v>
+        <v>4308.88</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4764</v>
+        <v>4746.74</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -8701,7 +8701,7 @@
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -8709,7 +8709,7 @@
         </is>
       </c>
       <c r="I5" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>0</v>
@@ -8959,7 +8959,7 @@
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -8967,7 +8967,7 @@
         </is>
       </c>
       <c r="I9" s="3" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>0</v>
@@ -9396,7 +9396,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -9407,13 +9407,13 @@
         <v>0</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0.22</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>12.76</v>
+        <v>13.2</v>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -11565,7 +11565,7 @@
         <v>0</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
@@ -11583,7 +11583,7 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>7 cable runs, 7.8 m + 15% margin</t>
+          <t>6 cable runs, 6.5 m + 15% margin</t>
         </is>
       </c>
     </row>
@@ -12936,7 +12936,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -12947,13 +12947,13 @@
         <v>0</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>20.08</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>80.31999999999999</v>
+        <v>60.24</v>
       </c>
       <c r="M74" s="5" t="inlineStr">
         <is>
@@ -12973,7 +12973,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>2.8 m of bundle + 10 % cut / recovery margin</t>
+          <t>2.7 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13062,7 +13062,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -13073,13 +13073,13 @@
         <v>0</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>14.24</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>113.92</v>
+        <v>99.68000000000001</v>
       </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>6.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.9 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13200,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -13211,13 +13211,13 @@
         <v>0</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>5.54</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>60.94</v>
+        <v>66.48</v>
       </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
@@ -13237,7 +13237,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>9.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>10.0 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13306,7 +13306,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>4.2 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.3 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -16839,7 +16839,7 @@
         </is>
       </c>
       <c r="G135" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
@@ -16850,13 +16850,13 @@
         <v>0</v>
       </c>
       <c r="J135" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="K135" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="L135" s="3" t="n">
-        <v>18.72</v>
+        <v>23.92</v>
       </c>
       <c r="M135" s="4" t="inlineStr">
         <is>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="Q135" s="3" t="inlineStr">
         <is>
-          <t>4.7 m in the master + 15% margin</t>
+          <t>6.1 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17058,7 +17058,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -17069,13 +17069,13 @@
         <v>0</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K138" s="2" t="n">
         <v>1.08</v>
       </c>
       <c r="L138" s="2" t="n">
-        <v>35.64</v>
+        <v>36.72</v>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
@@ -17099,7 +17099,7 @@
       </c>
       <c r="Q138" s="2" t="inlineStr">
         <is>
-          <t>8.5 m in the master + 15% margin</t>
+          <t>9.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17131,7 +17131,7 @@
         </is>
       </c>
       <c r="G139" s="3" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
@@ -17142,13 +17142,13 @@
         <v>0</v>
       </c>
       <c r="J139" s="3" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="K139" s="3" t="n">
         <v>0.96</v>
       </c>
       <c r="L139" s="3" t="n">
-        <v>77.76000000000001</v>
+        <v>82.56</v>
       </c>
       <c r="M139" s="4" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
       </c>
       <c r="Q139" s="3" t="inlineStr">
         <is>
-          <t>21.2 m in the master + 15% margin</t>
+          <t>22.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gearbox speed sensor: plain wires, no shield (Dan 2026-11-01) (#461)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="To do" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanical assemblies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire harness" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4326.14</v>
+        <v>4308.88</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4764</v>
+        <v>4746.74</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -8701,7 +8701,7 @@
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -8709,7 +8709,7 @@
         </is>
       </c>
       <c r="I5" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>0</v>
@@ -8959,7 +8959,7 @@
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -8967,7 +8967,7 @@
         </is>
       </c>
       <c r="I9" s="3" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>0</v>
@@ -9396,7 +9396,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -9407,13 +9407,13 @@
         <v>0</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0.22</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>12.76</v>
+        <v>13.2</v>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -11565,7 +11565,7 @@
         <v>0</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
@@ -11583,7 +11583,7 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>7 cable runs, 7.8 m + 15% margin</t>
+          <t>6 cable runs, 6.5 m + 15% margin</t>
         </is>
       </c>
     </row>
@@ -12936,7 +12936,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -12947,13 +12947,13 @@
         <v>0</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>20.08</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>80.31999999999999</v>
+        <v>60.24</v>
       </c>
       <c r="M74" s="5" t="inlineStr">
         <is>
@@ -12973,7 +12973,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>2.8 m of bundle + 10 % cut / recovery margin</t>
+          <t>2.7 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13062,7 +13062,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -13073,13 +13073,13 @@
         <v>0</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>14.24</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>113.92</v>
+        <v>99.68000000000001</v>
       </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>6.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.9 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13200,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -13211,13 +13211,13 @@
         <v>0</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>5.54</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>60.94</v>
+        <v>66.48</v>
       </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
@@ -13237,7 +13237,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>9.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>10.0 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13306,7 +13306,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>4.2 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.3 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -16839,7 +16839,7 @@
         </is>
       </c>
       <c r="G135" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
@@ -16850,13 +16850,13 @@
         <v>0</v>
       </c>
       <c r="J135" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="K135" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="L135" s="3" t="n">
-        <v>18.72</v>
+        <v>23.92</v>
       </c>
       <c r="M135" s="4" t="inlineStr">
         <is>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="Q135" s="3" t="inlineStr">
         <is>
-          <t>4.7 m in the master + 15% margin</t>
+          <t>6.1 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17058,7 +17058,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -17069,13 +17069,13 @@
         <v>0</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K138" s="2" t="n">
         <v>1.08</v>
       </c>
       <c r="L138" s="2" t="n">
-        <v>35.64</v>
+        <v>36.72</v>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
@@ -17099,7 +17099,7 @@
       </c>
       <c r="Q138" s="2" t="inlineStr">
         <is>
-          <t>8.5 m in the master + 15% margin</t>
+          <t>9.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17131,7 +17131,7 @@
         </is>
       </c>
       <c r="G139" s="3" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
@@ -17142,13 +17142,13 @@
         <v>0</v>
       </c>
       <c r="J139" s="3" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="K139" s="3" t="n">
         <v>0.96</v>
       </c>
       <c r="L139" s="3" t="n">
-        <v>77.76000000000001</v>
+        <v>82.56</v>
       </c>
       <c r="M139" s="4" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
       </c>
       <c r="Q139" s="3" t="inlineStr">
         <is>
-          <t>21.2 m in the master + 15% margin</t>
+          <t>22.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harness C from Dan's placement; front side marker lamps; EB on its factory bolt
- Route 17 rebuilt from Dan's harness C placement (lines, spots, picture, tables)
- Master: LH / RH front side marker lamps (F5 / F6) off SP-CLR, grounds to EB / EA
- EB on the factory bolt (EWD p.36) via a short front-run stub; block strap lands as lug GND-EB-2
- Route 16 devices 18 / H1 keep only HeavyDC ends; harness C owns its own block-stud and alternator-plug spots
- EngineRoom-C lengths from the tree; wire lists, pin chart, BOM regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$204</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,16 +540,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4308.88</v>
+        <v>4373.57</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4746.74</v>
+        <v>4811.43</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -8369,7 +8369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q204"/>
+  <dimension ref="A1:Q205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12586,7 +12586,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -12597,7 +12597,7 @@
         <v>0</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
@@ -12611,7 +12611,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>4.3 m in the master + 15% margin</t>
+          <t>0.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>5.9 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13168,7 +13168,7 @@
       </c>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>5.1 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.4 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13249,7 +13249,7 @@
         </is>
       </c>
       <c r="G79" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -13260,13 +13260,13 @@
         <v>0</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K79" s="3" t="n">
         <v>5.54</v>
       </c>
       <c r="L79" s="3" t="n">
-        <v>66.48</v>
+        <v>72.02</v>
       </c>
       <c r="M79" s="4" t="inlineStr">
         <is>
@@ -13286,7 +13286,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>10.0 m of bundle + 10 % cut / recovery margin</t>
+          <t>11.1 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13318,7 +13318,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13329,13 +13329,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>14.99</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>74.95</v>
+        <v>89.94</v>
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
@@ -13355,7 +13355,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>4.3 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.6 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>7.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>8.0 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -15234,7 +15234,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -15245,7 +15245,7 @@
         <v>0</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr"/>
@@ -15259,7 +15259,7 @@
       </c>
       <c r="Q110" s="2" t="inlineStr">
         <is>
-          <t>14.4 m in the master + 15% margin</t>
+          <t>14.3 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15348,7 +15348,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -15359,7 +15359,7 @@
         <v>0</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K112" s="2" t="inlineStr"/>
       <c r="L112" s="2" t="inlineStr"/>
@@ -15373,7 +15373,7 @@
       </c>
       <c r="Q112" s="2" t="inlineStr">
         <is>
-          <t>12.2 m in the master + 15% margin</t>
+          <t>12.4 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15633,7 +15633,7 @@
         </is>
       </c>
       <c r="G117" s="3" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
@@ -15644,7 +15644,7 @@
         <v>0</v>
       </c>
       <c r="J117" s="3" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="K117" s="3" t="inlineStr"/>
       <c r="L117" s="3" t="inlineStr"/>
@@ -15658,7 +15658,7 @@
       </c>
       <c r="Q117" s="3" t="inlineStr">
         <is>
-          <t>24.5 m in the master + 15% margin</t>
+          <t>24.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15914,7 +15914,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -15925,13 +15925,13 @@
         <v>0</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>1.95</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>23.4</v>
+        <v>31.2</v>
       </c>
       <c r="M122" s="5" t="inlineStr">
         <is>
@@ -15955,7 +15955,7 @@
       </c>
       <c r="Q122" s="2" t="inlineStr">
         <is>
-          <t>3.2 m in the master + 15% margin</t>
+          <t>4.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15987,7 +15987,7 @@
         </is>
       </c>
       <c r="G123" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
@@ -15998,13 +15998,13 @@
         <v>0</v>
       </c>
       <c r="J123" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K123" s="3" t="n">
         <v>1.95</v>
       </c>
       <c r="L123" s="3" t="n">
-        <v>74.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="M123" s="4" t="inlineStr">
         <is>
@@ -16028,7 +16028,7 @@
       </c>
       <c r="Q123" s="3" t="inlineStr">
         <is>
-          <t>9.8 m in the master + 15% margin</t>
+          <t>10.4 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
         </is>
       </c>
       <c r="G125" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
@@ -16128,13 +16128,13 @@
         <v>0</v>
       </c>
       <c r="J125" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K125" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>23.4</v>
+        <v>25.2</v>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>3.4 m in the master + 15% margin</t>
+          <t>3.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16190,7 +16190,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -16201,13 +16201,13 @@
         <v>0</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>1.8</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>73.8</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
@@ -16231,7 +16231,7 @@
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>10.7 m in the master + 15% margin</t>
+          <t>10.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16304,7 +16304,7 @@
       </c>
       <c r="Q127" s="3" t="inlineStr">
         <is>
-          <t>4.0 m in the master + 15% margin</t>
+          <t>4.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16336,7 +16336,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -16347,13 +16347,13 @@
         <v>0</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="K128" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L128" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="M128" s="5" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
       </c>
       <c r="Q128" s="2" t="inlineStr">
         <is>
-          <t>22.4 m in the master + 15% margin</t>
+          <t>21.7 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16434,7 +16434,7 @@
       </c>
       <c r="Q129" s="3" t="inlineStr">
         <is>
-          <t>1.0 m in the master + 15% margin</t>
+          <t>0.8 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16466,7 +16466,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -16477,13 +16477,13 @@
         <v>0</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K130" s="2" t="n">
         <v>1.88</v>
       </c>
       <c r="L130" s="2" t="n">
-        <v>39.48</v>
+        <v>50.76</v>
       </c>
       <c r="M130" s="5" t="inlineStr">
         <is>
@@ -16507,7 +16507,7 @@
       </c>
       <c r="Q130" s="2" t="inlineStr">
         <is>
-          <t>5.5 m in the master + 15% margin</t>
+          <t>7.1 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16539,7 +16539,7 @@
         </is>
       </c>
       <c r="G131" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
@@ -16550,13 +16550,13 @@
         <v>0</v>
       </c>
       <c r="J131" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="K131" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L131" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="M131" s="4" t="inlineStr">
         <is>
@@ -16580,7 +16580,7 @@
       </c>
       <c r="Q131" s="3" t="inlineStr">
         <is>
-          <t>29.2 m in the master + 15% margin</t>
+          <t>31.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17253,7 +17253,7 @@
         </is>
       </c>
       <c r="G141" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
@@ -17264,13 +17264,13 @@
         <v>0</v>
       </c>
       <c r="J141" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K141" s="3" t="n">
         <v>3.86</v>
       </c>
       <c r="L141" s="3" t="n">
-        <v>34.74</v>
+        <v>27.02</v>
       </c>
       <c r="M141" s="4" t="inlineStr">
         <is>
@@ -17294,7 +17294,7 @@
       </c>
       <c r="Q141" s="3" t="inlineStr">
         <is>
-          <t>2.1 m in the master + 15% margin</t>
+          <t>1.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17326,7 +17326,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -17337,13 +17337,13 @@
         <v>0</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K142" s="2" t="n">
         <v>3.86</v>
       </c>
       <c r="L142" s="2" t="n">
-        <v>42.46</v>
+        <v>61.76</v>
       </c>
       <c r="M142" s="5" t="inlineStr">
         <is>
@@ -17367,7 +17367,7 @@
       </c>
       <c r="Q142" s="2" t="inlineStr">
         <is>
-          <t>2.8 m in the master + 15% margin</t>
+          <t>4.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -18797,7 +18797,7 @@
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K169" s="3" t="inlineStr"/>
       <c r="L169" s="3" t="inlineStr"/>
@@ -18899,11 +18899,11 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
@@ -18914,7 +18914,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K171" s="3" t="inlineStr"/>
       <c r="L171" s="3" t="inlineStr"/>
@@ -18952,11 +18952,11 @@
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18967,7 +18967,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K172" s="2" t="inlineStr"/>
       <c r="L172" s="2" t="inlineStr"/>
@@ -19005,7 +19005,7 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
@@ -19058,11 +19058,11 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -19073,7 +19073,7 @@
         <v>0</v>
       </c>
       <c r="J174" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K174" s="2" t="inlineStr"/>
       <c r="L174" s="2" t="inlineStr"/>
@@ -19111,7 +19111,7 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
@@ -19164,11 +19164,11 @@
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -19179,7 +19179,7 @@
         <v>0</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K176" s="2" t="inlineStr"/>
       <c r="L176" s="2" t="inlineStr"/>
@@ -19217,7 +19217,7 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
@@ -19270,7 +19270,7 @@
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
@@ -19323,7 +19323,7 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
@@ -19376,7 +19376,7 @@
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19429,7 +19429,7 @@
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G181" s="3" t="n">
@@ -19482,7 +19482,7 @@
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G182" s="2" t="n">
@@ -19535,7 +19535,7 @@
       <c r="E183" s="3" t="inlineStr"/>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
@@ -19588,7 +19588,7 @@
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G184" s="2" t="n">
@@ -19641,7 +19641,7 @@
       <c r="E185" s="3" t="inlineStr"/>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G185" s="3" t="n">
@@ -19687,22 +19687,18 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr"/>
       <c r="E186" s="2" t="inlineStr"/>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -19713,27 +19709,23 @@
         <v>0</v>
       </c>
       <c r="J186" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K186" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L186" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr"/>
       <c r="M186" s="2" t="inlineStr"/>
       <c r="N186" s="2" t="inlineStr"/>
-      <c r="O186" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O186" s="2" t="inlineStr"/>
       <c r="P186" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
-        </is>
-      </c>
-      <c r="Q186" s="2" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="inlineStr">
+        <is>
+          <t>no maker document in the repo yet; never guessed</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -19748,7 +19740,7 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>TMS-SCE-1/2-2.0-9</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -19759,11 +19751,11 @@
       <c r="E187" s="3" t="inlineStr"/>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G187" s="3" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
@@ -19774,7 +19766,7 @@
         <v>0</v>
       </c>
       <c r="J187" s="3" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="K187" s="3" t="n">
         <v>0</v>
@@ -19809,7 +19801,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>TMS-SCE-3/16-2.0-9</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -19820,11 +19812,11 @@
       <c r="E188" s="2" t="inlineStr"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -19835,7 +19827,7 @@
         <v>0</v>
       </c>
       <c r="J188" s="2" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="K188" s="2" t="n">
         <v>0</v>
@@ -19870,22 +19862,22 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>TMS-SCE-3/8-2.0-9</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
+          <t>TE Connectivity (Raychem)</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr"/>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G189" s="3" t="n">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
@@ -19893,31 +19885,27 @@
         </is>
       </c>
       <c r="I189" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J189" s="3" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="K189" s="3" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L189" s="3" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="M189" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M189" s="3" t="inlineStr"/>
       <c r="N189" s="3" t="inlineStr"/>
       <c r="O189" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>not priced (Dan)</t>
         </is>
       </c>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="Q189" s="3" t="inlineStr"/>
@@ -19935,58 +19923,54 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>W12S</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
+          <t>Deutsch (TE Connectivity)</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr"/>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G190" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H190" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I190" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="J190" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K190" s="2" t="n">
-        <v>0.13</v>
+        <v>0.42</v>
       </c>
       <c r="L190" s="2" t="n">
-        <v>0.26</v>
+        <v>1.26</v>
       </c>
       <c r="M190" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
         </is>
       </c>
       <c r="N190" s="2" t="inlineStr"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr"/>
@@ -20004,7 +19988,7 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>W2P</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -20019,11 +20003,11 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G191" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
@@ -20034,28 +20018,28 @@
         <v>0</v>
       </c>
       <c r="J191" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K191" s="3" t="n">
         <v>0.13</v>
       </c>
       <c r="L191" s="3" t="n">
-        <v>1.3</v>
+        <v>0.26</v>
       </c>
       <c r="M191" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="N191" s="3" t="inlineStr"/>
       <c r="O191" s="3" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1, 2026-10-19</t>
         </is>
       </c>
       <c r="P191" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q191" s="3" t="inlineStr"/>
@@ -20073,12 +20057,12 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>W3P</t>
+          <t>W2S</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
@@ -20088,11 +20072,11 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -20103,17 +20087,17 @@
         <v>0</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K192" s="2" t="n">
         <v>0.13</v>
       </c>
       <c r="L192" s="2" t="n">
-        <v>0.13</v>
+        <v>1.3</v>
       </c>
       <c r="M192" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3P.html</t>
+          <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="N192" s="2" t="inlineStr"/>
@@ -20142,7 +20126,7 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>W3P</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -20157,11 +20141,11 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
         </is>
       </c>
       <c r="G193" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H193" s="3" t="inlineStr">
         <is>
@@ -20172,17 +20156,17 @@
         <v>0</v>
       </c>
       <c r="J193" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K193" s="3" t="n">
         <v>0.13</v>
       </c>
       <c r="L193" s="3" t="n">
-        <v>0.39</v>
+        <v>0.13</v>
       </c>
       <c r="M193" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
+          <t>https://www.te.com/en/product-W3P.html</t>
         </is>
       </c>
       <c r="N193" s="3" t="inlineStr"/>
@@ -20193,7 +20177,7 @@
       </c>
       <c r="P193" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q193" s="3" t="inlineStr"/>
@@ -20211,12 +20195,12 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
+          <t>Deutsch</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
@@ -20226,11 +20210,11 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -20241,28 +20225,28 @@
         <v>0</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K194" s="2" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="L194" s="2" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="M194" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+          <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="N194" s="2" t="inlineStr"/>
       <c r="O194" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q194" s="2" t="inlineStr"/>
@@ -20280,7 +20264,7 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -20295,7 +20279,7 @@
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G195" s="3" t="n">
@@ -20313,14 +20297,14 @@
         <v>2</v>
       </c>
       <c r="K195" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="L195" s="3" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="M195" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
         </is>
       </c>
       <c r="N195" s="3" t="inlineStr"/>
@@ -20331,7 +20315,7 @@
       </c>
       <c r="P195" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q195" s="3" t="inlineStr"/>
@@ -20349,7 +20333,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -20364,11 +20348,11 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -20379,28 +20363,28 @@
         <v>0</v>
       </c>
       <c r="J196" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K196" s="2" t="n">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="L196" s="2" t="n">
-        <v>0.35</v>
+        <v>0.42</v>
       </c>
       <c r="M196" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N196" s="2" t="inlineStr"/>
       <c r="O196" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q196" s="2" t="inlineStr"/>
@@ -20418,7 +20402,7 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>WM-4S</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -20433,7 +20417,7 @@
       </c>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G197" s="3" t="n">
@@ -20451,14 +20435,14 @@
         <v>1</v>
       </c>
       <c r="K197" s="3" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="L197" s="3" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="M197" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N197" s="3" t="inlineStr"/>
@@ -20469,7 +20453,7 @@
       </c>
       <c r="P197" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
         </is>
       </c>
       <c r="Q197" s="3" t="inlineStr"/>
@@ -20487,12 +20471,12 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>WM-6S</t>
+          <t>WM-4S</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -20502,7 +20486,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
         </is>
       </c>
       <c r="G198" s="2" t="n">
@@ -20520,14 +20504,14 @@
         <v>1</v>
       </c>
       <c r="K198" s="2" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="L198" s="2" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="M198" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
         </is>
       </c>
       <c r="N198" s="2" t="inlineStr"/>
@@ -20538,7 +20522,7 @@
       </c>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
         </is>
       </c>
       <c r="Q198" s="2" t="inlineStr"/>
@@ -20556,14 +20540,26 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>in kit 354404</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="inlineStr"/>
-      <c r="E199" s="3" t="inlineStr"/>
-      <c r="F199" s="3" t="inlineStr"/>
+          <t>WM-6S</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+        </is>
+      </c>
       <c r="G199" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
@@ -20571,26 +20567,34 @@
         </is>
       </c>
       <c r="I199" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J199" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K199" s="3" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr"/>
-      <c r="M199" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K199" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="L199" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="M199" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+        </is>
+      </c>
       <c r="N199" s="3" t="inlineStr"/>
-      <c r="O199" s="3" t="inlineStr"/>
+      <c r="O199" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+        </is>
+      </c>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q199" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
+          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
+        </is>
+      </c>
+      <c r="Q199" s="3" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -20605,14 +20609,14 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>in kit CONN-75800</t>
+          <t>in kit 354404</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr"/>
       <c r="E200" s="2" t="inlineStr"/>
       <c r="F200" s="2" t="inlineStr"/>
       <c r="G200" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -20620,7 +20624,7 @@
         </is>
       </c>
       <c r="I200" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J200" s="2" t="n">
         <v>0</v>
@@ -20654,14 +20658,14 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr"/>
       <c r="E201" s="3" t="inlineStr"/>
       <c r="F201" s="3" t="inlineStr"/>
       <c r="G201" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
@@ -20669,10 +20673,10 @@
         </is>
       </c>
       <c r="I201" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J201" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K201" s="3" t="inlineStr"/>
       <c r="L201" s="3" t="inlineStr"/>
@@ -20684,7 +20688,11 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q201" s="3" t="inlineStr"/>
+      <c r="Q201" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -20699,14 +20707,14 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>in kit CONN-76270</t>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr"/>
       <c r="E202" s="2" t="inlineStr"/>
       <c r="F202" s="2" t="inlineStr"/>
       <c r="G202" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -20714,10 +20722,10 @@
         </is>
       </c>
       <c r="I202" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J202" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
       <c r="L202" s="2" t="inlineStr"/>
@@ -20729,11 +20737,7 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q202" s="2" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
+      <c r="Q202" s="2" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -20748,14 +20752,14 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>in kit D 261 205 358-01</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr"/>
       <c r="E203" s="3" t="inlineStr"/>
       <c r="F203" s="3" t="inlineStr"/>
       <c r="G203" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
@@ -20763,10 +20767,10 @@
         </is>
       </c>
       <c r="I203" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J203" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K203" s="3" t="inlineStr"/>
       <c r="L203" s="3" t="inlineStr"/>
@@ -20778,7 +20782,11 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q203" s="3" t="inlineStr"/>
+      <c r="Q203" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -20793,14 +20801,14 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>pigtail supplied with the sensor (owned)</t>
+          <t>in kit D 261 205 358-01</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr"/>
       <c r="E204" s="2" t="inlineStr"/>
       <c r="F204" s="2" t="inlineStr"/>
       <c r="G204" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -20808,10 +20816,10 @@
         </is>
       </c>
       <c r="I204" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J204" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K204" s="2" t="inlineStr"/>
       <c r="L204" s="2" t="inlineStr"/>
@@ -20823,14 +20831,59 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q204" s="2" t="inlineStr">
+      <c r="Q204" s="2" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>All harnesses (master wire list)</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>pigtail supplied with the sensor (owned)</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr"/>
+      <c r="E205" s="3" t="inlineStr"/>
+      <c r="F205" s="3" t="inlineStr"/>
+      <c r="G205" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J205" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K205" s="3" t="inlineStr"/>
+      <c r="L205" s="3" t="inlineStr"/>
+      <c r="M205" s="3" t="inlineStr"/>
+      <c r="N205" s="3" t="inlineStr"/>
+      <c r="O205" s="3" t="inlineStr"/>
+      <c r="P205" s="3" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q205" s="3" t="inlineStr">
         <is>
           <t>on hand (sensor plug / terminal: never a buy)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q204"/>
+  <autoFilter ref="A1:Q205"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -20948,16 +21001,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N142" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId126"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -20970,7 +21023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D106"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23275,7 +23328,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -23297,22 +23350,44 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
           <t>in kit D 261 205 358-01</t>
         </is>
       </c>
-      <c r="C106" s="2" t="inlineStr">
+      <c r="C107" s="3" t="inlineStr">
         <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
+      <c r="D107" s="3" t="inlineStr">
         <is>
           <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D106"/>
+  <autoFilter ref="A1:D107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Harness C from Dan's placement; front side marker lamps; EB on its factory bolt (#467)
- Route 17 rebuilt from Dan's harness C placement (lines, spots, picture, tables)
- Master: LH / RH front side marker lamps (F5 / F6) off SP-CLR, grounds to EB / EA
- EB on the factory bolt (EWD p.36) via a short front-run stub; block strap lands as lug GND-EB-2
- Route 16 devices 18 / H1 keep only HeavyDC ends; harness C owns its own block-stud and alternator-plug spots
- EngineRoom-C lengths from the tree; wire lists, pin chart, BOM regenerated


Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mechanical assemblies'!$A$1:$Q$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$204</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Wire harness'!$A$1:$Q$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'To do'!$A$1:$D$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,16 +540,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4308.88</v>
+        <v>4373.57</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4746.74</v>
+        <v>4811.43</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -8369,7 +8369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q204"/>
+  <dimension ref="A1:Q205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12586,7 +12586,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -12597,7 +12597,7 @@
         <v>0</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
@@ -12611,7 +12611,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>4.3 m in the master + 15% margin</t>
+          <t>0.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>5.9 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13168,7 +13168,7 @@
       </c>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>5.1 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.4 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13249,7 +13249,7 @@
         </is>
       </c>
       <c r="G79" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
@@ -13260,13 +13260,13 @@
         <v>0</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K79" s="3" t="n">
         <v>5.54</v>
       </c>
       <c r="L79" s="3" t="n">
-        <v>66.48</v>
+        <v>72.02</v>
       </c>
       <c r="M79" s="4" t="inlineStr">
         <is>
@@ -13286,7 +13286,7 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>10.0 m of bundle + 10 % cut / recovery margin</t>
+          <t>11.1 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13318,7 +13318,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13329,13 +13329,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>14.99</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>74.95</v>
+        <v>89.94</v>
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
@@ -13355,7 +13355,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>4.3 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.6 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>7.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>8.0 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -15234,7 +15234,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -15245,7 +15245,7 @@
         <v>0</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr"/>
@@ -15259,7 +15259,7 @@
       </c>
       <c r="Q110" s="2" t="inlineStr">
         <is>
-          <t>14.4 m in the master + 15% margin</t>
+          <t>14.3 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15348,7 +15348,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -15359,7 +15359,7 @@
         <v>0</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K112" s="2" t="inlineStr"/>
       <c r="L112" s="2" t="inlineStr"/>
@@ -15373,7 +15373,7 @@
       </c>
       <c r="Q112" s="2" t="inlineStr">
         <is>
-          <t>12.2 m in the master + 15% margin</t>
+          <t>12.4 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15633,7 +15633,7 @@
         </is>
       </c>
       <c r="G117" s="3" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
@@ -15644,7 +15644,7 @@
         <v>0</v>
       </c>
       <c r="J117" s="3" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="K117" s="3" t="inlineStr"/>
       <c r="L117" s="3" t="inlineStr"/>
@@ -15658,7 +15658,7 @@
       </c>
       <c r="Q117" s="3" t="inlineStr">
         <is>
-          <t>24.5 m in the master + 15% margin</t>
+          <t>24.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15914,7 +15914,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -15925,13 +15925,13 @@
         <v>0</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>1.95</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>23.4</v>
+        <v>31.2</v>
       </c>
       <c r="M122" s="5" t="inlineStr">
         <is>
@@ -15955,7 +15955,7 @@
       </c>
       <c r="Q122" s="2" t="inlineStr">
         <is>
-          <t>3.2 m in the master + 15% margin</t>
+          <t>4.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -15987,7 +15987,7 @@
         </is>
       </c>
       <c r="G123" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
@@ -15998,13 +15998,13 @@
         <v>0</v>
       </c>
       <c r="J123" s="3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K123" s="3" t="n">
         <v>1.95</v>
       </c>
       <c r="L123" s="3" t="n">
-        <v>74.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="M123" s="4" t="inlineStr">
         <is>
@@ -16028,7 +16028,7 @@
       </c>
       <c r="Q123" s="3" t="inlineStr">
         <is>
-          <t>9.8 m in the master + 15% margin</t>
+          <t>10.4 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
         </is>
       </c>
       <c r="G125" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
@@ -16128,13 +16128,13 @@
         <v>0</v>
       </c>
       <c r="J125" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K125" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>23.4</v>
+        <v>25.2</v>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>3.4 m in the master + 15% margin</t>
+          <t>3.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16190,7 +16190,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -16201,13 +16201,13 @@
         <v>0</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>1.8</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>73.8</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
@@ -16231,7 +16231,7 @@
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>10.7 m in the master + 15% margin</t>
+          <t>10.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16304,7 +16304,7 @@
       </c>
       <c r="Q127" s="3" t="inlineStr">
         <is>
-          <t>4.0 m in the master + 15% margin</t>
+          <t>4.2 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16336,7 +16336,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -16347,13 +16347,13 @@
         <v>0</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="K128" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L128" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="M128" s="5" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
       </c>
       <c r="Q128" s="2" t="inlineStr">
         <is>
-          <t>22.4 m in the master + 15% margin</t>
+          <t>21.7 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16434,7 +16434,7 @@
       </c>
       <c r="Q129" s="3" t="inlineStr">
         <is>
-          <t>1.0 m in the master + 15% margin</t>
+          <t>0.8 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16466,7 +16466,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -16477,13 +16477,13 @@
         <v>0</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K130" s="2" t="n">
         <v>1.88</v>
       </c>
       <c r="L130" s="2" t="n">
-        <v>39.48</v>
+        <v>50.76</v>
       </c>
       <c r="M130" s="5" t="inlineStr">
         <is>
@@ -16507,7 +16507,7 @@
       </c>
       <c r="Q130" s="2" t="inlineStr">
         <is>
-          <t>5.5 m in the master + 15% margin</t>
+          <t>7.1 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -16539,7 +16539,7 @@
         </is>
       </c>
       <c r="G131" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
@@ -16550,13 +16550,13 @@
         <v>0</v>
       </c>
       <c r="J131" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="K131" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L131" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="M131" s="4" t="inlineStr">
         <is>
@@ -16580,7 +16580,7 @@
       </c>
       <c r="Q131" s="3" t="inlineStr">
         <is>
-          <t>29.2 m in the master + 15% margin</t>
+          <t>31.6 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17253,7 +17253,7 @@
         </is>
       </c>
       <c r="G141" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
@@ -17264,13 +17264,13 @@
         <v>0</v>
       </c>
       <c r="J141" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K141" s="3" t="n">
         <v>3.86</v>
       </c>
       <c r="L141" s="3" t="n">
-        <v>34.74</v>
+        <v>27.02</v>
       </c>
       <c r="M141" s="4" t="inlineStr">
         <is>
@@ -17294,7 +17294,7 @@
       </c>
       <c r="Q141" s="3" t="inlineStr">
         <is>
-          <t>2.1 m in the master + 15% margin</t>
+          <t>1.9 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -17326,7 +17326,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -17337,13 +17337,13 @@
         <v>0</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K142" s="2" t="n">
         <v>3.86</v>
       </c>
       <c r="L142" s="2" t="n">
-        <v>42.46</v>
+        <v>61.76</v>
       </c>
       <c r="M142" s="5" t="inlineStr">
         <is>
@@ -17367,7 +17367,7 @@
       </c>
       <c r="Q142" s="2" t="inlineStr">
         <is>
-          <t>2.8 m in the master + 15% margin</t>
+          <t>4.0 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -18797,7 +18797,7 @@
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K169" s="3" t="inlineStr"/>
       <c r="L169" s="3" t="inlineStr"/>
@@ -18899,11 +18899,11 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-EB-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G171" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
@@ -18914,7 +18914,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K171" s="3" t="inlineStr"/>
       <c r="L171" s="3" t="inlineStr"/>
@@ -18952,11 +18952,11 @@
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-ID) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -18967,7 +18967,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K172" s="2" t="inlineStr"/>
       <c r="L172" s="2" t="inlineStr"/>
@@ -19005,7 +19005,7 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (GND-IG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G173" s="3" t="n">
@@ -19058,11 +19058,11 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ALT-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -19073,7 +19073,7 @@
         <v>0</v>
       </c>
       <c r="J174" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K174" s="2" t="inlineStr"/>
       <c r="L174" s="2" t="inlineStr"/>
@@ -19111,7 +19111,7 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
@@ -19164,11 +19164,11 @@
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -19179,7 +19179,7 @@
         <v>0</v>
       </c>
       <c r="J176" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K176" s="2" t="inlineStr"/>
       <c r="L176" s="2" t="inlineStr"/>
@@ -19217,7 +19217,7 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-AT-GND-C) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G177" s="3" t="n">
@@ -19270,7 +19270,7 @@
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-CLUSTER-HL) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
@@ -19323,7 +19323,7 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G179" s="3" t="n">
@@ -19376,7 +19376,7 @@
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G180" s="2" t="n">
@@ -19429,7 +19429,7 @@
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-ENG-BLOCK-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G181" s="3" t="n">
@@ -19482,7 +19482,7 @@
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G182" s="2" t="n">
@@ -19535,7 +19535,7 @@
       <c r="E183" s="3" t="inlineStr"/>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-2) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
@@ -19588,7 +19588,7 @@
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-STARTER-B-3) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G184" s="2" t="n">
@@ -19641,7 +19641,7 @@
       <c r="E185" s="3" t="inlineStr"/>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-FP-GND) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G185" s="3" t="n">
@@ -19687,22 +19687,18 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-1/2-2.0-9</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (Raychem)</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr"/>
       <c r="E186" s="2" t="inlineStr"/>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>part number not confirmed yet: lug / terminal (T-TRUNK-NEG) (check_wiring.py --tbd)</t>
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -19713,27 +19709,23 @@
         <v>0</v>
       </c>
       <c r="J186" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K186" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L186" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr"/>
       <c r="M186" s="2" t="inlineStr"/>
       <c r="N186" s="2" t="inlineStr"/>
-      <c r="O186" s="2" t="inlineStr">
-        <is>
-          <t>not priced (Dan)</t>
-        </is>
-      </c>
+      <c r="O186" s="2" t="inlineStr"/>
       <c r="P186" s="2" t="inlineStr">
         <is>
-          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
-        </is>
-      </c>
-      <c r="Q186" s="2" t="inlineStr"/>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="inlineStr">
+        <is>
+          <t>no maker document in the repo yet; never guessed</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -19748,7 +19740,7 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/16-2.0-9</t>
+          <t>TMS-SCE-1/2-2.0-9</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -19759,11 +19751,11 @@
       <c r="E187" s="3" t="inlineStr"/>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 12.7 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G187" s="3" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
@@ -19774,7 +19766,7 @@
         <v>0</v>
       </c>
       <c r="J187" s="3" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="K187" s="3" t="n">
         <v>0</v>
@@ -19809,7 +19801,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>TMS-SCE-3/8-2.0-9</t>
+          <t>TMS-SCE-3/16-2.0-9</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -19820,11 +19812,11 @@
       <c r="E188" s="2" t="inlineStr"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 4.8 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -19835,7 +19827,7 @@
         <v>0</v>
       </c>
       <c r="J188" s="2" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="K188" s="2" t="n">
         <v>0</v>
@@ -19870,22 +19862,22 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>W12S</t>
+          <t>TMS-SCE-3/8-2.0-9</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>Deutsch (TE Connectivity)</t>
+          <t>TE Connectivity (Raychem)</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr"/>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
+          <t>MARKER, HEAT SHRINK, PRINTABLE, TMS-SCE, WHITE, 3:1, 9.5 MM EXPANDED ID, 50 MM, THERMAL TRANSFER PRINT</t>
         </is>
       </c>
       <c r="G189" s="3" t="n">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
@@ -19893,31 +19885,27 @@
         </is>
       </c>
       <c r="I189" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J189" s="3" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="K189" s="3" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L189" s="3" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="M189" s="4" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M189" s="3" t="inlineStr"/>
       <c r="N189" s="3" t="inlineStr"/>
       <c r="O189" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
+          <t>not priced (Dan)</t>
         </is>
       </c>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
+          <t>404: te.com URL form is not a product page (checked 2026-10-19); find the real page</t>
         </is>
       </c>
       <c r="Q189" s="3" t="inlineStr"/>
@@ -19935,58 +19923,54 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>W2P</t>
+          <t>W12S</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr">
-        <is>
-          <t>✓ TE</t>
-        </is>
-      </c>
+          <t>Deutsch (TE Connectivity)</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr"/>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 12 POS, PLUG</t>
         </is>
       </c>
       <c r="G190" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H190" s="2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I190" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="J190" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K190" s="2" t="n">
-        <v>0.13</v>
+        <v>0.42</v>
       </c>
       <c r="L190" s="2" t="n">
-        <v>0.26</v>
+        <v>1.26</v>
       </c>
       <c r="M190" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W12S/6566599</t>
         </is>
       </c>
       <c r="N190" s="2" t="inlineStr"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1, 2026-10-19</t>
+          <t>Digi-Key qty 3 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key product page opened 2026-10-19</t>
+          <t>Digi-Key API 2026-10-20: 22279 in stock</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr"/>
@@ -20004,7 +19988,7 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>W2S</t>
+          <t>W2P</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -20019,11 +20003,11 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 2-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G191" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
@@ -20034,28 +20018,28 @@
         <v>0</v>
       </c>
       <c r="J191" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K191" s="3" t="n">
         <v>0.13</v>
       </c>
       <c r="L191" s="3" t="n">
-        <v>1.3</v>
+        <v>0.26</v>
       </c>
       <c r="M191" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W2S.html</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W2P/6566600</t>
         </is>
       </c>
       <c r="N191" s="3" t="inlineStr"/>
       <c r="O191" s="3" t="inlineStr">
         <is>
-          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
+          <t>Digi-Key qty 1, 2026-10-19</t>
         </is>
       </c>
       <c r="P191" s="3" t="inlineStr">
         <is>
-          <t>te.com page opened 2026-10-19</t>
+          <t>Digi-Key product page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q191" s="3" t="inlineStr"/>
@@ -20073,12 +20057,12 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>W3P</t>
+          <t>W2S</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
@@ -20088,11 +20072,11 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 2-WAY PLUG</t>
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -20103,17 +20087,17 @@
         <v>0</v>
       </c>
       <c r="J192" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K192" s="2" t="n">
         <v>0.13</v>
       </c>
       <c r="L192" s="2" t="n">
-        <v>0.13</v>
+        <v>1.3</v>
       </c>
       <c r="M192" s="5" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3P.html</t>
+          <t>https://www.te.com/en/product-W2S.html</t>
         </is>
       </c>
       <c r="N192" s="2" t="inlineStr"/>
@@ -20142,7 +20126,7 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>W3S</t>
+          <t>W3P</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -20157,11 +20141,11 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 3 POS, RECEPTACLE</t>
         </is>
       </c>
       <c r="G193" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H193" s="3" t="inlineStr">
         <is>
@@ -20172,17 +20156,17 @@
         <v>0</v>
       </c>
       <c r="J193" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K193" s="3" t="n">
         <v>0.13</v>
       </c>
       <c r="L193" s="3" t="n">
-        <v>0.39</v>
+        <v>0.13</v>
       </c>
       <c r="M193" s="4" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-W3S.html</t>
+          <t>https://www.te.com/en/product-W3P.html</t>
         </is>
       </c>
       <c r="N193" s="3" t="inlineStr"/>
@@ -20193,7 +20177,7 @@
       </c>
       <c r="P193" s="3" t="inlineStr">
         <is>
-          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
+          <t>te.com page opened 2026-10-19</t>
         </is>
       </c>
       <c r="Q193" s="3" t="inlineStr"/>
@@ -20211,12 +20195,12 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>W6P</t>
+          <t>W3S</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>TE DEUTSCH</t>
+          <t>Deutsch</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
@@ -20226,11 +20210,11 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
+          <t>WEDGELOCK, DT, 3 POS, PLUG</t>
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -20241,28 +20225,28 @@
         <v>0</v>
       </c>
       <c r="J194" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K194" s="2" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="L194" s="2" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="M194" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
+          <t>https://www.te.com/en/product-W3S.html</t>
         </is>
       </c>
       <c r="N194" s="2" t="inlineStr"/>
       <c r="O194" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
+          <t>family price (W2P, Digi-Key qty 1, 2026-10-19)</t>
         </is>
       </c>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
+          <t>te.com URL form, page NOT opened (te.com blocked the automated check): confirm</t>
         </is>
       </c>
       <c r="Q194" s="2" t="inlineStr"/>
@@ -20280,7 +20264,7 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>W6S</t>
+          <t>W6P</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -20295,7 +20279,7 @@
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY RECEPTACLE</t>
         </is>
       </c>
       <c r="G195" s="3" t="n">
@@ -20313,14 +20297,14 @@
         <v>2</v>
       </c>
       <c r="K195" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="L195" s="3" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="M195" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6P/6566692</t>
         </is>
       </c>
       <c r="N195" s="3" t="inlineStr"/>
@@ -20331,7 +20315,7 @@
       </c>
       <c r="P195" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
+          <t>Digi-Key API 2026-10-20: 18695 in stock</t>
         </is>
       </c>
       <c r="Q195" s="3" t="inlineStr"/>
@@ -20349,7 +20333,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>W8S</t>
+          <t>W6S</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -20364,11 +20348,11 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 6-WAY PLUG</t>
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -20379,28 +20363,28 @@
         <v>0</v>
       </c>
       <c r="J196" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K196" s="2" t="n">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="L196" s="2" t="n">
-        <v>0.35</v>
+        <v>0.42</v>
       </c>
       <c r="M196" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W6S/6566605</t>
         </is>
       </c>
       <c r="N196" s="2" t="inlineStr"/>
       <c r="O196" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+          <t>Digi-Key qty 2 (Box), 2026-10-20</t>
         </is>
       </c>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
+          <t>Digi-Key API 2026-10-20: 50335 in stock</t>
         </is>
       </c>
       <c r="Q196" s="2" t="inlineStr"/>
@@ -20418,7 +20402,7 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>WM-4S</t>
+          <t>W8S</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -20433,7 +20417,7 @@
       </c>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
+          <t>WEDGELOCK, DT, 8 POS, PLUG</t>
         </is>
       </c>
       <c r="G197" s="3" t="n">
@@ -20451,14 +20435,14 @@
         <v>1</v>
       </c>
       <c r="K197" s="3" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="L197" s="3" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="M197" s="4" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/W8S/9744670</t>
         </is>
       </c>
       <c r="N197" s="3" t="inlineStr"/>
@@ -20469,7 +20453,7 @@
       </c>
       <c r="P197" s="3" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
+          <t>Digi-Key API 2026-10-20: 2460 in stock</t>
         </is>
       </c>
       <c r="Q197" s="3" t="inlineStr"/>
@@ -20487,12 +20471,12 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>WM-6S</t>
+          <t>WM-4S</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Deutsch</t>
+          <t>TE DEUTSCH</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -20502,7 +20486,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+          <t>WEDGELOCK, DTM, 4 POS, PLUG</t>
         </is>
       </c>
       <c r="G198" s="2" t="n">
@@ -20520,14 +20504,14 @@
         <v>1</v>
       </c>
       <c r="K198" s="2" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="L198" s="2" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="M198" s="5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-4S/6566615</t>
         </is>
       </c>
       <c r="N198" s="2" t="inlineStr"/>
@@ -20538,7 +20522,7 @@
       </c>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
+          <t>Digi-Key API 2026-10-20: 12271 in stock</t>
         </is>
       </c>
       <c r="Q198" s="2" t="inlineStr"/>
@@ -20556,14 +20540,26 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>in kit 354404</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="inlineStr"/>
-      <c r="E199" s="3" t="inlineStr"/>
-      <c r="F199" s="3" t="inlineStr"/>
+          <t>WM-6S</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>✓ TE</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>WEDGELOCK, DTM, 6 POS, PLUG</t>
+        </is>
+      </c>
       <c r="G199" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
@@ -20571,26 +20567,34 @@
         </is>
       </c>
       <c r="I199" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J199" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K199" s="3" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr"/>
-      <c r="M199" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K199" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="L199" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="M199" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/detail/te-connectivity-deutsch-ict-connectors/WM-6S/6566617</t>
+        </is>
+      </c>
       <c r="N199" s="3" t="inlineStr"/>
-      <c r="O199" s="3" t="inlineStr"/>
+      <c r="O199" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key qty 1 (Box), 2026-10-20</t>
+        </is>
+      </c>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>NO LINK</t>
-        </is>
-      </c>
-      <c r="Q199" s="3" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
+          <t>Digi-Key API 2026-10-20: 2478 in stock</t>
+        </is>
+      </c>
+      <c r="Q199" s="3" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -20605,14 +20609,14 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>in kit CONN-75800</t>
+          <t>in kit 354404</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr"/>
       <c r="E200" s="2" t="inlineStr"/>
       <c r="F200" s="2" t="inlineStr"/>
       <c r="G200" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -20620,7 +20624,7 @@
         </is>
       </c>
       <c r="I200" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J200" s="2" t="n">
         <v>0</v>
@@ -20654,14 +20658,14 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr"/>
       <c r="E201" s="3" t="inlineStr"/>
       <c r="F201" s="3" t="inlineStr"/>
       <c r="G201" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
@@ -20669,10 +20673,10 @@
         </is>
       </c>
       <c r="I201" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J201" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K201" s="3" t="inlineStr"/>
       <c r="L201" s="3" t="inlineStr"/>
@@ -20684,7 +20688,11 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q201" s="3" t="inlineStr"/>
+      <c r="Q201" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -20699,14 +20707,14 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>in kit CONN-76270</t>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr"/>
       <c r="E202" s="2" t="inlineStr"/>
       <c r="F202" s="2" t="inlineStr"/>
       <c r="G202" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -20714,10 +20722,10 @@
         </is>
       </c>
       <c r="I202" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J202" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
       <c r="L202" s="2" t="inlineStr"/>
@@ -20729,11 +20737,7 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q202" s="2" t="inlineStr">
-        <is>
-          <t>on hand (sensor plug / terminal: never a buy)</t>
-        </is>
-      </c>
+      <c r="Q202" s="2" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -20748,14 +20752,14 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>in kit D 261 205 358-01</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr"/>
       <c r="E203" s="3" t="inlineStr"/>
       <c r="F203" s="3" t="inlineStr"/>
       <c r="G203" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
@@ -20763,10 +20767,10 @@
         </is>
       </c>
       <c r="I203" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J203" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K203" s="3" t="inlineStr"/>
       <c r="L203" s="3" t="inlineStr"/>
@@ -20778,7 +20782,11 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q203" s="3" t="inlineStr"/>
+      <c r="Q203" s="3" t="inlineStr">
+        <is>
+          <t>on hand (sensor plug / terminal: never a buy)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -20793,14 +20801,14 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>pigtail supplied with the sensor (owned)</t>
+          <t>in kit D 261 205 358-01</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr"/>
       <c r="E204" s="2" t="inlineStr"/>
       <c r="F204" s="2" t="inlineStr"/>
       <c r="G204" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -20808,10 +20816,10 @@
         </is>
       </c>
       <c r="I204" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J204" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K204" s="2" t="inlineStr"/>
       <c r="L204" s="2" t="inlineStr"/>
@@ -20823,14 +20831,59 @@
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="Q204" s="2" t="inlineStr">
+      <c r="Q204" s="2" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>All harnesses (master wire list)</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>pigtail supplied with the sensor (owned)</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr"/>
+      <c r="E205" s="3" t="inlineStr"/>
+      <c r="F205" s="3" t="inlineStr"/>
+      <c r="G205" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J205" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K205" s="3" t="inlineStr"/>
+      <c r="L205" s="3" t="inlineStr"/>
+      <c r="M205" s="3" t="inlineStr"/>
+      <c r="N205" s="3" t="inlineStr"/>
+      <c r="O205" s="3" t="inlineStr"/>
+      <c r="P205" s="3" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="Q205" s="3" t="inlineStr">
         <is>
           <t>on hand (sensor plug / terminal: never a buy)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q204"/>
+  <autoFilter ref="A1:Q205"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -20948,16 +21001,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N142" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId126"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -20970,7 +21023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D106"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23275,7 +23328,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -23297,22 +23350,44 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>NO LINK</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>I find and validate a maker page or approved-supplier listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>Wire harness</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
           <t>in kit D 261 205 358-01</t>
         </is>
       </c>
-      <c r="C106" s="2" t="inlineStr">
+      <c r="C107" s="3" t="inlineStr">
         <is>
           <t>NO LINK</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
+      <c r="D107" s="3" t="inlineStr">
         <is>
           <t>I find and validate a maker page or approved-supplier listing</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D106"/>
+  <autoFilter ref="A1:D107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
RH pop-up motor ground to EA; grounds drawn on their own side of the car
- Master: w_rtr_gnd_r3_t lands on GND-EA (RH fender), 1.0 m (was EB, 1.9 m)
- README schematic format: a ground stud is drawn on the side of the car its wires go to (Dan)
- Dates of the harness C placement entries set to 2026-11-01 (ET)
- Wire lists, pin chart and BOM regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4373.57</v>
+        <v>4358.79</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4811.43</v>
+        <v>4796.65</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>6.2 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13131,7 +13131,7 @@
         </is>
       </c>
       <c r="G77" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
@@ -13142,13 +13142,13 @@
         <v>0</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K77" s="3" t="n">
         <v>5.61</v>
       </c>
       <c r="L77" s="3" t="n">
-        <v>33.66</v>
+        <v>39.27</v>
       </c>
       <c r="M77" s="4" t="inlineStr">
         <is>
@@ -13168,7 +13168,7 @@
       </c>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>5.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13318,7 +13318,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13329,13 +13329,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>14.99</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>89.94</v>
+        <v>74.95</v>
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
@@ -13355,7 +13355,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>4.6 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.0 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>8.0 m of bundle + 10 % cut / recovery margin</t>
+          <t>7.8 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
         </is>
       </c>
       <c r="G125" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
@@ -16128,13 +16128,13 @@
         <v>0</v>
       </c>
       <c r="J125" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K125" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>25.2</v>
+        <v>19.8</v>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>3.6 m in the master + 15% margin</t>
+          <t>2.7 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -18797,7 +18797,7 @@
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K169" s="3" t="inlineStr"/>
       <c r="L169" s="3" t="inlineStr"/>
@@ -18850,7 +18850,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -18861,7 +18861,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K170" s="2" t="inlineStr"/>
       <c r="L170" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
RH pop-up motor ground to EA; grounds drawn on their own side of the car (#468)
- Master: w_rtr_gnd_r3_t lands on GND-EA (RH fender), 1.0 m (was EB, 1.9 m)
- README schematic format: a ground stud is drawn on the side of the car its wires go to (Dan)
- Dates of the harness C placement entries set to 2026-11-01 (ET)
- Wire lists, pin chart and BOM regenerated


Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sourcing/PROJECT-BOM.xlsx
+++ b/docs/sourcing/PROJECT-BOM.xlsx
@@ -549,7 +549,7 @@
         <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4373.57</v>
+        <v>4358.79</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>168</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4811.43</v>
+        <v>4796.65</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>18</v>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
+          <t>6.2 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13131,7 +13131,7 @@
         </is>
       </c>
       <c r="G77" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
@@ -13142,13 +13142,13 @@
         <v>0</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K77" s="3" t="n">
         <v>5.61</v>
       </c>
       <c r="L77" s="3" t="n">
-        <v>33.66</v>
+        <v>39.27</v>
       </c>
       <c r="M77" s="4" t="inlineStr">
         <is>
@@ -13168,7 +13168,7 @@
       </c>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>5.4 m of bundle + 10 % cut / recovery margin</t>
+          <t>5.5 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13318,7 +13318,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -13329,13 +13329,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>14.99</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>89.94</v>
+        <v>74.95</v>
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
@@ -13355,7 +13355,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>4.6 m of bundle + 10 % cut / recovery margin</t>
+          <t>4.0 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>8.0 m of bundle + 10 % cut / recovery margin</t>
+          <t>7.8 m of bundle + 10 % cut / recovery margin</t>
         </is>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
         </is>
       </c>
       <c r="G125" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
@@ -16128,13 +16128,13 @@
         <v>0</v>
       </c>
       <c r="J125" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K125" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="L125" s="3" t="n">
-        <v>25.2</v>
+        <v>19.8</v>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>3.6 m in the master + 15% margin</t>
+          <t>2.7 m in the master + 15% margin</t>
         </is>
       </c>
     </row>
@@ -18797,7 +18797,7 @@
         </is>
       </c>
       <c r="G169" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>0</v>
       </c>
       <c r="J169" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K169" s="3" t="inlineStr"/>
       <c r="L169" s="3" t="inlineStr"/>
@@ -18850,7 +18850,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -18861,7 +18861,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K170" s="2" t="inlineStr"/>
       <c r="L170" s="2" t="inlineStr"/>

</xml_diff>